<commit_message>
feat(pace): Live própria meta R$230k ago + REF551/REF528 mix premium (ajuste +148/+156)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
+++ b/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
@@ -9786,7 +9786,7 @@
       </c>
       <c r="B3" s="89" t="inlineStr">
         <is>
-          <t>Escalar sessões próprias + restaurar mídia de live</t>
+          <t>Escalar sessões próprias + restaurar mídia de live · MIX PREMIUM: Azul Médio (551) + Wide 528 puxados pra meta 230k</t>
         </is>
       </c>
     </row>
@@ -10196,7 +10196,7 @@
       </c>
       <c r="B11" s="74" t="inlineStr">
         <is>
-          <t>Azul Médio</t>
+          <t>Azul Médio · PREMIUM</t>
         </is>
       </c>
       <c r="C11" s="74" t="inlineStr">
@@ -10212,7 +10212,7 @@
         <v/>
       </c>
       <c r="F11" s="92" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="G11" s="112">
         <f>ROUND(D11*(1+$B$4),0)+F11</f>
@@ -10352,7 +10352,7 @@
       </c>
       <c r="B13" s="74" t="inlineStr">
         <is>
-          <t>Wide 528</t>
+          <t>Wide 528 · PREMIUM</t>
         </is>
       </c>
       <c r="C13" s="74" t="inlineStr">
@@ -10368,7 +10368,7 @@
         <v/>
       </c>
       <c r="F13" s="92" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="G13" s="112">
         <f>ROUND(D13*(1+$B$4),0)+F13</f>

</xml_diff>

<commit_message>
feat(pace): REF562 Chocolate pré-escala 700pç/mês distribuída (vídeo-led)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
+++ b/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
@@ -2188,7 +2188,7 @@
         <v/>
       </c>
       <c r="F14" s="92" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="G14" s="112">
         <f>ROUND(D14*(1+$B$4),0)+F14</f>
@@ -6777,7 +6777,7 @@
         <v/>
       </c>
       <c r="F11" s="92" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="G11" s="112">
         <f>ROUND(D11*(1+$B$4),0)+F11</f>
@@ -8650,7 +8650,7 @@
         <v/>
       </c>
       <c r="F17" s="92" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="G17" s="112">
         <f>ROUND(D17*(1+$B$4),0)+F17</f>
@@ -10446,7 +10446,7 @@
         <v/>
       </c>
       <c r="F14" s="92" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="G14" s="112">
         <f>ROUND(D14*(1+$B$4),0)+F14</f>

</xml_diff>

<commit_message>
style(pace): aba Soma SKU x Canal como Tabela Excel (zebra + filtro)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
+++ b/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
@@ -37,7 +37,7 @@
     <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="169" formatCode="&quot;R$ &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -178,8 +178,26 @@
       <color rgb="007A7A7A"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007A7A7A"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E7E34"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -222,6 +240,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EAF2FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -273,7 +296,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -672,6 +695,28 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="20" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -742,6 +787,27 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SomaSKUxCanal" displayName="SomaSKUxCanal" ref="A4:L33" headerRowCount="1">
+  <autoFilter ref="A4:L33"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="SKU"/>
+    <tableColumn id="2" name="Produto"/>
+    <tableColumn id="3" name="Cl"/>
+    <tableColumn id="4" name="Live afiliada"/>
+    <tableColumn id="5" name="Vídeo afiliada"/>
+    <tableColumn id="6" name="Card afiliada"/>
+    <tableColumn id="7" name="Live loja"/>
+    <tableColumn id="8" name="Vídeo loja"/>
+    <tableColumn id="9" name="Card loja"/>
+    <tableColumn id="10" name="Vitrine loja"/>
+    <tableColumn id="11" name="Busca e Mall"/>
+    <tableColumn id="12" name="TOTAL SKU"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6097,17 +6163,17 @@
   <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="63" min="1" max="1"/>
+    <col width="11" customWidth="1" style="63" min="1" max="1"/>
     <col width="18" customWidth="1" style="63" min="2" max="2"/>
     <col width="5" customWidth="1" style="63" min="3" max="3"/>
-    <col width="13" customWidth="1" style="63" min="4" max="4"/>
-    <col width="13" customWidth="1" style="63" min="5" max="5"/>
-    <col width="13" customWidth="1" style="63" min="6" max="6"/>
-    <col width="13" customWidth="1" style="63" min="7" max="7"/>
-    <col width="13" customWidth="1" style="63" min="8" max="8"/>
-    <col width="13" customWidth="1" style="63" min="9" max="9"/>
-    <col width="13" customWidth="1" style="63" min="10" max="10"/>
-    <col width="13" customWidth="1" style="63" min="11" max="11"/>
+    <col width="12" customWidth="1" style="63" min="4" max="4"/>
+    <col width="12" customWidth="1" style="63" min="5" max="5"/>
+    <col width="12" customWidth="1" style="63" min="6" max="6"/>
+    <col width="12" customWidth="1" style="63" min="7" max="7"/>
+    <col width="12" customWidth="1" style="63" min="8" max="8"/>
+    <col width="12" customWidth="1" style="63" min="9" max="9"/>
+    <col width="12" customWidth="1" style="63" min="10" max="10"/>
+    <col width="12" customWidth="1" style="63" min="11" max="11"/>
     <col width="11" customWidth="1" style="63" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -6121,1650 +6187,1650 @@
     <row r="2">
       <c r="A2" s="125" t="inlineStr">
         <is>
-          <t>Matriz viva: cada célula = Meta (pç) do SKU naquele canal (SUMIFS das abas). Muda growth/ajuste → recalcula.</t>
+          <t>Matriz viva (SUMIFS das abas de canal). Filtro no cabeçalho · linhas zebradas · muda growth/ajuste → recalcula.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="126" t="inlineStr">
+      <c r="A4" s="138" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="B4" s="126" t="inlineStr">
+      <c r="B4" s="138" t="inlineStr">
         <is>
           <t>Produto</t>
         </is>
       </c>
-      <c r="C4" s="126" t="inlineStr">
+      <c r="C4" s="138" t="inlineStr">
         <is>
           <t>Cl</t>
         </is>
       </c>
-      <c r="D4" s="126" t="inlineStr">
+      <c r="D4" s="138" t="inlineStr">
         <is>
           <t>Live afiliada</t>
         </is>
       </c>
-      <c r="E4" s="126" t="inlineStr">
+      <c r="E4" s="138" t="inlineStr">
         <is>
           <t>Vídeo afiliada</t>
         </is>
       </c>
-      <c r="F4" s="126" t="inlineStr">
+      <c r="F4" s="138" t="inlineStr">
         <is>
           <t>Card afiliada</t>
         </is>
       </c>
-      <c r="G4" s="126" t="inlineStr">
+      <c r="G4" s="138" t="inlineStr">
         <is>
           <t>Live loja</t>
         </is>
       </c>
-      <c r="H4" s="126" t="inlineStr">
+      <c r="H4" s="138" t="inlineStr">
         <is>
           <t>Vídeo loja</t>
         </is>
       </c>
-      <c r="I4" s="126" t="inlineStr">
+      <c r="I4" s="138" t="inlineStr">
         <is>
           <t>Card loja</t>
         </is>
       </c>
-      <c r="J4" s="126" t="inlineStr">
+      <c r="J4" s="138" t="inlineStr">
         <is>
           <t>Vitrine loja</t>
         </is>
       </c>
-      <c r="K4" s="126" t="inlineStr">
+      <c r="K4" s="138" t="inlineStr">
         <is>
           <t>Busca e Mall</t>
         </is>
       </c>
-      <c r="L4" s="126" t="inlineStr">
+      <c r="L4" s="138" t="inlineStr">
         <is>
           <t>TOTAL SKU</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="127" t="inlineStr">
+      <c r="A5" s="138" t="inlineStr">
         <is>
           <t>REF516</t>
         </is>
       </c>
-      <c r="B5" s="128" t="inlineStr">
+      <c r="B5" s="139" t="inlineStr">
         <is>
           <t>Marmorizada</t>
         </is>
       </c>
-      <c r="C5" s="129" t="inlineStr">
+      <c r="C5" s="140" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="D5" s="130">
+      <c r="D5" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="E5" s="130">
+      <c r="E5" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="F5" s="130">
+      <c r="F5" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="G5" s="130">
+      <c r="G5" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="H5" s="130">
+      <c r="H5" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="I5" s="130">
+      <c r="I5" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="J5" s="130">
+      <c r="J5" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="K5" s="130">
+      <c r="K5" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A5)</f>
         <v/>
       </c>
-      <c r="L5" s="131">
+      <c r="L5" s="142">
         <f>SUM(D5:K5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="127" t="inlineStr">
+      <c r="A6" s="138" t="inlineStr">
         <is>
           <t>REF525</t>
         </is>
       </c>
-      <c r="B6" s="128" t="inlineStr">
+      <c r="B6" s="139" t="inlineStr">
         <is>
           <t>Stone Used</t>
         </is>
       </c>
-      <c r="C6" s="129" t="inlineStr">
+      <c r="C6" s="140" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="D6" s="130">
+      <c r="D6" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="E6" s="130">
+      <c r="E6" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="F6" s="130">
+      <c r="F6" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="G6" s="130">
+      <c r="G6" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="H6" s="130">
+      <c r="H6" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="I6" s="130">
+      <c r="I6" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="J6" s="130">
+      <c r="J6" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="K6" s="130">
+      <c r="K6" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A6)</f>
         <v/>
       </c>
-      <c r="L6" s="131">
+      <c r="L6" s="142">
         <f>SUM(D6:K6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="127" t="inlineStr">
+      <c r="A7" s="138" t="inlineStr">
         <is>
           <t>REF527</t>
         </is>
       </c>
-      <c r="B7" s="128" t="inlineStr">
+      <c r="B7" s="139" t="inlineStr">
         <is>
           <t>Sky Used</t>
         </is>
       </c>
-      <c r="C7" s="129" t="inlineStr">
+      <c r="C7" s="140" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="D7" s="130">
+      <c r="D7" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="E7" s="130">
+      <c r="E7" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="F7" s="130">
+      <c r="F7" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="G7" s="130">
+      <c r="G7" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="H7" s="130">
+      <c r="H7" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="I7" s="130">
+      <c r="I7" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="J7" s="130">
+      <c r="J7" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="K7" s="130">
+      <c r="K7" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A7)</f>
         <v/>
       </c>
-      <c r="L7" s="131">
+      <c r="L7" s="142">
         <f>SUM(D7:K7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="127" t="inlineStr">
+      <c r="A8" s="138" t="inlineStr">
         <is>
           <t>REF562</t>
         </is>
       </c>
-      <c r="B8" s="128" t="inlineStr">
+      <c r="B8" s="139" t="inlineStr">
         <is>
           <t>Chocolate</t>
         </is>
       </c>
-      <c r="C8" s="132" t="inlineStr">
+      <c r="C8" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D8" s="130">
+      <c r="D8" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="E8" s="130">
+      <c r="E8" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="F8" s="130">
+      <c r="F8" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="G8" s="130">
+      <c r="G8" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="H8" s="130">
+      <c r="H8" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="I8" s="130">
+      <c r="I8" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="J8" s="130">
+      <c r="J8" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="K8" s="130">
+      <c r="K8" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A8)</f>
         <v/>
       </c>
-      <c r="L8" s="133">
+      <c r="L8" s="142">
         <f>SUM(D8:K8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="127" t="inlineStr">
+      <c r="A9" s="138" t="inlineStr">
         <is>
           <t>REF551</t>
         </is>
       </c>
-      <c r="B9" s="128" t="inlineStr">
+      <c r="B9" s="139" t="inlineStr">
         <is>
           <t>Azul Médio</t>
         </is>
       </c>
-      <c r="C9" s="132" t="inlineStr">
+      <c r="C9" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D9" s="130">
+      <c r="D9" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="E9" s="130">
+      <c r="E9" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="F9" s="130">
+      <c r="F9" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="G9" s="130">
+      <c r="G9" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="H9" s="130">
+      <c r="H9" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="I9" s="130">
+      <c r="I9" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="J9" s="130">
+      <c r="J9" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="K9" s="130">
+      <c r="K9" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A9)</f>
         <v/>
       </c>
-      <c r="L9" s="133">
+      <c r="L9" s="142">
         <f>SUM(D9:K9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="127" t="inlineStr">
+      <c r="A10" s="138" t="inlineStr">
         <is>
           <t>REF587</t>
         </is>
       </c>
-      <c r="B10" s="128" t="inlineStr">
+      <c r="B10" s="139" t="inlineStr">
         <is>
           <t>Baggy Marmorizada</t>
         </is>
       </c>
-      <c r="C10" s="132" t="inlineStr">
+      <c r="C10" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D10" s="130">
+      <c r="D10" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="E10" s="130">
+      <c r="E10" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="F10" s="130">
+      <c r="F10" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="G10" s="130">
+      <c r="G10" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="H10" s="130">
+      <c r="H10" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="I10" s="130">
+      <c r="I10" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="J10" s="130">
+      <c r="J10" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="K10" s="130">
+      <c r="K10" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A10)</f>
         <v/>
       </c>
-      <c r="L10" s="133">
+      <c r="L10" s="142">
         <f>SUM(D10:K10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="127" t="inlineStr">
+      <c r="A11" s="138" t="inlineStr">
         <is>
           <t>REF528</t>
         </is>
       </c>
-      <c r="B11" s="128" t="inlineStr">
+      <c r="B11" s="139" t="inlineStr">
         <is>
           <t>Wide 528</t>
         </is>
       </c>
-      <c r="C11" s="132" t="inlineStr">
+      <c r="C11" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D11" s="130">
+      <c r="D11" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="E11" s="130">
+      <c r="E11" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="F11" s="130">
+      <c r="F11" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="G11" s="130">
+      <c r="G11" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="H11" s="130">
+      <c r="H11" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="I11" s="130">
+      <c r="I11" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="J11" s="130">
+      <c r="J11" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="K11" s="130">
+      <c r="K11" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A11)</f>
         <v/>
       </c>
-      <c r="L11" s="133">
+      <c r="L11" s="142">
         <f>SUM(D11:K11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="127" t="inlineStr">
+      <c r="A12" s="138" t="inlineStr">
         <is>
           <t>REF588</t>
         </is>
       </c>
-      <c r="B12" s="128" t="inlineStr">
+      <c r="B12" s="139" t="inlineStr">
         <is>
           <t>Mom Marmorizada</t>
         </is>
       </c>
-      <c r="C12" s="132" t="inlineStr">
+      <c r="C12" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D12" s="130">
+      <c r="D12" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="E12" s="130">
+      <c r="E12" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="F12" s="130">
+      <c r="F12" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="G12" s="130">
+      <c r="G12" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="H12" s="130">
+      <c r="H12" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="I12" s="130">
+      <c r="I12" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="J12" s="130">
+      <c r="J12" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="K12" s="130">
+      <c r="K12" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A12)</f>
         <v/>
       </c>
-      <c r="L12" s="133">
+      <c r="L12" s="142">
         <f>SUM(D12:K12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="127" t="inlineStr">
+      <c r="A13" s="138" t="inlineStr">
         <is>
           <t>REF529</t>
         </is>
       </c>
-      <c r="B13" s="128" t="inlineStr">
+      <c r="B13" s="139" t="inlineStr">
         <is>
           <t>Wide 529</t>
         </is>
       </c>
-      <c r="C13" s="132" t="inlineStr">
+      <c r="C13" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D13" s="130">
+      <c r="D13" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="E13" s="130">
+      <c r="E13" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="F13" s="130">
+      <c r="F13" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="G13" s="130">
+      <c r="G13" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="H13" s="130">
+      <c r="H13" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="I13" s="130">
+      <c r="I13" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="J13" s="130">
+      <c r="J13" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="K13" s="130">
+      <c r="K13" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A13)</f>
         <v/>
       </c>
-      <c r="L13" s="133">
+      <c r="L13" s="142">
         <f>SUM(D13:K13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="127" t="inlineStr">
+      <c r="A14" s="138" t="inlineStr">
         <is>
           <t>REF549</t>
         </is>
       </c>
-      <c r="B14" s="128" t="inlineStr">
+      <c r="B14" s="139" t="inlineStr">
         <is>
           <t>Rosa Bebê</t>
         </is>
       </c>
-      <c r="C14" s="132" t="inlineStr">
+      <c r="C14" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D14" s="130">
+      <c r="D14" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="E14" s="130">
+      <c r="E14" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="F14" s="130">
+      <c r="F14" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="G14" s="130">
+      <c r="G14" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="H14" s="130">
+      <c r="H14" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="I14" s="130">
+      <c r="I14" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="J14" s="130">
+      <c r="J14" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="K14" s="130">
+      <c r="K14" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A14)</f>
         <v/>
       </c>
-      <c r="L14" s="133">
+      <c r="L14" s="142">
         <f>SUM(D14:K14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="127" t="inlineStr">
+      <c r="A15" s="138" t="inlineStr">
         <is>
           <t>REF550</t>
         </is>
       </c>
-      <c r="B15" s="128" t="inlineStr">
+      <c r="B15" s="139" t="inlineStr">
         <is>
           <t>Amarela</t>
         </is>
       </c>
-      <c r="C15" s="132" t="inlineStr">
+      <c r="C15" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D15" s="130">
+      <c r="D15" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="E15" s="130">
+      <c r="E15" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="F15" s="130">
+      <c r="F15" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="G15" s="130">
+      <c r="G15" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="H15" s="130">
+      <c r="H15" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="I15" s="130">
+      <c r="I15" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="J15" s="130">
+      <c r="J15" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="K15" s="130">
+      <c r="K15" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A15)</f>
         <v/>
       </c>
-      <c r="L15" s="133">
+      <c r="L15" s="142">
         <f>SUM(D15:K15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="127" t="inlineStr">
+      <c r="A16" s="138" t="inlineStr">
         <is>
           <t>REF547</t>
         </is>
       </c>
-      <c r="B16" s="128" t="inlineStr">
+      <c r="B16" s="139" t="inlineStr">
         <is>
           <t>REF547</t>
         </is>
       </c>
-      <c r="C16" s="132" t="inlineStr">
+      <c r="C16" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D16" s="130">
+      <c r="D16" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="E16" s="130">
+      <c r="E16" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="F16" s="130">
+      <c r="F16" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="G16" s="130">
+      <c r="G16" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="H16" s="130">
+      <c r="H16" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="I16" s="130">
+      <c r="I16" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="J16" s="130">
+      <c r="J16" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="K16" s="130">
+      <c r="K16" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A16)</f>
         <v/>
       </c>
-      <c r="L16" s="133">
+      <c r="L16" s="142">
         <f>SUM(D16:K16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="127" t="inlineStr">
+      <c r="A17" s="138" t="inlineStr">
         <is>
           <t>CAUDA</t>
         </is>
       </c>
-      <c r="B17" s="128" t="inlineStr">
+      <c r="B17" s="139" t="inlineStr">
         <is>
           <t>CAUDA</t>
         </is>
       </c>
-      <c r="C17" s="132" t="inlineStr">
+      <c r="C17" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D17" s="130">
+      <c r="D17" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="E17" s="130">
+      <c r="E17" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="F17" s="130">
+      <c r="F17" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="G17" s="130">
+      <c r="G17" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="H17" s="130">
+      <c r="H17" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="I17" s="130">
+      <c r="I17" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="J17" s="130">
+      <c r="J17" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="K17" s="130">
+      <c r="K17" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A17)</f>
         <v/>
       </c>
-      <c r="L17" s="133">
+      <c r="L17" s="142">
         <f>SUM(D17:K17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="127" t="inlineStr">
+      <c r="A18" s="138" t="inlineStr">
         <is>
           <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
         </is>
       </c>
-      <c r="B18" s="128" t="inlineStr">
+      <c r="B18" s="139" t="inlineStr">
         <is>
           <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
         </is>
       </c>
-      <c r="C18" s="132" t="inlineStr">
+      <c r="C18" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D18" s="130">
+      <c r="D18" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="E18" s="130">
+      <c r="E18" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="F18" s="130">
+      <c r="F18" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="G18" s="130">
+      <c r="G18" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="H18" s="130">
+      <c r="H18" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="I18" s="130">
+      <c r="I18" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="J18" s="130">
+      <c r="J18" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="K18" s="130">
+      <c r="K18" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A18)</f>
         <v/>
       </c>
-      <c r="L18" s="133">
+      <c r="L18" s="142">
         <f>SUM(D18:K18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="127" t="inlineStr">
+      <c r="A19" s="138" t="inlineStr">
         <is>
           <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
         </is>
       </c>
-      <c r="B19" s="128" t="inlineStr">
+      <c r="B19" s="139" t="inlineStr">
         <is>
           <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
         </is>
       </c>
-      <c r="C19" s="132" t="inlineStr">
+      <c r="C19" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D19" s="130">
+      <c r="D19" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="E19" s="130">
+      <c r="E19" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="F19" s="130">
+      <c r="F19" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="G19" s="130">
+      <c r="G19" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="H19" s="130">
+      <c r="H19" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="I19" s="130">
+      <c r="I19" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="J19" s="130">
+      <c r="J19" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="K19" s="130">
+      <c r="K19" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A19)</f>
         <v/>
       </c>
-      <c r="L19" s="133">
+      <c r="L19" s="142">
         <f>SUM(D19:K19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="127" t="inlineStr">
+      <c r="A20" s="138" t="inlineStr">
         <is>
           <t>REF559</t>
         </is>
       </c>
-      <c r="B20" s="128" t="inlineStr">
+      <c r="B20" s="139" t="inlineStr">
         <is>
           <t>Mom Rosa</t>
         </is>
       </c>
-      <c r="C20" s="132" t="inlineStr">
+      <c r="C20" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D20" s="130">
+      <c r="D20" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="E20" s="130">
+      <c r="E20" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="F20" s="130">
+      <c r="F20" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="G20" s="130">
+      <c r="G20" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="H20" s="130">
+      <c r="H20" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="I20" s="130">
+      <c r="I20" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="J20" s="130">
+      <c r="J20" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="K20" s="130">
+      <c r="K20" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A20)</f>
         <v/>
       </c>
-      <c r="L20" s="133">
+      <c r="L20" s="142">
         <f>SUM(D20:K20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="127" t="inlineStr">
+      <c r="A21" s="138" t="inlineStr">
         <is>
           <t>REF566</t>
         </is>
       </c>
-      <c r="B21" s="128" t="inlineStr">
+      <c r="B21" s="139" t="inlineStr">
         <is>
           <t>Mom Choco</t>
         </is>
       </c>
-      <c r="C21" s="132" t="inlineStr">
+      <c r="C21" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D21" s="130">
+      <c r="D21" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="E21" s="130">
+      <c r="E21" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="F21" s="130">
+      <c r="F21" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="G21" s="130">
+      <c r="G21" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="H21" s="130">
+      <c r="H21" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="I21" s="130">
+      <c r="I21" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="J21" s="130">
+      <c r="J21" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="K21" s="130">
+      <c r="K21" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A21)</f>
         <v/>
       </c>
-      <c r="L21" s="133">
+      <c r="L21" s="142">
         <f>SUM(D21:K21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="127" t="inlineStr">
+      <c r="A22" s="138" t="inlineStr">
         <is>
           <t>REF558</t>
         </is>
       </c>
-      <c r="B22" s="128" t="inlineStr">
+      <c r="B22" s="139" t="inlineStr">
         <is>
           <t>REF558</t>
         </is>
       </c>
-      <c r="C22" s="132" t="inlineStr">
+      <c r="C22" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D22" s="130">
+      <c r="D22" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="E22" s="130">
+      <c r="E22" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="F22" s="130">
+      <c r="F22" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="G22" s="130">
+      <c r="G22" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="H22" s="130">
+      <c r="H22" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="I22" s="130">
+      <c r="I22" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="J22" s="130">
+      <c r="J22" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="K22" s="130">
+      <c r="K22" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A22)</f>
         <v/>
       </c>
-      <c r="L22" s="133">
+      <c r="L22" s="142">
         <f>SUM(D22:K22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="127" t="inlineStr">
+      <c r="A23" s="138" t="inlineStr">
         <is>
           <t>REF546</t>
         </is>
       </c>
-      <c r="B23" s="128" t="inlineStr">
+      <c r="B23" s="139" t="inlineStr">
         <is>
           <t>REF546</t>
         </is>
       </c>
-      <c r="C23" s="132" t="inlineStr">
+      <c r="C23" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D23" s="130">
+      <c r="D23" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="E23" s="130">
+      <c r="E23" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="F23" s="130">
+      <c r="F23" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="G23" s="130">
+      <c r="G23" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="H23" s="130">
+      <c r="H23" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="I23" s="130">
+      <c r="I23" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="J23" s="130">
+      <c r="J23" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="K23" s="130">
+      <c r="K23" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A23)</f>
         <v/>
       </c>
-      <c r="L23" s="133">
+      <c r="L23" s="142">
         <f>SUM(D23:K23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="127" t="inlineStr">
+      <c r="A24" s="138" t="inlineStr">
         <is>
           <t>AGREGADO</t>
         </is>
       </c>
-      <c r="B24" s="128" t="inlineStr">
+      <c r="B24" s="139" t="inlineStr">
         <is>
           <t>AGREGADO</t>
         </is>
       </c>
-      <c r="C24" s="132" t="inlineStr">
+      <c r="C24" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D24" s="130">
+      <c r="D24" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="E24" s="130">
+      <c r="E24" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="F24" s="130">
+      <c r="F24" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="G24" s="130">
+      <c r="G24" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="H24" s="130">
+      <c r="H24" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="I24" s="130">
+      <c r="I24" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="J24" s="130">
+      <c r="J24" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="K24" s="130">
+      <c r="K24" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A24)</f>
         <v/>
       </c>
-      <c r="L24" s="133">
+      <c r="L24" s="142">
         <f>SUM(D24:K24)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="127" t="inlineStr">
+      <c r="A25" s="138" t="inlineStr">
         <is>
           <t>REF574</t>
         </is>
       </c>
-      <c r="B25" s="128" t="inlineStr">
+      <c r="B25" s="139" t="inlineStr">
         <is>
           <t>REF574</t>
         </is>
       </c>
-      <c r="C25" s="132" t="inlineStr">
+      <c r="C25" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D25" s="130">
+      <c r="D25" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="E25" s="130">
+      <c r="E25" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="F25" s="130">
+      <c r="F25" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="G25" s="130">
+      <c r="G25" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="H25" s="130">
+      <c r="H25" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="I25" s="130">
+      <c r="I25" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="J25" s="130">
+      <c r="J25" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="K25" s="130">
+      <c r="K25" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A25)</f>
         <v/>
       </c>
-      <c r="L25" s="133">
+      <c r="L25" s="142">
         <f>SUM(D25:K25)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="127" t="inlineStr">
+      <c r="A26" s="138" t="inlineStr">
         <is>
           <t>REF573</t>
         </is>
       </c>
-      <c r="B26" s="128" t="inlineStr">
+      <c r="B26" s="139" t="inlineStr">
         <is>
           <t>REF573</t>
         </is>
       </c>
-      <c r="C26" s="132" t="inlineStr">
+      <c r="C26" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D26" s="130">
+      <c r="D26" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="E26" s="130">
+      <c r="E26" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="F26" s="130">
+      <c r="F26" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="G26" s="130">
+      <c r="G26" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="H26" s="130">
+      <c r="H26" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="I26" s="130">
+      <c r="I26" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="J26" s="130">
+      <c r="J26" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="K26" s="130">
+      <c r="K26" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A26)</f>
         <v/>
       </c>
-      <c r="L26" s="133">
+      <c r="L26" s="142">
         <f>SUM(D26:K26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="127" t="inlineStr">
+      <c r="A27" s="138" t="inlineStr">
         <is>
           <t>REF555</t>
         </is>
       </c>
-      <c r="B27" s="128" t="inlineStr">
+      <c r="B27" s="139" t="inlineStr">
         <is>
           <t>REF555</t>
         </is>
       </c>
-      <c r="C27" s="132" t="inlineStr">
+      <c r="C27" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D27" s="130">
+      <c r="D27" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="E27" s="130">
+      <c r="E27" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="F27" s="130">
+      <c r="F27" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="G27" s="130">
+      <c r="G27" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="H27" s="130">
+      <c r="H27" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="I27" s="130">
+      <c r="I27" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="J27" s="130">
+      <c r="J27" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="K27" s="130">
+      <c r="K27" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A27)</f>
         <v/>
       </c>
-      <c r="L27" s="133">
+      <c r="L27" s="142">
         <f>SUM(D27:K27)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="127" t="inlineStr">
+      <c r="A28" s="138" t="inlineStr">
         <is>
           <t>REF554</t>
         </is>
       </c>
-      <c r="B28" s="128" t="inlineStr">
+      <c r="B28" s="139" t="inlineStr">
         <is>
           <t>REF554</t>
         </is>
       </c>
-      <c r="C28" s="132" t="inlineStr">
+      <c r="C28" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D28" s="130">
+      <c r="D28" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="E28" s="130">
+      <c r="E28" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="F28" s="130">
+      <c r="F28" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="G28" s="130">
+      <c r="G28" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="H28" s="130">
+      <c r="H28" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="I28" s="130">
+      <c r="I28" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="J28" s="130">
+      <c r="J28" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="K28" s="130">
+      <c r="K28" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A28)</f>
         <v/>
       </c>
-      <c r="L28" s="133">
+      <c r="L28" s="142">
         <f>SUM(D28:K28)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="127" t="inlineStr">
+      <c r="A29" s="138" t="inlineStr">
         <is>
           <t>REF575</t>
         </is>
       </c>
-      <c r="B29" s="128" t="inlineStr">
+      <c r="B29" s="139" t="inlineStr">
         <is>
           <t>REF575</t>
         </is>
       </c>
-      <c r="C29" s="132" t="inlineStr">
+      <c r="C29" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D29" s="130">
+      <c r="D29" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="E29" s="130">
+      <c r="E29" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="F29" s="130">
+      <c r="F29" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="G29" s="130">
+      <c r="G29" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="H29" s="130">
+      <c r="H29" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="I29" s="130">
+      <c r="I29" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="J29" s="130">
+      <c r="J29" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="K29" s="130">
+      <c r="K29" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A29)</f>
         <v/>
       </c>
-      <c r="L29" s="133">
+      <c r="L29" s="142">
         <f>SUM(D29:K29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="127" t="inlineStr">
+      <c r="A30" s="138" t="inlineStr">
         <is>
           <t>REF548</t>
         </is>
       </c>
-      <c r="B30" s="128" t="inlineStr">
+      <c r="B30" s="139" t="inlineStr">
         <is>
           <t>REF548</t>
         </is>
       </c>
-      <c r="C30" s="132" t="inlineStr">
+      <c r="C30" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D30" s="130">
+      <c r="D30" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="E30" s="130">
+      <c r="E30" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="F30" s="130">
+      <c r="F30" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="G30" s="130">
+      <c r="G30" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="H30" s="130">
+      <c r="H30" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="I30" s="130">
+      <c r="I30" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="J30" s="130">
+      <c r="J30" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="K30" s="130">
+      <c r="K30" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A30)</f>
         <v/>
       </c>
-      <c r="L30" s="133">
+      <c r="L30" s="142">
         <f>SUM(D30:K30)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="127" t="inlineStr">
+      <c r="A31" s="138" t="inlineStr">
         <is>
           <t>REF557</t>
         </is>
       </c>
-      <c r="B31" s="128" t="inlineStr">
+      <c r="B31" s="139" t="inlineStr">
         <is>
           <t>REF557</t>
         </is>
       </c>
-      <c r="C31" s="132" t="inlineStr">
+      <c r="C31" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D31" s="130">
+      <c r="D31" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="E31" s="130">
+      <c r="E31" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="F31" s="130">
+      <c r="F31" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="G31" s="130">
+      <c r="G31" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="H31" s="130">
+      <c r="H31" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="I31" s="130">
+      <c r="I31" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="J31" s="130">
+      <c r="J31" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="K31" s="130">
+      <c r="K31" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A31)</f>
         <v/>
       </c>
-      <c r="L31" s="133">
+      <c r="L31" s="142">
         <f>SUM(D31:K31)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="127" t="inlineStr">
+      <c r="A32" s="138" t="inlineStr">
         <is>
           <t>REF568</t>
         </is>
       </c>
-      <c r="B32" s="128" t="inlineStr">
+      <c r="B32" s="139" t="inlineStr">
         <is>
           <t>REF568</t>
         </is>
       </c>
-      <c r="C32" s="132" t="inlineStr">
+      <c r="C32" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D32" s="130">
+      <c r="D32" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="E32" s="130">
+      <c r="E32" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="F32" s="130">
+      <c r="F32" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="G32" s="130">
+      <c r="G32" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="H32" s="130">
+      <c r="H32" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="I32" s="130">
+      <c r="I32" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="J32" s="130">
+      <c r="J32" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="K32" s="130">
+      <c r="K32" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A32)</f>
         <v/>
       </c>
-      <c r="L32" s="133">
+      <c r="L32" s="142">
         <f>SUM(D32:K32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="127" t="inlineStr">
+      <c r="A33" s="138" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B33" s="128" t="inlineStr">
+      <c r="B33" s="139" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C33" s="132" t="inlineStr">
+      <c r="C33" s="143" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D33" s="130">
+      <c r="D33" s="141">
         <f>SUMIFS('Live afiliada'!$G:$G,'Live afiliada'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="E33" s="130">
+      <c r="E33" s="141">
         <f>SUMIFS('Vídeo afiliada'!$G:$G,'Vídeo afiliada'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="F33" s="130">
+      <c r="F33" s="141">
         <f>SUMIFS('Card afiliada'!$G:$G,'Card afiliada'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="G33" s="130">
+      <c r="G33" s="141">
         <f>SUMIFS('Live loja'!$G:$G,'Live loja'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="H33" s="130">
+      <c r="H33" s="141">
         <f>SUMIFS('Vídeo loja'!$G:$G,'Vídeo loja'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="I33" s="130">
+      <c r="I33" s="141">
         <f>SUMIFS('Card loja'!$G:$G,'Card loja'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="J33" s="130">
+      <c r="J33" s="141">
         <f>SUMIFS('Vitrine loja'!$G:$G,'Vitrine loja'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="K33" s="130">
+      <c r="K33" s="141">
         <f>SUMIFS('Busca e Mall'!$G:$G,'Busca e Mall'!$A:$A,$A33)</f>
         <v/>
       </c>
-      <c r="L33" s="133">
+      <c r="L33" s="142">
         <f>SUM(D33:K33)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="134" t="inlineStr">
+      <c r="A34" s="144" t="inlineStr">
         <is>
           <t>TOTAL CANAL</t>
         </is>
       </c>
-      <c r="B34" s="135" t="n"/>
-      <c r="C34" s="135" t="n"/>
-      <c r="D34" s="136">
+      <c r="B34" s="145" t="n"/>
+      <c r="C34" s="145" t="n"/>
+      <c r="D34" s="146">
         <f>SUM(D5:D33)</f>
         <v/>
       </c>
-      <c r="E34" s="136">
+      <c r="E34" s="146">
         <f>SUM(E5:E33)</f>
         <v/>
       </c>
-      <c r="F34" s="136">
+      <c r="F34" s="146">
         <f>SUM(F5:F33)</f>
         <v/>
       </c>
-      <c r="G34" s="136">
+      <c r="G34" s="146">
         <f>SUM(G5:G33)</f>
         <v/>
       </c>
-      <c r="H34" s="136">
+      <c r="H34" s="146">
         <f>SUM(H5:H33)</f>
         <v/>
       </c>
-      <c r="I34" s="136">
+      <c r="I34" s="146">
         <f>SUM(I5:I33)</f>
         <v/>
       </c>
-      <c r="J34" s="136">
+      <c r="J34" s="146">
         <f>SUM(J5:J33)</f>
         <v/>
       </c>
-      <c r="K34" s="136">
+      <c r="K34" s="146">
         <f>SUM(K5:K33)</f>
         <v/>
       </c>
-      <c r="L34" s="136">
+      <c r="L34" s="147">
         <f>SUM(L5:L33)</f>
         <v/>
       </c>
@@ -7772,15 +7838,15 @@
     <row r="36">
       <c r="A36" s="137" t="inlineStr">
         <is>
-          <t>Hero=REF516/525/527. Card afiliada=linha AGREGADO. Vitrine (transversal) e Busca (=0) não somam peças. Recalcula ao editar Premissas/Ajuste.</t>
+          <t>Hero=REF516/525/527. Card afiliada=AGREGADO. Vitrine (transversal) e Busca (=0) não somam peças.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A36:L36"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(margem): aba Alavancas de Margem — 4 alavancas ranqueadas por R$/mês (devolução/combo/recompra/mídia) + P&L da peça única
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
+++ b/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
@@ -13,15 +13,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Soma SKU x Canal" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alavancas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live afiliada" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo afiliada" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card afiliada" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live loja" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo loja" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card loja" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitrine loja" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busca e Mall" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log diário" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alavancas de Margem" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live afiliada" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo afiliada" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card afiliada" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live loja" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo loja" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card loja" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitrine loja" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busca e Mall" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log diário" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -30,7 +31,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.00\x"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -41,8 +42,9 @@
     <numFmt numFmtId="171" formatCode="#,##0&quot;/d&quot;"/>
     <numFmt numFmtId="172" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
+    <numFmt numFmtId="174" formatCode="&quot;R$&quot; #,##0"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="43">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -265,8 +267,47 @@
       <color rgb="001E7E34"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E7E34"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00777777"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B8860B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E7E34"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A1A1A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -331,6 +372,21 @@
         <fgColor rgb="00E8F5E9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C0392B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E7E34"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007A7A7A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -380,7 +436,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -871,6 +927,74 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="41" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="37" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="34" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="34" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="34" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="42" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="24" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="32" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -943,6 +1067,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="B35" authorId="0" shapeId="0">
+      <text>
+        <t>Se 7,8 for ROI de LUCRO (nao ROAS), esta alavanca dispara pra 6 digitos e vira a #1. Preciso puxar o dado real de contribuicao da midia pra travar. Formula conservadora (ROAS x margem - midia): a 11% de margem ela mal se paga.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1786,6 +1925,475 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="10" customWidth="1" style="62" min="1" max="1"/>
+    <col width="22" customWidth="1" style="62" min="2" max="2"/>
+    <col width="5" customWidth="1" style="62" min="3" max="3"/>
+    <col width="12" customWidth="1" style="62" min="4" max="4"/>
+    <col width="8" customWidth="1" style="62" min="5" max="5"/>
+    <col width="10" customWidth="1" style="62" min="6" max="7"/>
+    <col width="11" customWidth="1" style="62" min="8" max="8"/>
+    <col width="12" customWidth="1" style="62" min="9" max="9"/>
+    <col width="9" customWidth="1" style="62" min="10" max="10"/>
+    <col width="11" customWidth="1" style="62" min="11" max="11"/>
+    <col width="13" customWidth="1" style="62" min="12" max="12"/>
+    <col width="12" customWidth="1" style="62" min="13" max="13"/>
+    <col width="13" customWidth="1" style="62" min="14" max="15"/>
+    <col width="11" customWidth="1" style="62" min="16" max="16"/>
+    <col width="12" customWidth="1" style="62" min="17" max="18"/>
+    <col width="14" customWidth="1" style="62" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.15" customHeight="1" s="63">
+      <c r="A1" s="64" t="inlineStr">
+        <is>
+          <t>Card afiliada — meta por SKU e pace diário</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="63">
+      <c r="A2" s="66" t="inlineStr">
+        <is>
+          <t>Canal (chave):</t>
+        </is>
+      </c>
+      <c r="B2" s="89" t="inlineStr">
+        <is>
+          <t>Card afiliada</t>
+        </is>
+      </c>
+      <c r="C2" s="66" t="inlineStr">
+        <is>
+          <t>Superfície:</t>
+        </is>
+      </c>
+      <c r="D2" s="89" t="inlineStr">
+        <is>
+          <t>CARD DE PRODUTO</t>
+        </is>
+      </c>
+      <c r="F2" s="66" t="inlineStr">
+        <is>
+          <t>Atribuição:</t>
+        </is>
+      </c>
+      <c r="G2" s="89" t="inlineStr">
+        <is>
+          <t>Afiliada</t>
+        </is>
+      </c>
+      <c r="I2" s="66" t="inlineStr">
+        <is>
+          <t>Confiança da base jul:</t>
+        </is>
+      </c>
+      <c r="K2" s="121" t="inlineStr">
+        <is>
+          <t>EXATO — afiliada showcase/card (SHOP+LINKSHARE) do extrato. ~1,5% do GMV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="63">
+      <c r="A3" s="66" t="inlineStr">
+        <is>
+          <t>Alavanca principal:</t>
+        </is>
+      </c>
+      <c r="B3" s="89" t="inlineStr">
+        <is>
+          <t>A definir — depende de abrir a fonte no extrato de afiliada</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="63">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>Crescimento vs base:</t>
+        </is>
+      </c>
+      <c r="B4" s="107">
+        <f>Premissas!$C$27</f>
+        <v/>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Comissão afiliada:</t>
+        </is>
+      </c>
+      <c r="D4" s="107">
+        <f>Premissas!$D$27</f>
+        <v/>
+      </c>
+      <c r="F4" s="66" t="inlineStr">
+        <is>
+          <t>CPV padrão:</t>
+        </is>
+      </c>
+      <c r="G4" s="108">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="63">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>Meta do canal (pç):</t>
+        </is>
+      </c>
+      <c r="B5" s="109">
+        <f>G9</f>
+        <v/>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>Meta GMV:</t>
+        </is>
+      </c>
+      <c r="D5" s="110">
+        <f>I9</f>
+        <v/>
+      </c>
+      <c r="F5" s="66" t="inlineStr">
+        <is>
+          <t>Contribuição meta:</t>
+        </is>
+      </c>
+      <c r="G5" s="110">
+        <f>L9</f>
+        <v/>
+      </c>
+      <c r="I5" s="66" t="inlineStr">
+        <is>
+          <t>Índice de pace:</t>
+        </is>
+      </c>
+      <c r="K5" s="111">
+        <f>P9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="63">
+      <c r="A7" s="72" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B7" s="72" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>Base jul (pç)</t>
+        </is>
+      </c>
+      <c r="E7" s="72" t="inlineStr">
+        <is>
+          <t>Mix jul</t>
+        </is>
+      </c>
+      <c r="F7" s="72" t="inlineStr">
+        <is>
+          <t>Ajuste (pç)</t>
+        </is>
+      </c>
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>Meta (pç)</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="inlineStr">
+        <is>
+          <t>Preço plan.</t>
+        </is>
+      </c>
+      <c r="I7" s="72" t="inlineStr">
+        <is>
+          <t>Meta GMV</t>
+        </is>
+      </c>
+      <c r="J7" s="72" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="K7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib./pç</t>
+        </is>
+      </c>
+      <c r="L7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib. meta</t>
+        </is>
+      </c>
+      <c r="M7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (pç)</t>
+        </is>
+      </c>
+      <c r="N7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (R$)</t>
+        </is>
+      </c>
+      <c r="O7" s="72" t="inlineStr">
+        <is>
+          <t>Esperado MTD</t>
+        </is>
+      </c>
+      <c r="P7" s="72" t="inlineStr">
+        <is>
+          <t>Índice pace</t>
+        </is>
+      </c>
+      <c r="Q7" s="72" t="inlineStr">
+        <is>
+          <t>Projeção fim</t>
+        </is>
+      </c>
+      <c r="R7" s="72" t="inlineStr">
+        <is>
+          <t>Gap vs meta</t>
+        </is>
+      </c>
+      <c r="S7" s="72" t="inlineStr">
+        <is>
+          <t>Pç/dia p/ fechar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="63">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>AGREGADO</t>
+        </is>
+      </c>
+      <c r="B8" s="74" t="inlineStr">
+        <is>
+          <t>Afiliada showcase/card (SHOP+LINKSHARE)</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D8" s="112" t="n">
+        <v>75</v>
+      </c>
+      <c r="E8" s="113">
+        <f>IFERROR(D8/$D$9,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="112">
+        <f>ROUND(D8*(1+$B$4),0)+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="97" t="n">
+        <v>94.98</v>
+      </c>
+      <c r="I8" s="114">
+        <f>G8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K8" s="116">
+        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="114">
+        <f>G8*K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="112">
+        <f>G8*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P8" s="117">
+        <f>IFERROR(M8/O8,0)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="112">
+        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R8" s="112">
+        <f>Q8-G8</f>
+        <v/>
+      </c>
+      <c r="S8" s="118">
+        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="63">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="n"/>
+      <c r="C9" s="81" t="n"/>
+      <c r="D9" s="82">
+        <f>SUM(D8:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="85">
+        <f>SUM(E8:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="82">
+        <f>SUM(F8:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="82">
+        <f>SUM(G8:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="119" t="n"/>
+      <c r="I9" s="83">
+        <f>SUM(I8:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="119" t="n"/>
+      <c r="K9" s="119" t="n"/>
+      <c r="L9" s="83">
+        <f>SUM(L8:L8)</f>
+        <v/>
+      </c>
+      <c r="M9" s="82">
+        <f>SUM(M8:M8)</f>
+        <v/>
+      </c>
+      <c r="N9" s="83">
+        <f>SUM(N8:N8)</f>
+        <v/>
+      </c>
+      <c r="O9" s="82">
+        <f>SUM(O8:O8)</f>
+        <v/>
+      </c>
+      <c r="P9" s="84">
+        <f>IFERROR(M9/O9,0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="82">
+        <f>SUM(Q8:Q8)</f>
+        <v/>
+      </c>
+      <c r="R9" s="82">
+        <f>SUM(R8:R8)</f>
+        <v/>
+      </c>
+      <c r="S9" s="120">
+        <f>SUM(S8:S8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="63">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>Σ Hero</t>
+        </is>
+      </c>
+      <c r="B10" s="74" t="n"/>
+      <c r="C10" s="74" t="n"/>
+      <c r="D10" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="E10" s="74" t="n"/>
+      <c r="F10" s="74" t="n"/>
+      <c r="G10" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="H10" s="74" t="n"/>
+      <c r="I10" s="74" t="n"/>
+      <c r="J10" s="74" t="n"/>
+      <c r="K10" s="74" t="n"/>
+      <c r="L10" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="63">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>Σ Esteira</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="n"/>
+      <c r="C11" s="74" t="n"/>
+      <c r="D11" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="E11" s="74" t="n"/>
+      <c r="F11" s="74" t="n"/>
+      <c r="G11" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="H11" s="74" t="n"/>
+      <c r="I11" s="74" t="n"/>
+      <c r="J11" s="74" t="n"/>
+      <c r="K11" s="74" t="n"/>
+      <c r="L11" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="63">
+      <c r="A13" s="71" t="inlineStr">
+        <is>
+          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="63">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:S36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
@@ -3965,7 +4573,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4590,7 +5198,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5593,475 +6201,6 @@
     </row>
     <row r="21" ht="15" customHeight="1" s="63">
       <c r="A21" s="71" t="inlineStr">
-        <is>
-          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="10" customWidth="1" style="62" min="1" max="1"/>
-    <col width="22" customWidth="1" style="62" min="2" max="2"/>
-    <col width="5" customWidth="1" style="62" min="3" max="3"/>
-    <col width="12" customWidth="1" style="62" min="4" max="4"/>
-    <col width="8" customWidth="1" style="62" min="5" max="5"/>
-    <col width="10" customWidth="1" style="62" min="6" max="7"/>
-    <col width="11" customWidth="1" style="62" min="8" max="8"/>
-    <col width="12" customWidth="1" style="62" min="9" max="9"/>
-    <col width="9" customWidth="1" style="62" min="10" max="10"/>
-    <col width="11" customWidth="1" style="62" min="11" max="11"/>
-    <col width="13" customWidth="1" style="62" min="12" max="12"/>
-    <col width="12" customWidth="1" style="62" min="13" max="13"/>
-    <col width="13" customWidth="1" style="62" min="14" max="15"/>
-    <col width="11" customWidth="1" style="62" min="16" max="16"/>
-    <col width="12" customWidth="1" style="62" min="17" max="18"/>
-    <col width="14" customWidth="1" style="62" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="63">
-      <c r="A1" s="64" t="inlineStr">
-        <is>
-          <t>Vitrine loja — meta por SKU e pace diário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="63">
-      <c r="A2" s="66" t="inlineStr">
-        <is>
-          <t>Canal (chave):</t>
-        </is>
-      </c>
-      <c r="B2" s="89" t="inlineStr">
-        <is>
-          <t>Vitrine loja</t>
-        </is>
-      </c>
-      <c r="C2" s="66" t="inlineStr">
-        <is>
-          <t>Superfície:</t>
-        </is>
-      </c>
-      <c r="D2" s="89" t="inlineStr">
-        <is>
-          <t>VITRINE DA LOJA</t>
-        </is>
-      </c>
-      <c r="F2" s="66" t="inlineStr">
-        <is>
-          <t>Atribuição:</t>
-        </is>
-      </c>
-      <c r="G2" s="89" t="inlineStr">
-        <is>
-          <t>Loja / vendedor</t>
-        </is>
-      </c>
-      <c r="I2" s="66" t="inlineStr">
-        <is>
-          <t>Confiança da base jul:</t>
-        </is>
-      </c>
-      <c r="K2" s="121" t="inlineStr">
-        <is>
-          <t>TRANSVERSAL — shop_tab R$89.369 (jul, API 202605) SOBREPÕE card/loja; não somável no NET (lente de superfície, não de último-conteúdo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="63">
-      <c r="A3" s="66" t="inlineStr">
-        <is>
-          <t>Alavanca principal:</t>
-        </is>
-      </c>
-      <c r="B3" s="89" t="inlineStr">
-        <is>
-          <t>A definir — organizar vitrine por curva e coleção</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="63">
-      <c r="A4" s="66" t="inlineStr">
-        <is>
-          <t>Crescimento vs base:</t>
-        </is>
-      </c>
-      <c r="B4" s="107">
-        <f>Premissas!$C$31</f>
-        <v/>
-      </c>
-      <c r="C4" s="66" t="inlineStr">
-        <is>
-          <t>Comissão afiliada:</t>
-        </is>
-      </c>
-      <c r="D4" s="107">
-        <f>Premissas!$D$31</f>
-        <v/>
-      </c>
-      <c r="F4" s="66" t="inlineStr">
-        <is>
-          <t>CPV padrão:</t>
-        </is>
-      </c>
-      <c r="G4" s="108">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="63">
-      <c r="A5" s="66" t="inlineStr">
-        <is>
-          <t>Meta do canal (pç):</t>
-        </is>
-      </c>
-      <c r="B5" s="109">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="C5" s="66" t="inlineStr">
-        <is>
-          <t>Meta GMV:</t>
-        </is>
-      </c>
-      <c r="D5" s="110">
-        <f>I9</f>
-        <v/>
-      </c>
-      <c r="F5" s="66" t="inlineStr">
-        <is>
-          <t>Contribuição meta:</t>
-        </is>
-      </c>
-      <c r="G5" s="110">
-        <f>L9</f>
-        <v/>
-      </c>
-      <c r="I5" s="66" t="inlineStr">
-        <is>
-          <t>Índice de pace:</t>
-        </is>
-      </c>
-      <c r="K5" s="111">
-        <f>P9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="63">
-      <c r="A7" s="72" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B7" s="72" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="C7" s="72" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="D7" s="72" t="inlineStr">
-        <is>
-          <t>Base jul (pç)</t>
-        </is>
-      </c>
-      <c r="E7" s="72" t="inlineStr">
-        <is>
-          <t>Mix jul</t>
-        </is>
-      </c>
-      <c r="F7" s="72" t="inlineStr">
-        <is>
-          <t>Ajuste (pç)</t>
-        </is>
-      </c>
-      <c r="G7" s="72" t="inlineStr">
-        <is>
-          <t>Meta (pç)</t>
-        </is>
-      </c>
-      <c r="H7" s="72" t="inlineStr">
-        <is>
-          <t>Preço plan.</t>
-        </is>
-      </c>
-      <c r="I7" s="72" t="inlineStr">
-        <is>
-          <t>Meta GMV</t>
-        </is>
-      </c>
-      <c r="J7" s="72" t="inlineStr">
-        <is>
-          <t>CPV</t>
-        </is>
-      </c>
-      <c r="K7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib./pç</t>
-        </is>
-      </c>
-      <c r="L7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib. meta</t>
-        </is>
-      </c>
-      <c r="M7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (pç)</t>
-        </is>
-      </c>
-      <c r="N7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (R$)</t>
-        </is>
-      </c>
-      <c r="O7" s="72" t="inlineStr">
-        <is>
-          <t>Esperado MTD</t>
-        </is>
-      </c>
-      <c r="P7" s="72" t="inlineStr">
-        <is>
-          <t>Índice pace</t>
-        </is>
-      </c>
-      <c r="Q7" s="72" t="inlineStr">
-        <is>
-          <t>Projeção fim</t>
-        </is>
-      </c>
-      <c r="R7" s="72" t="inlineStr">
-        <is>
-          <t>Gap vs meta</t>
-        </is>
-      </c>
-      <c r="S7" s="72" t="inlineStr">
-        <is>
-          <t>Pç/dia p/ fechar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="63">
-      <c r="A8" s="73" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B8" s="74" t="inlineStr">
-        <is>
-          <t>Sem base de julho para este canal</t>
-        </is>
-      </c>
-      <c r="C8" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="113">
-        <f>IFERROR(D8/$D$9,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="112">
-        <f>ROUND(D8*(1+$B$4),0)+F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="97" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="114">
-        <f>G8*H8</f>
-        <v/>
-      </c>
-      <c r="J8" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K8" s="116">
-        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="114">
-        <f>G8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="112">
-        <f>G8*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P8" s="117">
-        <f>IFERROR(M8/O8,0)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="112">
-        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R8" s="112">
-        <f>Q8-G8</f>
-        <v/>
-      </c>
-      <c r="S8" s="118">
-        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="63">
-      <c r="A9" s="81" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B9" s="81" t="n"/>
-      <c r="C9" s="81" t="n"/>
-      <c r="D9" s="82">
-        <f>SUM(D8:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="85">
-        <f>SUM(E8:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="82">
-        <f>SUM(F8:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="82">
-        <f>SUM(G8:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="119" t="n"/>
-      <c r="I9" s="83">
-        <f>SUM(I8:I8)</f>
-        <v/>
-      </c>
-      <c r="J9" s="119" t="n"/>
-      <c r="K9" s="119" t="n"/>
-      <c r="L9" s="83">
-        <f>SUM(L8:L8)</f>
-        <v/>
-      </c>
-      <c r="M9" s="82">
-        <f>SUM(M8:M8)</f>
-        <v/>
-      </c>
-      <c r="N9" s="83">
-        <f>SUM(N8:N8)</f>
-        <v/>
-      </c>
-      <c r="O9" s="82">
-        <f>SUM(O8:O8)</f>
-        <v/>
-      </c>
-      <c r="P9" s="84">
-        <f>IFERROR(M9/O9,0)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="82">
-        <f>SUM(Q8:Q8)</f>
-        <v/>
-      </c>
-      <c r="R9" s="82">
-        <f>SUM(R8:R8)</f>
-        <v/>
-      </c>
-      <c r="S9" s="120">
-        <f>SUM(S8:S8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="63">
-      <c r="A10" s="73" t="inlineStr">
-        <is>
-          <t>Σ Hero</t>
-        </is>
-      </c>
-      <c r="B10" s="74" t="n"/>
-      <c r="C10" s="74" t="n"/>
-      <c r="D10" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="E10" s="74" t="n"/>
-      <c r="F10" s="74" t="n"/>
-      <c r="G10" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="H10" s="74" t="n"/>
-      <c r="I10" s="74" t="n"/>
-      <c r="J10" s="74" t="n"/>
-      <c r="K10" s="74" t="n"/>
-      <c r="L10" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="63">
-      <c r="A11" s="73" t="inlineStr">
-        <is>
-          <t>Σ Esteira</t>
-        </is>
-      </c>
-      <c r="B11" s="74" t="n"/>
-      <c r="C11" s="74" t="n"/>
-      <c r="D11" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="E11" s="74" t="n"/>
-      <c r="F11" s="74" t="n"/>
-      <c r="G11" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="H11" s="74" t="n"/>
-      <c r="I11" s="74" t="n"/>
-      <c r="J11" s="74" t="n"/>
-      <c r="K11" s="74" t="n"/>
-      <c r="L11" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="63">
-      <c r="A13" s="71" t="inlineStr">
-        <is>
-          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="63">
-      <c r="A14" s="71" t="inlineStr">
         <is>
           <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
         </is>
@@ -6104,7 +6243,7 @@
     <row r="1" ht="16.15" customHeight="1" s="63">
       <c r="A1" s="64" t="inlineStr">
         <is>
-          <t>Busca e Mall — meta por SKU e pace diário</t>
+          <t>Vitrine loja — meta por SKU e pace diário</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6255,7 @@
       </c>
       <c r="B2" s="89" t="inlineStr">
         <is>
-          <t>Busca e Mall</t>
+          <t>Vitrine loja</t>
         </is>
       </c>
       <c r="C2" s="66" t="inlineStr">
@@ -6126,7 +6265,7 @@
       </c>
       <c r="D2" s="89" t="inlineStr">
         <is>
-          <t>BUSCA / MALL / OUTROS</t>
+          <t>VITRINE DA LOJA</t>
         </is>
       </c>
       <c r="F2" s="66" t="inlineStr">
@@ -6136,7 +6275,7 @@
       </c>
       <c r="G2" s="89" t="inlineStr">
         <is>
-          <t>Misto</t>
+          <t>Loja / vendedor</t>
         </is>
       </c>
       <c r="I2" s="66" t="inlineStr">
@@ -6146,7 +6285,7 @@
       </c>
       <c r="K2" s="121" t="inlineStr">
         <is>
-          <t>R$0 — nesta atribuição (API 202605) total = seller(live+vídeo+card)+afiliada, resíduo zero. Sem balde separado.</t>
+          <t>TRANSVERSAL — shop_tab R$89.369 (jul, API 202605) SOBREPÕE card/loja; não somável no NET (lente de superfície, não de último-conteúdo).</t>
         </is>
       </c>
     </row>
@@ -6158,7 +6297,7 @@
       </c>
       <c r="B3" s="89" t="inlineStr">
         <is>
-          <t>A definir — SEO de título/atributo de produto</t>
+          <t>A definir — organizar vitrine por curva e coleção</t>
         </is>
       </c>
     </row>
@@ -6169,7 +6308,7 @@
         </is>
       </c>
       <c r="B4" s="107">
-        <f>Premissas!$C$32</f>
+        <f>Premissas!$C$31</f>
         <v/>
       </c>
       <c r="C4" s="66" t="inlineStr">
@@ -6178,7 +6317,7 @@
         </is>
       </c>
       <c r="D4" s="107">
-        <f>Premissas!$D$32</f>
+        <f>Premissas!$D$31</f>
         <v/>
       </c>
       <c r="F4" s="66" t="inlineStr">
@@ -6544,6 +6683,475 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="10" customWidth="1" style="62" min="1" max="1"/>
+    <col width="22" customWidth="1" style="62" min="2" max="2"/>
+    <col width="5" customWidth="1" style="62" min="3" max="3"/>
+    <col width="12" customWidth="1" style="62" min="4" max="4"/>
+    <col width="8" customWidth="1" style="62" min="5" max="5"/>
+    <col width="10" customWidth="1" style="62" min="6" max="7"/>
+    <col width="11" customWidth="1" style="62" min="8" max="8"/>
+    <col width="12" customWidth="1" style="62" min="9" max="9"/>
+    <col width="9" customWidth="1" style="62" min="10" max="10"/>
+    <col width="11" customWidth="1" style="62" min="11" max="11"/>
+    <col width="13" customWidth="1" style="62" min="12" max="12"/>
+    <col width="12" customWidth="1" style="62" min="13" max="13"/>
+    <col width="13" customWidth="1" style="62" min="14" max="15"/>
+    <col width="11" customWidth="1" style="62" min="16" max="16"/>
+    <col width="12" customWidth="1" style="62" min="17" max="18"/>
+    <col width="14" customWidth="1" style="62" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.15" customHeight="1" s="63">
+      <c r="A1" s="64" t="inlineStr">
+        <is>
+          <t>Busca e Mall — meta por SKU e pace diário</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="63">
+      <c r="A2" s="66" t="inlineStr">
+        <is>
+          <t>Canal (chave):</t>
+        </is>
+      </c>
+      <c r="B2" s="89" t="inlineStr">
+        <is>
+          <t>Busca e Mall</t>
+        </is>
+      </c>
+      <c r="C2" s="66" t="inlineStr">
+        <is>
+          <t>Superfície:</t>
+        </is>
+      </c>
+      <c r="D2" s="89" t="inlineStr">
+        <is>
+          <t>BUSCA / MALL / OUTROS</t>
+        </is>
+      </c>
+      <c r="F2" s="66" t="inlineStr">
+        <is>
+          <t>Atribuição:</t>
+        </is>
+      </c>
+      <c r="G2" s="89" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="I2" s="66" t="inlineStr">
+        <is>
+          <t>Confiança da base jul:</t>
+        </is>
+      </c>
+      <c r="K2" s="121" t="inlineStr">
+        <is>
+          <t>R$0 — nesta atribuição (API 202605) total = seller(live+vídeo+card)+afiliada, resíduo zero. Sem balde separado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="63">
+      <c r="A3" s="66" t="inlineStr">
+        <is>
+          <t>Alavanca principal:</t>
+        </is>
+      </c>
+      <c r="B3" s="89" t="inlineStr">
+        <is>
+          <t>A definir — SEO de título/atributo de produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="63">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>Crescimento vs base:</t>
+        </is>
+      </c>
+      <c r="B4" s="107">
+        <f>Premissas!$C$32</f>
+        <v/>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Comissão afiliada:</t>
+        </is>
+      </c>
+      <c r="D4" s="107">
+        <f>Premissas!$D$32</f>
+        <v/>
+      </c>
+      <c r="F4" s="66" t="inlineStr">
+        <is>
+          <t>CPV padrão:</t>
+        </is>
+      </c>
+      <c r="G4" s="108">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="63">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>Meta do canal (pç):</t>
+        </is>
+      </c>
+      <c r="B5" s="109">
+        <f>G9</f>
+        <v/>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>Meta GMV:</t>
+        </is>
+      </c>
+      <c r="D5" s="110">
+        <f>I9</f>
+        <v/>
+      </c>
+      <c r="F5" s="66" t="inlineStr">
+        <is>
+          <t>Contribuição meta:</t>
+        </is>
+      </c>
+      <c r="G5" s="110">
+        <f>L9</f>
+        <v/>
+      </c>
+      <c r="I5" s="66" t="inlineStr">
+        <is>
+          <t>Índice de pace:</t>
+        </is>
+      </c>
+      <c r="K5" s="111">
+        <f>P9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="63">
+      <c r="A7" s="72" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B7" s="72" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>Base jul (pç)</t>
+        </is>
+      </c>
+      <c r="E7" s="72" t="inlineStr">
+        <is>
+          <t>Mix jul</t>
+        </is>
+      </c>
+      <c r="F7" s="72" t="inlineStr">
+        <is>
+          <t>Ajuste (pç)</t>
+        </is>
+      </c>
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>Meta (pç)</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="inlineStr">
+        <is>
+          <t>Preço plan.</t>
+        </is>
+      </c>
+      <c r="I7" s="72" t="inlineStr">
+        <is>
+          <t>Meta GMV</t>
+        </is>
+      </c>
+      <c r="J7" s="72" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="K7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib./pç</t>
+        </is>
+      </c>
+      <c r="L7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib. meta</t>
+        </is>
+      </c>
+      <c r="M7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (pç)</t>
+        </is>
+      </c>
+      <c r="N7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (R$)</t>
+        </is>
+      </c>
+      <c r="O7" s="72" t="inlineStr">
+        <is>
+          <t>Esperado MTD</t>
+        </is>
+      </c>
+      <c r="P7" s="72" t="inlineStr">
+        <is>
+          <t>Índice pace</t>
+        </is>
+      </c>
+      <c r="Q7" s="72" t="inlineStr">
+        <is>
+          <t>Projeção fim</t>
+        </is>
+      </c>
+      <c r="R7" s="72" t="inlineStr">
+        <is>
+          <t>Gap vs meta</t>
+        </is>
+      </c>
+      <c r="S7" s="72" t="inlineStr">
+        <is>
+          <t>Pç/dia p/ fechar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="63">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B8" s="74" t="inlineStr">
+        <is>
+          <t>Sem base de julho para este canal</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="113">
+        <f>IFERROR(D8/$D$9,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="112">
+        <f>ROUND(D8*(1+$B$4),0)+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="114">
+        <f>G8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K8" s="116">
+        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="114">
+        <f>G8*K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="112">
+        <f>G8*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P8" s="117">
+        <f>IFERROR(M8/O8,0)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="112">
+        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R8" s="112">
+        <f>Q8-G8</f>
+        <v/>
+      </c>
+      <c r="S8" s="118">
+        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="63">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="n"/>
+      <c r="C9" s="81" t="n"/>
+      <c r="D9" s="82">
+        <f>SUM(D8:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="85">
+        <f>SUM(E8:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="82">
+        <f>SUM(F8:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="82">
+        <f>SUM(G8:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="119" t="n"/>
+      <c r="I9" s="83">
+        <f>SUM(I8:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="119" t="n"/>
+      <c r="K9" s="119" t="n"/>
+      <c r="L9" s="83">
+        <f>SUM(L8:L8)</f>
+        <v/>
+      </c>
+      <c r="M9" s="82">
+        <f>SUM(M8:M8)</f>
+        <v/>
+      </c>
+      <c r="N9" s="83">
+        <f>SUM(N8:N8)</f>
+        <v/>
+      </c>
+      <c r="O9" s="82">
+        <f>SUM(O8:O8)</f>
+        <v/>
+      </c>
+      <c r="P9" s="84">
+        <f>IFERROR(M9/O9,0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="82">
+        <f>SUM(Q8:Q8)</f>
+        <v/>
+      </c>
+      <c r="R9" s="82">
+        <f>SUM(R8:R8)</f>
+        <v/>
+      </c>
+      <c r="S9" s="120">
+        <f>SUM(S8:S8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="63">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>Σ Hero</t>
+        </is>
+      </c>
+      <c r="B10" s="74" t="n"/>
+      <c r="C10" s="74" t="n"/>
+      <c r="D10" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="E10" s="74" t="n"/>
+      <c r="F10" s="74" t="n"/>
+      <c r="G10" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="H10" s="74" t="n"/>
+      <c r="I10" s="74" t="n"/>
+      <c r="J10" s="74" t="n"/>
+      <c r="K10" s="74" t="n"/>
+      <c r="L10" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="63">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>Σ Esteira</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="n"/>
+      <c r="C11" s="74" t="n"/>
+      <c r="D11" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="E11" s="74" t="n"/>
+      <c r="F11" s="74" t="n"/>
+      <c r="G11" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="H11" s="74" t="n"/>
+      <c r="I11" s="74" t="n"/>
+      <c r="J11" s="74" t="n"/>
+      <c r="K11" s="74" t="n"/>
+      <c r="L11" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="63">
+      <c r="A13" s="71" t="inlineStr">
+        <is>
+          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="63">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11579,6 +12187,598 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" style="63" min="1" max="1"/>
+    <col width="15" customWidth="1" style="63" min="2" max="2"/>
+    <col width="34" customWidth="1" style="63" min="3" max="3"/>
+    <col width="12" customWidth="1" style="63" min="4" max="4"/>
+    <col width="10" customWidth="1" style="63" min="5" max="5"/>
+    <col width="12" customWidth="1" style="63" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="63">
+      <c r="A1" s="148" t="inlineStr">
+        <is>
+          <t>Alavancas de Margem — como escalar SEM promoção</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="125" t="inlineStr">
+        <is>
+          <t>A peça única com mídia dá contribuição NEGATIVA (ver diagnóstico no rodapé). A alavanca não é preço — é tapar vazamento, subir cesta e vender sem CAC. Amarelo = premissa editável. Ranqueado por R$/mês.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="176" t="inlineStr">
+        <is>
+          <t>POTENCIAL TOTAL/mês (aprox)</t>
+        </is>
+      </c>
+      <c r="B4" s="177">
+        <f>B16+B21+B27+B34</f>
+        <v/>
+      </c>
+      <c r="C4" s="178" t="inlineStr">
+        <is>
+          <t>L3=por ciclo · L4=condicional (ver nota). Priorização, não caixa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="156" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="156" t="inlineStr">
+        <is>
+          <t>Alavanca</t>
+        </is>
+      </c>
+      <c r="C6" s="156" t="inlineStr">
+        <is>
+          <t>R$/mês</t>
+        </is>
+      </c>
+      <c r="D6" s="156" t="inlineStr">
+        <is>
+          <t>CAC</t>
+        </is>
+      </c>
+      <c r="E6" s="156" t="inlineStr">
+        <is>
+          <t>Prazo</t>
+        </is>
+      </c>
+      <c r="F6" s="156" t="inlineStr">
+        <is>
+          <t>Confiança</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="179" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="180" t="inlineStr">
+        <is>
+          <t>Tapar devolução por modelagem</t>
+        </is>
+      </c>
+      <c r="C7" s="181">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="D7" s="182" t="inlineStr">
+        <is>
+          <t>zero</t>
+        </is>
+      </c>
+      <c r="E7" s="182" t="inlineStr">
+        <is>
+          <t>2–4 sem</t>
+        </is>
+      </c>
+      <c r="F7" s="182" t="inlineStr">
+        <is>
+          <t>✅ dado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="179" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="180" t="inlineStr">
+        <is>
+          <t>Combo / AOV (cesta)</t>
+        </is>
+      </c>
+      <c r="C8" s="181">
+        <f>B21</f>
+        <v/>
+      </c>
+      <c r="D8" s="182" t="inlineStr">
+        <is>
+          <t>dilui</t>
+        </is>
+      </c>
+      <c r="E8" s="182" t="inlineStr">
+        <is>
+          <t>1–2 sem</t>
+        </is>
+      </c>
+      <c r="F8" s="182" t="inlineStr">
+        <is>
+          <t>⏳ modelar</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="179" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="180" t="inlineStr">
+        <is>
+          <t>Recompra — dono da base</t>
+        </is>
+      </c>
+      <c r="C9" s="181">
+        <f>B27</f>
+        <v/>
+      </c>
+      <c r="D9" s="182" t="inlineStr">
+        <is>
+          <t>zero</t>
+        </is>
+      </c>
+      <c r="E9" s="182" t="inlineStr">
+        <is>
+          <t>4–8 sem</t>
+        </is>
+      </c>
+      <c r="F9" s="182" t="inlineStr">
+        <is>
+          <t>⏳ ciclo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="179" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="180" t="inlineStr">
+        <is>
+          <t>Mídia lucrativa (SKUs certos)</t>
+        </is>
+      </c>
+      <c r="C10" s="181">
+        <f>B34</f>
+        <v/>
+      </c>
+      <c r="D10" s="182" t="inlineStr">
+        <is>
+          <t>alto</t>
+        </is>
+      </c>
+      <c r="E10" s="182" t="inlineStr">
+        <is>
+          <t>imediato</t>
+        </is>
+      </c>
+      <c r="F10" s="182" t="inlineStr">
+        <is>
+          <t>⏳ confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="175" t="inlineStr">
+        <is>
+          <t>Ordem de ataque: 1→2→3 destravam margem com CAC baixo/zero e sobem a base de contribuição. Só DEPOIS a mídia (4) escala com folga — a nota da L4 mostra por que ela mal se paga na margem de hoje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="15" ht="20" customHeight="1" s="63">
+      <c r="A15" s="183" t="inlineStr">
+        <is>
+          <t>1 · Tapar o vazamento de devolução por modelagem</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="149" t="inlineStr">
+        <is>
+          <t>R$/mês destravado</t>
+        </is>
+      </c>
+      <c r="B16" s="184">
+        <f>B16*B17</f>
+        <v/>
+      </c>
+      <c r="C16" s="185" t="inlineStr">
+        <is>
+          <t>CAC: zero  ·  2–4 sem</t>
+        </is>
+      </c>
+      <c r="D16" s="186" t="inlineStr">
+        <is>
+          <t>✅ dado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="187" t="inlineStr">
+        <is>
+          <t>Perda mensal por modelagem ("não serviu", pior tam 46)</t>
+        </is>
+      </c>
+      <c r="B17" s="188" t="n">
+        <v>77000</v>
+      </c>
+      <c r="C17" s="178" t="inlineStr">
+        <is>
+          <t>análise devoluções ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="187" t="inlineStr">
+        <is>
+          <t>% recuperável (grade/size finder/foto de caimento)</t>
+        </is>
+      </c>
+      <c r="B18" s="189" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C18" s="178" t="inlineStr">
+        <is>
+          <t>premissa ⏳ — o mais controlável</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" s="63">
+      <c r="A20" s="190" t="inlineStr">
+        <is>
+          <t>2 · Subir a cesta (AOV) — combo dilui o CAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="149" t="inlineStr">
+        <is>
+          <t>R$/mês destravado</t>
+        </is>
+      </c>
+      <c r="B21" s="184">
+        <f>B22*B23*B24</f>
+        <v/>
+      </c>
+      <c r="C21" s="185" t="inlineStr">
+        <is>
+          <t>CAC: dilui  ·  1–2 sem</t>
+        </is>
+      </c>
+      <c r="D21" s="191" t="inlineStr">
+        <is>
+          <t>⏳ modelar</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="187" t="inlineStr">
+        <is>
+          <t>Pedidos/mês elegíveis a combo</t>
+        </is>
+      </c>
+      <c r="B22" s="170" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C22" s="178" t="inlineStr">
+        <is>
+          <t>base editável</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="187" t="inlineStr">
+        <is>
+          <t>% adesão ao combo</t>
+        </is>
+      </c>
+      <c r="B23" s="189" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="178" t="inlineStr">
+        <is>
+          <t>meta editável</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="187" t="inlineStr">
+        <is>
+          <t>Contribuição incremental por combo (R$)</t>
+        </is>
+      </c>
+      <c r="B24" s="188" t="n">
+        <v>30</v>
+      </c>
+      <c r="C24" s="178" t="inlineStr">
+        <is>
+          <t>2ª peça + frete 1x/pedido + CAC diluído ⏳</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" s="63">
+      <c r="A26" s="192" t="inlineStr">
+        <is>
+          <t>3 · Vender na 2ª compra — CAC ZERO (dono da base)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="149" t="inlineStr">
+        <is>
+          <t>R$/mês destravado</t>
+        </is>
+      </c>
+      <c r="B27" s="184">
+        <f>B28*(B30-B29)*B31</f>
+        <v/>
+      </c>
+      <c r="C27" s="185" t="inlineStr">
+        <is>
+          <t>CAC: zero  ·  4–8 sem</t>
+        </is>
+      </c>
+      <c r="D27" s="191" t="inlineStr">
+        <is>
+          <t>⏳ ciclo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="187" t="inlineStr">
+        <is>
+          <t>Base de clientes (abr–jun)</t>
+        </is>
+      </c>
+      <c r="B28" s="170" t="n">
+        <v>19513</v>
+      </c>
+      <c r="C28" s="178" t="inlineStr">
+        <is>
+          <t>Orders API ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="187" t="inlineStr">
+        <is>
+          <t>Taxa de recompra HOJE</t>
+        </is>
+      </c>
+      <c r="B29" s="189" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="C29" s="178" t="inlineStr">
+        <is>
+          <t>piso medido ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="187" t="inlineStr">
+        <is>
+          <t>Meta de recompra</t>
+        </is>
+      </c>
+      <c r="B30" s="189" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="C30" s="178" t="inlineStr">
+        <is>
+          <t>+3pp editável</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="187" t="inlineStr">
+        <is>
+          <t>Contribuição por pedido de recompra (sem CAC)</t>
+        </is>
+      </c>
+      <c r="B31" s="188" t="n">
+        <v>25</v>
+      </c>
+      <c r="C31" s="178" t="inlineStr">
+        <is>
+          <t>aprox contrib s/ mídia ⏳</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" s="63">
+      <c r="A33" s="193" t="inlineStr">
+        <is>
+          <t>4 · Reabastecer a mídia lucrativa (só nos SKUs certos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="149" t="inlineStr">
+        <is>
+          <t>R$/mês destravado</t>
+        </is>
+      </c>
+      <c r="B34" s="184">
+        <f>B35*B36*B37-B35</f>
+        <v/>
+      </c>
+      <c r="C34" s="185" t="inlineStr">
+        <is>
+          <t>CAC: alto  ·  imediato</t>
+        </is>
+      </c>
+      <c r="D34" s="191" t="inlineStr">
+        <is>
+          <t>⏳ confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="187" t="inlineStr">
+        <is>
+          <t>Mídia adicional/mês (recompor corte de jul)</t>
+        </is>
+      </c>
+      <c r="B35" s="188" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C35" s="178" t="inlineStr">
+        <is>
+          <t>corte foi -42% ✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="187" t="inlineStr">
+        <is>
+          <t>ROAS (receita/mídia)</t>
+        </is>
+      </c>
+      <c r="B36" s="194" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="C36" s="178" t="inlineStr">
+        <is>
+          <t>confirmar se ROAS ou ROI-lucro</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="187" t="inlineStr">
+        <is>
+          <t>Margem de contribuição s/ GMV</t>
+        </is>
+      </c>
+      <c r="B37" s="189" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="C37" s="178" t="inlineStr">
+        <is>
+          <t>~R$10 em R$90 ⏳</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="169" t="inlineStr">
+        <is>
+          <t>DIAGNÓSTICO — por que promoção não resolve (P&amp;L da peça única, ordem de grandeza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="187" t="inlineStr">
+        <is>
+          <t>Preço realizado (líq. seller_discount)</t>
+        </is>
+      </c>
+      <c r="B41" s="195" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="187" t="inlineStr">
+        <is>
+          <t>− Fee (27,3%)</t>
+        </is>
+      </c>
+      <c r="B42" s="195" t="n">
+        <v>-24.6</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="187" t="inlineStr">
+        <is>
+          <t>− CPV (estimado · custo_unitario NULL)</t>
+        </is>
+      </c>
+      <c r="B43" s="195" t="n">
+        <v>-44.3</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="187" t="inlineStr">
+        <is>
+          <t>− Frete grátis absorvido</t>
+        </is>
+      </c>
+      <c r="B44" s="195" t="n">
+        <v>-11.8</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="175">
+        <f> Contribuição SEM mídia</f>
+        <v/>
+      </c>
+      <c r="B45" s="196" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="187" t="inlineStr">
+        <is>
+          <t>− CAC / mídia (R$23/pedido)</t>
+        </is>
+      </c>
+      <c r="B46" s="195" t="n">
+        <v>-23</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="197">
+        <f> Contribuição peça única COM mídia</f>
+        <v/>
+      </c>
+      <c r="B47" s="198" t="n">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1" s="63">
+      <c r="A48" s="199" t="inlineStr">
+        <is>
+          <t>Leitura: uma peça sozinha com mídia dá −R$14. Por isso todo desconto te empurra pro vermelho. O combo (L2) faz o pedido virar 2 peças com 1 frete e 1 CAC → positivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A48:D49"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A12:F13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -12982,7 +14182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14541,473 +15741,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="10" customWidth="1" style="62" min="1" max="1"/>
-    <col width="22" customWidth="1" style="62" min="2" max="2"/>
-    <col width="5" customWidth="1" style="62" min="3" max="3"/>
-    <col width="12" customWidth="1" style="62" min="4" max="4"/>
-    <col width="8" customWidth="1" style="62" min="5" max="5"/>
-    <col width="10" customWidth="1" style="62" min="6" max="7"/>
-    <col width="11" customWidth="1" style="62" min="8" max="8"/>
-    <col width="12" customWidth="1" style="62" min="9" max="9"/>
-    <col width="9" customWidth="1" style="62" min="10" max="10"/>
-    <col width="11" customWidth="1" style="62" min="11" max="11"/>
-    <col width="13" customWidth="1" style="62" min="12" max="12"/>
-    <col width="12" customWidth="1" style="62" min="13" max="13"/>
-    <col width="13" customWidth="1" style="62" min="14" max="15"/>
-    <col width="11" customWidth="1" style="62" min="16" max="16"/>
-    <col width="12" customWidth="1" style="62" min="17" max="18"/>
-    <col width="14" customWidth="1" style="62" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="63">
-      <c r="A1" s="64" t="inlineStr">
-        <is>
-          <t>Card afiliada — meta por SKU e pace diário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="63">
-      <c r="A2" s="66" t="inlineStr">
-        <is>
-          <t>Canal (chave):</t>
-        </is>
-      </c>
-      <c r="B2" s="89" t="inlineStr">
-        <is>
-          <t>Card afiliada</t>
-        </is>
-      </c>
-      <c r="C2" s="66" t="inlineStr">
-        <is>
-          <t>Superfície:</t>
-        </is>
-      </c>
-      <c r="D2" s="89" t="inlineStr">
-        <is>
-          <t>CARD DE PRODUTO</t>
-        </is>
-      </c>
-      <c r="F2" s="66" t="inlineStr">
-        <is>
-          <t>Atribuição:</t>
-        </is>
-      </c>
-      <c r="G2" s="89" t="inlineStr">
-        <is>
-          <t>Afiliada</t>
-        </is>
-      </c>
-      <c r="I2" s="66" t="inlineStr">
-        <is>
-          <t>Confiança da base jul:</t>
-        </is>
-      </c>
-      <c r="K2" s="121" t="inlineStr">
-        <is>
-          <t>EXATO — afiliada showcase/card (SHOP+LINKSHARE) do extrato. ~1,5% do GMV.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="63">
-      <c r="A3" s="66" t="inlineStr">
-        <is>
-          <t>Alavanca principal:</t>
-        </is>
-      </c>
-      <c r="B3" s="89" t="inlineStr">
-        <is>
-          <t>A definir — depende de abrir a fonte no extrato de afiliada</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="63">
-      <c r="A4" s="66" t="inlineStr">
-        <is>
-          <t>Crescimento vs base:</t>
-        </is>
-      </c>
-      <c r="B4" s="107">
-        <f>Premissas!$C$27</f>
-        <v/>
-      </c>
-      <c r="C4" s="66" t="inlineStr">
-        <is>
-          <t>Comissão afiliada:</t>
-        </is>
-      </c>
-      <c r="D4" s="107">
-        <f>Premissas!$D$27</f>
-        <v/>
-      </c>
-      <c r="F4" s="66" t="inlineStr">
-        <is>
-          <t>CPV padrão:</t>
-        </is>
-      </c>
-      <c r="G4" s="108">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="63">
-      <c r="A5" s="66" t="inlineStr">
-        <is>
-          <t>Meta do canal (pç):</t>
-        </is>
-      </c>
-      <c r="B5" s="109">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="C5" s="66" t="inlineStr">
-        <is>
-          <t>Meta GMV:</t>
-        </is>
-      </c>
-      <c r="D5" s="110">
-        <f>I9</f>
-        <v/>
-      </c>
-      <c r="F5" s="66" t="inlineStr">
-        <is>
-          <t>Contribuição meta:</t>
-        </is>
-      </c>
-      <c r="G5" s="110">
-        <f>L9</f>
-        <v/>
-      </c>
-      <c r="I5" s="66" t="inlineStr">
-        <is>
-          <t>Índice de pace:</t>
-        </is>
-      </c>
-      <c r="K5" s="111">
-        <f>P9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="63">
-      <c r="A7" s="72" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B7" s="72" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="C7" s="72" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="D7" s="72" t="inlineStr">
-        <is>
-          <t>Base jul (pç)</t>
-        </is>
-      </c>
-      <c r="E7" s="72" t="inlineStr">
-        <is>
-          <t>Mix jul</t>
-        </is>
-      </c>
-      <c r="F7" s="72" t="inlineStr">
-        <is>
-          <t>Ajuste (pç)</t>
-        </is>
-      </c>
-      <c r="G7" s="72" t="inlineStr">
-        <is>
-          <t>Meta (pç)</t>
-        </is>
-      </c>
-      <c r="H7" s="72" t="inlineStr">
-        <is>
-          <t>Preço plan.</t>
-        </is>
-      </c>
-      <c r="I7" s="72" t="inlineStr">
-        <is>
-          <t>Meta GMV</t>
-        </is>
-      </c>
-      <c r="J7" s="72" t="inlineStr">
-        <is>
-          <t>CPV</t>
-        </is>
-      </c>
-      <c r="K7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib./pç</t>
-        </is>
-      </c>
-      <c r="L7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib. meta</t>
-        </is>
-      </c>
-      <c r="M7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (pç)</t>
-        </is>
-      </c>
-      <c r="N7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (R$)</t>
-        </is>
-      </c>
-      <c r="O7" s="72" t="inlineStr">
-        <is>
-          <t>Esperado MTD</t>
-        </is>
-      </c>
-      <c r="P7" s="72" t="inlineStr">
-        <is>
-          <t>Índice pace</t>
-        </is>
-      </c>
-      <c r="Q7" s="72" t="inlineStr">
-        <is>
-          <t>Projeção fim</t>
-        </is>
-      </c>
-      <c r="R7" s="72" t="inlineStr">
-        <is>
-          <t>Gap vs meta</t>
-        </is>
-      </c>
-      <c r="S7" s="72" t="inlineStr">
-        <is>
-          <t>Pç/dia p/ fechar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="63">
-      <c r="A8" s="73" t="inlineStr">
-        <is>
-          <t>AGREGADO</t>
-        </is>
-      </c>
-      <c r="B8" s="74" t="inlineStr">
-        <is>
-          <t>Afiliada showcase/card (SHOP+LINKSHARE)</t>
-        </is>
-      </c>
-      <c r="C8" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D8" s="112" t="n">
-        <v>75</v>
-      </c>
-      <c r="E8" s="113">
-        <f>IFERROR(D8/$D$9,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="112">
-        <f>ROUND(D8*(1+$B$4),0)+F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="97" t="n">
-        <v>94.98</v>
-      </c>
-      <c r="I8" s="114">
-        <f>G8*H8</f>
-        <v/>
-      </c>
-      <c r="J8" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K8" s="116">
-        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="114">
-        <f>G8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="112">
-        <f>G8*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P8" s="117">
-        <f>IFERROR(M8/O8,0)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="112">
-        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R8" s="112">
-        <f>Q8-G8</f>
-        <v/>
-      </c>
-      <c r="S8" s="118">
-        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="63">
-      <c r="A9" s="81" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B9" s="81" t="n"/>
-      <c r="C9" s="81" t="n"/>
-      <c r="D9" s="82">
-        <f>SUM(D8:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="85">
-        <f>SUM(E8:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="82">
-        <f>SUM(F8:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="82">
-        <f>SUM(G8:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="119" t="n"/>
-      <c r="I9" s="83">
-        <f>SUM(I8:I8)</f>
-        <v/>
-      </c>
-      <c r="J9" s="119" t="n"/>
-      <c r="K9" s="119" t="n"/>
-      <c r="L9" s="83">
-        <f>SUM(L8:L8)</f>
-        <v/>
-      </c>
-      <c r="M9" s="82">
-        <f>SUM(M8:M8)</f>
-        <v/>
-      </c>
-      <c r="N9" s="83">
-        <f>SUM(N8:N8)</f>
-        <v/>
-      </c>
-      <c r="O9" s="82">
-        <f>SUM(O8:O8)</f>
-        <v/>
-      </c>
-      <c r="P9" s="84">
-        <f>IFERROR(M9/O9,0)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="82">
-        <f>SUM(Q8:Q8)</f>
-        <v/>
-      </c>
-      <c r="R9" s="82">
-        <f>SUM(R8:R8)</f>
-        <v/>
-      </c>
-      <c r="S9" s="120">
-        <f>SUM(S8:S8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="63">
-      <c r="A10" s="73" t="inlineStr">
-        <is>
-          <t>Σ Hero</t>
-        </is>
-      </c>
-      <c r="B10" s="74" t="n"/>
-      <c r="C10" s="74" t="n"/>
-      <c r="D10" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="E10" s="74" t="n"/>
-      <c r="F10" s="74" t="n"/>
-      <c r="G10" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="H10" s="74" t="n"/>
-      <c r="I10" s="74" t="n"/>
-      <c r="J10" s="74" t="n"/>
-      <c r="K10" s="74" t="n"/>
-      <c r="L10" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="63">
-      <c r="A11" s="73" t="inlineStr">
-        <is>
-          <t>Σ Esteira</t>
-        </is>
-      </c>
-      <c r="B11" s="74" t="n"/>
-      <c r="C11" s="74" t="n"/>
-      <c r="D11" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="E11" s="74" t="n"/>
-      <c r="F11" s="74" t="n"/>
-      <c r="G11" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="H11" s="74" t="n"/>
-      <c r="I11" s="74" t="n"/>
-      <c r="J11" s="74" t="n"/>
-      <c r="K11" s="74" t="n"/>
-      <c r="L11" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="63">
-      <c r="A13" s="71" t="inlineStr">
-        <is>
-          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="63">
-      <c r="A14" s="71" t="inlineStr">
-        <is>
-          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sim): aba Simulador Corrida — corrida de vídeos + GMV Max, 1ª e 2ª ordem, CPV real e co-financiamento TT (dado statement_tx)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
+++ b/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
@@ -14,15 +14,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Premissas" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alavancas" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alavancas de Margem" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live afiliada" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo afiliada" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card afiliada" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live loja" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo loja" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card loja" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitrine loja" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busca e Mall" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log diário" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulador Corrida" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live afiliada" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo afiliada" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card afiliada" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live loja" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo loja" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card loja" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitrine loja" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busca e Mall" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log diário" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -31,7 +32,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.00\x"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -43,8 +44,9 @@
     <numFmt numFmtId="172" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="173" formatCode="0.0"/>
     <numFmt numFmtId="174" formatCode="&quot;R$&quot; #,##0"/>
+    <numFmt numFmtId="175" formatCode="&quot;R$&quot; #,##0.00"/>
   </numFmts>
-  <fonts count="43">
+  <fonts count="46">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -306,8 +308,26 @@
       <color rgb="001A1A1A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E7E34"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -387,6 +407,11 @@
         <fgColor rgb="007A7A7A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000000FF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -436,7 +461,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="200">
+  <cellXfs count="209">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -996,6 +1021,33 @@
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="175" fontId="34" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="32" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="43" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="32" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="44" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="174" fontId="45" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1078,6 +1130,21 @@
     <comment ref="B35" authorId="0" shapeId="0">
       <text>
         <t>Se 7,8 for ROI de LUCRO (nao ROAS), esta alavanca dispara pra 6 digitos e vira a #1. Preciso puxar o dado real de contribuicao da midia pra travar. Formula conservadora (ROAS x margem - midia): a 11% de margem ela mal se paga.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>DADO REAL jun-ago: TikTok banca ~3,5% do gross (platform_discount); Rhode banca 47% (seller_discount). Proporcao ~13:1. So sobe entrando em campanha/voucher TT (jun bateu 5,4%). Default 0% = premissa honesta de que o cupom novo e seu.</t>
       </text>
     </comment>
   </commentList>
@@ -1925,6 +1992,1567 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:S28"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="10" customWidth="1" style="62" min="1" max="1"/>
+    <col width="22" customWidth="1" style="62" min="2" max="2"/>
+    <col width="5" customWidth="1" style="62" min="3" max="3"/>
+    <col width="12" customWidth="1" style="62" min="4" max="4"/>
+    <col width="8" customWidth="1" style="62" min="5" max="5"/>
+    <col width="10" customWidth="1" style="62" min="6" max="7"/>
+    <col width="11" customWidth="1" style="62" min="8" max="8"/>
+    <col width="12" customWidth="1" style="62" min="9" max="9"/>
+    <col width="9" customWidth="1" style="62" min="10" max="10"/>
+    <col width="11" customWidth="1" style="62" min="11" max="11"/>
+    <col width="13" customWidth="1" style="62" min="12" max="12"/>
+    <col width="12" customWidth="1" style="62" min="13" max="13"/>
+    <col width="13" customWidth="1" style="62" min="14" max="15"/>
+    <col width="11" customWidth="1" style="62" min="16" max="16"/>
+    <col width="12" customWidth="1" style="62" min="17" max="18"/>
+    <col width="14" customWidth="1" style="62" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.15" customHeight="1" s="63">
+      <c r="A1" s="64" t="inlineStr">
+        <is>
+          <t>Vídeo afiliada — meta por SKU e pace diário</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="63">
+      <c r="A2" s="66" t="inlineStr">
+        <is>
+          <t>Canal (chave):</t>
+        </is>
+      </c>
+      <c r="B2" s="89" t="inlineStr">
+        <is>
+          <t>Vídeo afiliada</t>
+        </is>
+      </c>
+      <c r="C2" s="66" t="inlineStr">
+        <is>
+          <t>Superfície:</t>
+        </is>
+      </c>
+      <c r="D2" s="89" t="inlineStr">
+        <is>
+          <t>VÍDEO</t>
+        </is>
+      </c>
+      <c r="F2" s="66" t="inlineStr">
+        <is>
+          <t>Atribuição:</t>
+        </is>
+      </c>
+      <c r="G2" s="89" t="inlineStr">
+        <is>
+          <t>Afiliada</t>
+        </is>
+      </c>
+      <c r="I2" s="66" t="inlineStr">
+        <is>
+          <t>Confiança da base jul:</t>
+        </is>
+      </c>
+      <c r="K2" s="89" t="inlineStr">
+        <is>
+          <t>EXATO — extrato de afiliada</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="63">
+      <c r="A3" s="66" t="inlineStr">
+        <is>
+          <t>Alavanca principal:</t>
+        </is>
+      </c>
+      <c r="B3" s="89" t="inlineStr">
+        <is>
+          <t>Copa Rhode Creators (gamificação) + Academia + desova de seeding</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="63">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>Crescimento vs base:</t>
+        </is>
+      </c>
+      <c r="B4" s="107">
+        <f>Premissas!$C$26</f>
+        <v/>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Comissão afiliada:</t>
+        </is>
+      </c>
+      <c r="D4" s="107">
+        <f>Premissas!$D$26</f>
+        <v/>
+      </c>
+      <c r="F4" s="66" t="inlineStr">
+        <is>
+          <t>CPV padrão:</t>
+        </is>
+      </c>
+      <c r="G4" s="108">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="63">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>Meta do canal (pç):</t>
+        </is>
+      </c>
+      <c r="B5" s="109">
+        <f>G23</f>
+        <v/>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>Meta GMV:</t>
+        </is>
+      </c>
+      <c r="D5" s="110">
+        <f>I23</f>
+        <v/>
+      </c>
+      <c r="F5" s="66" t="inlineStr">
+        <is>
+          <t>Contribuição meta:</t>
+        </is>
+      </c>
+      <c r="G5" s="110">
+        <f>L23</f>
+        <v/>
+      </c>
+      <c r="I5" s="66" t="inlineStr">
+        <is>
+          <t>Índice de pace:</t>
+        </is>
+      </c>
+      <c r="K5" s="111">
+        <f>P23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="63">
+      <c r="A7" s="72" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B7" s="72" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>Base jul (pç)</t>
+        </is>
+      </c>
+      <c r="E7" s="72" t="inlineStr">
+        <is>
+          <t>Mix jul</t>
+        </is>
+      </c>
+      <c r="F7" s="72" t="inlineStr">
+        <is>
+          <t>Ajuste (pç)</t>
+        </is>
+      </c>
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>Meta (pç)</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="inlineStr">
+        <is>
+          <t>Preço plan.</t>
+        </is>
+      </c>
+      <c r="I7" s="72" t="inlineStr">
+        <is>
+          <t>Meta GMV</t>
+        </is>
+      </c>
+      <c r="J7" s="72" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="K7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib./pç</t>
+        </is>
+      </c>
+      <c r="L7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib. meta</t>
+        </is>
+      </c>
+      <c r="M7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (pç)</t>
+        </is>
+      </c>
+      <c r="N7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (R$)</t>
+        </is>
+      </c>
+      <c r="O7" s="72" t="inlineStr">
+        <is>
+          <t>Esperado MTD</t>
+        </is>
+      </c>
+      <c r="P7" s="72" t="inlineStr">
+        <is>
+          <t>Índice pace</t>
+        </is>
+      </c>
+      <c r="Q7" s="72" t="inlineStr">
+        <is>
+          <t>Projeção fim</t>
+        </is>
+      </c>
+      <c r="R7" s="72" t="inlineStr">
+        <is>
+          <t>Gap vs meta</t>
+        </is>
+      </c>
+      <c r="S7" s="72" t="inlineStr">
+        <is>
+          <t>Pç/dia p/ fechar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="63">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>REF516</t>
+        </is>
+      </c>
+      <c r="B8" s="74" t="inlineStr">
+        <is>
+          <t>Marmorizada</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D8" s="112" t="n">
+        <v>715</v>
+      </c>
+      <c r="E8" s="113">
+        <f>IFERROR(D8/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="112">
+        <f>ROUND(D8*(1+$B$4),0)+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="97" t="n">
+        <v>93</v>
+      </c>
+      <c r="I8" s="114">
+        <f>G8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K8" s="116">
+        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="114">
+        <f>G8*K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="112">
+        <f>G8*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P8" s="117">
+        <f>IFERROR(M8/O8,0)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="112">
+        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R8" s="112">
+        <f>Q8-G8</f>
+        <v/>
+      </c>
+      <c r="S8" s="118">
+        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="63">
+      <c r="A9" s="73" t="inlineStr">
+        <is>
+          <t>REF527</t>
+        </is>
+      </c>
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>Sky Used</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D9" s="112" t="n">
+        <v>183</v>
+      </c>
+      <c r="E9" s="113">
+        <f>IFERROR(D9/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="112">
+        <f>ROUND(D9*(1+$B$4),0)+F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="97" t="n">
+        <v>93.73999999999999</v>
+      </c>
+      <c r="I9" s="114">
+        <f>G9*H9</f>
+        <v/>
+      </c>
+      <c r="J9" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K9" s="116">
+        <f>H9*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J9</f>
+        <v/>
+      </c>
+      <c r="L9" s="114">
+        <f>G9*K9</f>
+        <v/>
+      </c>
+      <c r="M9" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A9)</f>
+        <v/>
+      </c>
+      <c r="O9" s="112">
+        <f>G9*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P9" s="117">
+        <f>IFERROR(M9/O9,0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="112">
+        <f>IFERROR(M9/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R9" s="112">
+        <f>Q9-G9</f>
+        <v/>
+      </c>
+      <c r="S9" s="118">
+        <f>IFERROR(MAX(0,G9-M9)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="63">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>REF525</t>
+        </is>
+      </c>
+      <c r="B10" s="74" t="inlineStr">
+        <is>
+          <t>Stone Used</t>
+        </is>
+      </c>
+      <c r="C10" s="74" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D10" s="112" t="n">
+        <v>139</v>
+      </c>
+      <c r="E10" s="113">
+        <f>IFERROR(D10/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="112">
+        <f>ROUND(D10*(1+$B$4),0)+F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="97" t="n">
+        <v>98.27</v>
+      </c>
+      <c r="I10" s="114">
+        <f>G10*H10</f>
+        <v/>
+      </c>
+      <c r="J10" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K10" s="116">
+        <f>H10*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J10</f>
+        <v/>
+      </c>
+      <c r="L10" s="114">
+        <f>G10*K10</f>
+        <v/>
+      </c>
+      <c r="M10" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A10)</f>
+        <v/>
+      </c>
+      <c r="O10" s="112">
+        <f>G10*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P10" s="117">
+        <f>IFERROR(M10/O10,0)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="112">
+        <f>IFERROR(M10/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R10" s="112">
+        <f>Q10-G10</f>
+        <v/>
+      </c>
+      <c r="S10" s="118">
+        <f>IFERROR(MAX(0,G10-M10)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="63">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>REF588</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>Mom Marmorizada</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D11" s="112" t="n">
+        <v>127</v>
+      </c>
+      <c r="E11" s="113">
+        <f>IFERROR(D11/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="112">
+        <f>ROUND(D11*(1+$B$4),0)+F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="97" t="n">
+        <v>95.76000000000001</v>
+      </c>
+      <c r="I11" s="114">
+        <f>G11*H11</f>
+        <v/>
+      </c>
+      <c r="J11" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K11" s="116">
+        <f>H11*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J11</f>
+        <v/>
+      </c>
+      <c r="L11" s="114">
+        <f>G11*K11</f>
+        <v/>
+      </c>
+      <c r="M11" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A11)</f>
+        <v/>
+      </c>
+      <c r="O11" s="112">
+        <f>G11*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P11" s="117">
+        <f>IFERROR(M11/O11,0)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="112">
+        <f>IFERROR(M11/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R11" s="112">
+        <f>Q11-G11</f>
+        <v/>
+      </c>
+      <c r="S11" s="118">
+        <f>IFERROR(MAX(0,G11-M11)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="63">
+      <c r="A12" s="73" t="inlineStr">
+        <is>
+          <t>REF587</t>
+        </is>
+      </c>
+      <c r="B12" s="74" t="inlineStr">
+        <is>
+          <t>Baggy Marmorizada</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D12" s="112" t="n">
+        <v>83</v>
+      </c>
+      <c r="E12" s="113">
+        <f>IFERROR(D12/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="112">
+        <f>ROUND(D12*(1+$B$4),0)+F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="97" t="n">
+        <v>98.44</v>
+      </c>
+      <c r="I12" s="114">
+        <f>G12*H12</f>
+        <v/>
+      </c>
+      <c r="J12" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K12" s="116">
+        <f>H12*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J12</f>
+        <v/>
+      </c>
+      <c r="L12" s="114">
+        <f>G12*K12</f>
+        <v/>
+      </c>
+      <c r="M12" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="112">
+        <f>G12*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P12" s="117">
+        <f>IFERROR(M12/O12,0)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="112">
+        <f>IFERROR(M12/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R12" s="112">
+        <f>Q12-G12</f>
+        <v/>
+      </c>
+      <c r="S12" s="118">
+        <f>IFERROR(MAX(0,G12-M12)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="63">
+      <c r="A13" s="73" t="inlineStr">
+        <is>
+          <t>REF549</t>
+        </is>
+      </c>
+      <c r="B13" s="74" t="inlineStr">
+        <is>
+          <t>Rosa Bebê</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D13" s="112" t="n">
+        <v>45</v>
+      </c>
+      <c r="E13" s="113">
+        <f>IFERROR(D13/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="112">
+        <f>ROUND(D13*(1+$B$4),0)+F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="97" t="n">
+        <v>97.23</v>
+      </c>
+      <c r="I13" s="114">
+        <f>G13*H13</f>
+        <v/>
+      </c>
+      <c r="J13" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K13" s="116">
+        <f>H13*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J13</f>
+        <v/>
+      </c>
+      <c r="L13" s="114">
+        <f>G13*K13</f>
+        <v/>
+      </c>
+      <c r="M13" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="112">
+        <f>G13*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P13" s="117">
+        <f>IFERROR(M13/O13,0)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="112">
+        <f>IFERROR(M13/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R13" s="112">
+        <f>Q13-G13</f>
+        <v/>
+      </c>
+      <c r="S13" s="118">
+        <f>IFERROR(MAX(0,G13-M13)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="63">
+      <c r="A14" s="73" t="inlineStr">
+        <is>
+          <t>REF559</t>
+        </is>
+      </c>
+      <c r="B14" s="74" t="inlineStr">
+        <is>
+          <t>Mom Rosa</t>
+        </is>
+      </c>
+      <c r="C14" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D14" s="112" t="n">
+        <v>26</v>
+      </c>
+      <c r="E14" s="113">
+        <f>IFERROR(D14/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="112">
+        <f>ROUND(D14*(1+$B$4),0)+F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="97" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="I14" s="114">
+        <f>G14*H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K14" s="116">
+        <f>H14*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J14</f>
+        <v/>
+      </c>
+      <c r="L14" s="114">
+        <f>G14*K14</f>
+        <v/>
+      </c>
+      <c r="M14" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="112">
+        <f>G14*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P14" s="117">
+        <f>IFERROR(M14/O14,0)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="112">
+        <f>IFERROR(M14/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R14" s="112">
+        <f>Q14-G14</f>
+        <v/>
+      </c>
+      <c r="S14" s="118">
+        <f>IFERROR(MAX(0,G14-M14)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="63">
+      <c r="A15" s="73" t="inlineStr">
+        <is>
+          <t>REF566</t>
+        </is>
+      </c>
+      <c r="B15" s="74" t="inlineStr">
+        <is>
+          <t>Mom Choco</t>
+        </is>
+      </c>
+      <c r="C15" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D15" s="112" t="n">
+        <v>21</v>
+      </c>
+      <c r="E15" s="113">
+        <f>IFERROR(D15/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="112">
+        <f>ROUND(D15*(1+$B$4),0)+F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="97" t="n">
+        <v>95.68000000000001</v>
+      </c>
+      <c r="I15" s="114">
+        <f>G15*H15</f>
+        <v/>
+      </c>
+      <c r="J15" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K15" s="116">
+        <f>H15*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J15</f>
+        <v/>
+      </c>
+      <c r="L15" s="114">
+        <f>G15*K15</f>
+        <v/>
+      </c>
+      <c r="M15" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="112">
+        <f>G15*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P15" s="117">
+        <f>IFERROR(M15/O15,0)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="112">
+        <f>IFERROR(M15/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R15" s="112">
+        <f>Q15-G15</f>
+        <v/>
+      </c>
+      <c r="S15" s="118">
+        <f>IFERROR(MAX(0,G15-M15)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="63">
+      <c r="A16" s="73" t="inlineStr">
+        <is>
+          <t>REF558</t>
+        </is>
+      </c>
+      <c r="B16" s="74" t="inlineStr">
+        <is>
+          <t>(sem de-para)</t>
+        </is>
+      </c>
+      <c r="C16" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D16" s="112" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" s="113">
+        <f>IFERROR(D16/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="112">
+        <f>ROUND(D16*(1+$B$4),0)+F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="97" t="n">
+        <v>75.98999999999999</v>
+      </c>
+      <c r="I16" s="114">
+        <f>G16*H16</f>
+        <v/>
+      </c>
+      <c r="J16" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K16" s="116">
+        <f>H16*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J16</f>
+        <v/>
+      </c>
+      <c r="L16" s="114">
+        <f>G16*K16</f>
+        <v/>
+      </c>
+      <c r="M16" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="112">
+        <f>G16*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P16" s="117">
+        <f>IFERROR(M16/O16,0)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="112">
+        <f>IFERROR(M16/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R16" s="112">
+        <f>Q16-G16</f>
+        <v/>
+      </c>
+      <c r="S16" s="118">
+        <f>IFERROR(MAX(0,G16-M16)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="63">
+      <c r="A17" s="73" t="inlineStr">
+        <is>
+          <t>REF562</t>
+        </is>
+      </c>
+      <c r="B17" s="74" t="inlineStr">
+        <is>
+          <t>Chocolate</t>
+        </is>
+      </c>
+      <c r="C17" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D17" s="112" t="n">
+        <v>20</v>
+      </c>
+      <c r="E17" s="113">
+        <f>IFERROR(D17/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="92" t="n">
+        <v>149</v>
+      </c>
+      <c r="G17" s="112">
+        <f>ROUND(D17*(1+$B$4),0)+F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="97" t="n">
+        <v>101.71</v>
+      </c>
+      <c r="I17" s="114">
+        <f>G17*H17</f>
+        <v/>
+      </c>
+      <c r="J17" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K17" s="116">
+        <f>H17*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J17</f>
+        <v/>
+      </c>
+      <c r="L17" s="114">
+        <f>G17*K17</f>
+        <v/>
+      </c>
+      <c r="M17" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="112">
+        <f>G17*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P17" s="117">
+        <f>IFERROR(M17/O17,0)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="112">
+        <f>IFERROR(M17/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R17" s="112">
+        <f>Q17-G17</f>
+        <v/>
+      </c>
+      <c r="S17" s="118">
+        <f>IFERROR(MAX(0,G17-M17)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="63">
+      <c r="A18" s="73" t="inlineStr">
+        <is>
+          <t>REF550</t>
+        </is>
+      </c>
+      <c r="B18" s="74" t="inlineStr">
+        <is>
+          <t>Amarela</t>
+        </is>
+      </c>
+      <c r="C18" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D18" s="112" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" s="113">
+        <f>IFERROR(D18/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="112">
+        <f>ROUND(D18*(1+$B$4),0)+F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="97" t="n">
+        <v>101.41</v>
+      </c>
+      <c r="I18" s="114">
+        <f>G18*H18</f>
+        <v/>
+      </c>
+      <c r="J18" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K18" s="116">
+        <f>H18*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J18</f>
+        <v/>
+      </c>
+      <c r="L18" s="114">
+        <f>G18*K18</f>
+        <v/>
+      </c>
+      <c r="M18" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="O18" s="112">
+        <f>G18*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P18" s="117">
+        <f>IFERROR(M18/O18,0)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="112">
+        <f>IFERROR(M18/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R18" s="112">
+        <f>Q18-G18</f>
+        <v/>
+      </c>
+      <c r="S18" s="118">
+        <f>IFERROR(MAX(0,G18-M18)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="63">
+      <c r="A19" s="73" t="inlineStr">
+        <is>
+          <t>REF551</t>
+        </is>
+      </c>
+      <c r="B19" s="74" t="inlineStr">
+        <is>
+          <t>Azul Médio</t>
+        </is>
+      </c>
+      <c r="C19" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D19" s="112" t="n">
+        <v>16</v>
+      </c>
+      <c r="E19" s="113">
+        <f>IFERROR(D19/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="112">
+        <f>ROUND(D19*(1+$B$4),0)+F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="97" t="n">
+        <v>101.08</v>
+      </c>
+      <c r="I19" s="114">
+        <f>G19*H19</f>
+        <v/>
+      </c>
+      <c r="J19" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K19" s="116">
+        <f>H19*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J19</f>
+        <v/>
+      </c>
+      <c r="L19" s="114">
+        <f>G19*K19</f>
+        <v/>
+      </c>
+      <c r="M19" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="O19" s="112">
+        <f>G19*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P19" s="117">
+        <f>IFERROR(M19/O19,0)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="112">
+        <f>IFERROR(M19/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R19" s="112">
+        <f>Q19-G19</f>
+        <v/>
+      </c>
+      <c r="S19" s="118">
+        <f>IFERROR(MAX(0,G19-M19)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1" s="63">
+      <c r="A20" s="73" t="inlineStr">
+        <is>
+          <t>REF528</t>
+        </is>
+      </c>
+      <c r="B20" s="74" t="inlineStr">
+        <is>
+          <t>Wide 528</t>
+        </is>
+      </c>
+      <c r="C20" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D20" s="112" t="n">
+        <v>15</v>
+      </c>
+      <c r="E20" s="113">
+        <f>IFERROR(D20/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="112">
+        <f>ROUND(D20*(1+$B$4),0)+F20</f>
+        <v/>
+      </c>
+      <c r="H20" s="97" t="n">
+        <v>83.68000000000001</v>
+      </c>
+      <c r="I20" s="114">
+        <f>G20*H20</f>
+        <v/>
+      </c>
+      <c r="J20" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K20" s="116">
+        <f>H20*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J20</f>
+        <v/>
+      </c>
+      <c r="L20" s="114">
+        <f>G20*K20</f>
+        <v/>
+      </c>
+      <c r="M20" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="O20" s="112">
+        <f>G20*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P20" s="117">
+        <f>IFERROR(M20/O20,0)</f>
+        <v/>
+      </c>
+      <c r="Q20" s="112">
+        <f>IFERROR(M20/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R20" s="112">
+        <f>Q20-G20</f>
+        <v/>
+      </c>
+      <c r="S20" s="118">
+        <f>IFERROR(MAX(0,G20-M20)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1" s="63">
+      <c r="A21" s="73" t="inlineStr">
+        <is>
+          <t>REF546</t>
+        </is>
+      </c>
+      <c r="B21" s="74" t="inlineStr">
+        <is>
+          <t>(sem de-para)</t>
+        </is>
+      </c>
+      <c r="C21" s="74" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="D21" s="112" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" s="113">
+        <f>IFERROR(D21/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F21" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="112">
+        <f>ROUND(D21*(1+$B$4),0)+F21</f>
+        <v/>
+      </c>
+      <c r="H21" s="97" t="n">
+        <v>116.95</v>
+      </c>
+      <c r="I21" s="114">
+        <f>G21*H21</f>
+        <v/>
+      </c>
+      <c r="J21" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K21" s="116">
+        <f>H21*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J21</f>
+        <v/>
+      </c>
+      <c r="L21" s="114">
+        <f>G21*K21</f>
+        <v/>
+      </c>
+      <c r="M21" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="N21" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="O21" s="112">
+        <f>G21*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P21" s="117">
+        <f>IFERROR(M21/O21,0)</f>
+        <v/>
+      </c>
+      <c r="Q21" s="112">
+        <f>IFERROR(M21/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R21" s="112">
+        <f>Q21-G21</f>
+        <v/>
+      </c>
+      <c r="S21" s="118">
+        <f>IFERROR(MAX(0,G21-M21)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1" s="63">
+      <c r="A22" s="73" t="inlineStr">
+        <is>
+          <t>CAUDA</t>
+        </is>
+      </c>
+      <c r="B22" s="74" t="inlineStr">
+        <is>
+          <t>SKUs de cauda não detalhados</t>
+        </is>
+      </c>
+      <c r="C22" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D22" s="112" t="n">
+        <v>39</v>
+      </c>
+      <c r="E22" s="113">
+        <f>IFERROR(D22/$D$23,0)</f>
+        <v/>
+      </c>
+      <c r="F22" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="112">
+        <f>ROUND(D22*(1+$B$4),0)+F22</f>
+        <v/>
+      </c>
+      <c r="H22" s="97" t="n">
+        <v>94.16</v>
+      </c>
+      <c r="I22" s="114">
+        <f>G22*H22</f>
+        <v/>
+      </c>
+      <c r="J22" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K22" s="116">
+        <f>H22*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J22</f>
+        <v/>
+      </c>
+      <c r="L22" s="114">
+        <f>G22*K22</f>
+        <v/>
+      </c>
+      <c r="M22" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="O22" s="112">
+        <f>G22*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P22" s="117">
+        <f>IFERROR(M22/O22,0)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="112">
+        <f>IFERROR(M22/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R22" s="112">
+        <f>Q22-G22</f>
+        <v/>
+      </c>
+      <c r="S22" s="118">
+        <f>IFERROR(MAX(0,G22-M22)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="63">
+      <c r="A23" s="81" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B23" s="81" t="n"/>
+      <c r="C23" s="81" t="n"/>
+      <c r="D23" s="82">
+        <f>SUM(D8:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="85">
+        <f>SUM(E8:E22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="82">
+        <f>SUM(F8:F22)</f>
+        <v/>
+      </c>
+      <c r="G23" s="82">
+        <f>SUM(G8:G22)</f>
+        <v/>
+      </c>
+      <c r="H23" s="119" t="n"/>
+      <c r="I23" s="83">
+        <f>SUM(I8:I22)</f>
+        <v/>
+      </c>
+      <c r="J23" s="119" t="n"/>
+      <c r="K23" s="119" t="n"/>
+      <c r="L23" s="83">
+        <f>SUM(L8:L22)</f>
+        <v/>
+      </c>
+      <c r="M23" s="82">
+        <f>SUM(M8:M22)</f>
+        <v/>
+      </c>
+      <c r="N23" s="83">
+        <f>SUM(N8:N22)</f>
+        <v/>
+      </c>
+      <c r="O23" s="82">
+        <f>SUM(O8:O22)</f>
+        <v/>
+      </c>
+      <c r="P23" s="84">
+        <f>IFERROR(M23/O23,0)</f>
+        <v/>
+      </c>
+      <c r="Q23" s="82">
+        <f>SUM(Q8:Q22)</f>
+        <v/>
+      </c>
+      <c r="R23" s="82">
+        <f>SUM(R8:R22)</f>
+        <v/>
+      </c>
+      <c r="S23" s="120">
+        <f>SUM(S8:S22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="63">
+      <c r="A24" s="73" t="inlineStr">
+        <is>
+          <t>Σ Hero</t>
+        </is>
+      </c>
+      <c r="B24" s="74" t="n"/>
+      <c r="C24" s="74" t="n"/>
+      <c r="D24" s="112">
+        <f>SUMIFS(D8:D22,$C$8:$C$22,"H")</f>
+        <v/>
+      </c>
+      <c r="E24" s="74" t="n"/>
+      <c r="F24" s="74" t="n"/>
+      <c r="G24" s="112">
+        <f>SUMIFS(G8:G22,$C$8:$C$22,"H")</f>
+        <v/>
+      </c>
+      <c r="H24" s="74" t="n"/>
+      <c r="I24" s="74" t="n"/>
+      <c r="J24" s="74" t="n"/>
+      <c r="K24" s="74" t="n"/>
+      <c r="L24" s="114">
+        <f>SUMIFS(L8:L22,$C$8:$C$22,"H")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="63">
+      <c r="A25" s="73" t="inlineStr">
+        <is>
+          <t>Σ Esteira</t>
+        </is>
+      </c>
+      <c r="B25" s="74" t="n"/>
+      <c r="C25" s="74" t="n"/>
+      <c r="D25" s="112">
+        <f>SUMIFS(D8:D22,$C$8:$C$22,"E")</f>
+        <v/>
+      </c>
+      <c r="E25" s="74" t="n"/>
+      <c r="F25" s="74" t="n"/>
+      <c r="G25" s="112">
+        <f>SUMIFS(G8:G22,$C$8:$C$22,"E")</f>
+        <v/>
+      </c>
+      <c r="H25" s="74" t="n"/>
+      <c r="I25" s="74" t="n"/>
+      <c r="J25" s="74" t="n"/>
+      <c r="K25" s="74" t="n"/>
+      <c r="L25" s="114">
+        <f>SUMIFS(L8:L22,$C$8:$C$22,"E")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="63">
+      <c r="A27" s="71" t="inlineStr">
+        <is>
+          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="63">
+      <c r="A28" s="71" t="inlineStr">
+        <is>
+          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
@@ -2388,7 +4016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4573,7 +6201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5198,7 +6826,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6201,475 +7829,6 @@
     </row>
     <row r="21" ht="15" customHeight="1" s="63">
       <c r="A21" s="71" t="inlineStr">
-        <is>
-          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="10" customWidth="1" style="62" min="1" max="1"/>
-    <col width="22" customWidth="1" style="62" min="2" max="2"/>
-    <col width="5" customWidth="1" style="62" min="3" max="3"/>
-    <col width="12" customWidth="1" style="62" min="4" max="4"/>
-    <col width="8" customWidth="1" style="62" min="5" max="5"/>
-    <col width="10" customWidth="1" style="62" min="6" max="7"/>
-    <col width="11" customWidth="1" style="62" min="8" max="8"/>
-    <col width="12" customWidth="1" style="62" min="9" max="9"/>
-    <col width="9" customWidth="1" style="62" min="10" max="10"/>
-    <col width="11" customWidth="1" style="62" min="11" max="11"/>
-    <col width="13" customWidth="1" style="62" min="12" max="12"/>
-    <col width="12" customWidth="1" style="62" min="13" max="13"/>
-    <col width="13" customWidth="1" style="62" min="14" max="15"/>
-    <col width="11" customWidth="1" style="62" min="16" max="16"/>
-    <col width="12" customWidth="1" style="62" min="17" max="18"/>
-    <col width="14" customWidth="1" style="62" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="63">
-      <c r="A1" s="64" t="inlineStr">
-        <is>
-          <t>Vitrine loja — meta por SKU e pace diário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="63">
-      <c r="A2" s="66" t="inlineStr">
-        <is>
-          <t>Canal (chave):</t>
-        </is>
-      </c>
-      <c r="B2" s="89" t="inlineStr">
-        <is>
-          <t>Vitrine loja</t>
-        </is>
-      </c>
-      <c r="C2" s="66" t="inlineStr">
-        <is>
-          <t>Superfície:</t>
-        </is>
-      </c>
-      <c r="D2" s="89" t="inlineStr">
-        <is>
-          <t>VITRINE DA LOJA</t>
-        </is>
-      </c>
-      <c r="F2" s="66" t="inlineStr">
-        <is>
-          <t>Atribuição:</t>
-        </is>
-      </c>
-      <c r="G2" s="89" t="inlineStr">
-        <is>
-          <t>Loja / vendedor</t>
-        </is>
-      </c>
-      <c r="I2" s="66" t="inlineStr">
-        <is>
-          <t>Confiança da base jul:</t>
-        </is>
-      </c>
-      <c r="K2" s="121" t="inlineStr">
-        <is>
-          <t>TRANSVERSAL — shop_tab R$89.369 (jul, API 202605) SOBREPÕE card/loja; não somável no NET (lente de superfície, não de último-conteúdo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="63">
-      <c r="A3" s="66" t="inlineStr">
-        <is>
-          <t>Alavanca principal:</t>
-        </is>
-      </c>
-      <c r="B3" s="89" t="inlineStr">
-        <is>
-          <t>A definir — organizar vitrine por curva e coleção</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="63">
-      <c r="A4" s="66" t="inlineStr">
-        <is>
-          <t>Crescimento vs base:</t>
-        </is>
-      </c>
-      <c r="B4" s="107">
-        <f>Premissas!$C$31</f>
-        <v/>
-      </c>
-      <c r="C4" s="66" t="inlineStr">
-        <is>
-          <t>Comissão afiliada:</t>
-        </is>
-      </c>
-      <c r="D4" s="107">
-        <f>Premissas!$D$31</f>
-        <v/>
-      </c>
-      <c r="F4" s="66" t="inlineStr">
-        <is>
-          <t>CPV padrão:</t>
-        </is>
-      </c>
-      <c r="G4" s="108">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="63">
-      <c r="A5" s="66" t="inlineStr">
-        <is>
-          <t>Meta do canal (pç):</t>
-        </is>
-      </c>
-      <c r="B5" s="109">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="C5" s="66" t="inlineStr">
-        <is>
-          <t>Meta GMV:</t>
-        </is>
-      </c>
-      <c r="D5" s="110">
-        <f>I9</f>
-        <v/>
-      </c>
-      <c r="F5" s="66" t="inlineStr">
-        <is>
-          <t>Contribuição meta:</t>
-        </is>
-      </c>
-      <c r="G5" s="110">
-        <f>L9</f>
-        <v/>
-      </c>
-      <c r="I5" s="66" t="inlineStr">
-        <is>
-          <t>Índice de pace:</t>
-        </is>
-      </c>
-      <c r="K5" s="111">
-        <f>P9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="63">
-      <c r="A7" s="72" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B7" s="72" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="C7" s="72" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="D7" s="72" t="inlineStr">
-        <is>
-          <t>Base jul (pç)</t>
-        </is>
-      </c>
-      <c r="E7" s="72" t="inlineStr">
-        <is>
-          <t>Mix jul</t>
-        </is>
-      </c>
-      <c r="F7" s="72" t="inlineStr">
-        <is>
-          <t>Ajuste (pç)</t>
-        </is>
-      </c>
-      <c r="G7" s="72" t="inlineStr">
-        <is>
-          <t>Meta (pç)</t>
-        </is>
-      </c>
-      <c r="H7" s="72" t="inlineStr">
-        <is>
-          <t>Preço plan.</t>
-        </is>
-      </c>
-      <c r="I7" s="72" t="inlineStr">
-        <is>
-          <t>Meta GMV</t>
-        </is>
-      </c>
-      <c r="J7" s="72" t="inlineStr">
-        <is>
-          <t>CPV</t>
-        </is>
-      </c>
-      <c r="K7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib./pç</t>
-        </is>
-      </c>
-      <c r="L7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib. meta</t>
-        </is>
-      </c>
-      <c r="M7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (pç)</t>
-        </is>
-      </c>
-      <c r="N7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (R$)</t>
-        </is>
-      </c>
-      <c r="O7" s="72" t="inlineStr">
-        <is>
-          <t>Esperado MTD</t>
-        </is>
-      </c>
-      <c r="P7" s="72" t="inlineStr">
-        <is>
-          <t>Índice pace</t>
-        </is>
-      </c>
-      <c r="Q7" s="72" t="inlineStr">
-        <is>
-          <t>Projeção fim</t>
-        </is>
-      </c>
-      <c r="R7" s="72" t="inlineStr">
-        <is>
-          <t>Gap vs meta</t>
-        </is>
-      </c>
-      <c r="S7" s="72" t="inlineStr">
-        <is>
-          <t>Pç/dia p/ fechar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="63">
-      <c r="A8" s="73" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B8" s="74" t="inlineStr">
-        <is>
-          <t>Sem base de julho para este canal</t>
-        </is>
-      </c>
-      <c r="C8" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="113">
-        <f>IFERROR(D8/$D$9,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="112">
-        <f>ROUND(D8*(1+$B$4),0)+F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="97" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="114">
-        <f>G8*H8</f>
-        <v/>
-      </c>
-      <c r="J8" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K8" s="116">
-        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="114">
-        <f>G8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="112">
-        <f>G8*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P8" s="117">
-        <f>IFERROR(M8/O8,0)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="112">
-        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R8" s="112">
-        <f>Q8-G8</f>
-        <v/>
-      </c>
-      <c r="S8" s="118">
-        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="63">
-      <c r="A9" s="81" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B9" s="81" t="n"/>
-      <c r="C9" s="81" t="n"/>
-      <c r="D9" s="82">
-        <f>SUM(D8:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="85">
-        <f>SUM(E8:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="82">
-        <f>SUM(F8:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="82">
-        <f>SUM(G8:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="119" t="n"/>
-      <c r="I9" s="83">
-        <f>SUM(I8:I8)</f>
-        <v/>
-      </c>
-      <c r="J9" s="119" t="n"/>
-      <c r="K9" s="119" t="n"/>
-      <c r="L9" s="83">
-        <f>SUM(L8:L8)</f>
-        <v/>
-      </c>
-      <c r="M9" s="82">
-        <f>SUM(M8:M8)</f>
-        <v/>
-      </c>
-      <c r="N9" s="83">
-        <f>SUM(N8:N8)</f>
-        <v/>
-      </c>
-      <c r="O9" s="82">
-        <f>SUM(O8:O8)</f>
-        <v/>
-      </c>
-      <c r="P9" s="84">
-        <f>IFERROR(M9/O9,0)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="82">
-        <f>SUM(Q8:Q8)</f>
-        <v/>
-      </c>
-      <c r="R9" s="82">
-        <f>SUM(R8:R8)</f>
-        <v/>
-      </c>
-      <c r="S9" s="120">
-        <f>SUM(S8:S8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="63">
-      <c r="A10" s="73" t="inlineStr">
-        <is>
-          <t>Σ Hero</t>
-        </is>
-      </c>
-      <c r="B10" s="74" t="n"/>
-      <c r="C10" s="74" t="n"/>
-      <c r="D10" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="E10" s="74" t="n"/>
-      <c r="F10" s="74" t="n"/>
-      <c r="G10" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="H10" s="74" t="n"/>
-      <c r="I10" s="74" t="n"/>
-      <c r="J10" s="74" t="n"/>
-      <c r="K10" s="74" t="n"/>
-      <c r="L10" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="63">
-      <c r="A11" s="73" t="inlineStr">
-        <is>
-          <t>Σ Esteira</t>
-        </is>
-      </c>
-      <c r="B11" s="74" t="n"/>
-      <c r="C11" s="74" t="n"/>
-      <c r="D11" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="E11" s="74" t="n"/>
-      <c r="F11" s="74" t="n"/>
-      <c r="G11" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="H11" s="74" t="n"/>
-      <c r="I11" s="74" t="n"/>
-      <c r="J11" s="74" t="n"/>
-      <c r="K11" s="74" t="n"/>
-      <c r="L11" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="63">
-      <c r="A13" s="71" t="inlineStr">
-        <is>
-          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="63">
-      <c r="A14" s="71" t="inlineStr">
         <is>
           <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
         </is>
@@ -6712,7 +7871,7 @@
     <row r="1" ht="16.15" customHeight="1" s="63">
       <c r="A1" s="64" t="inlineStr">
         <is>
-          <t>Busca e Mall — meta por SKU e pace diário</t>
+          <t>Vitrine loja — meta por SKU e pace diário</t>
         </is>
       </c>
     </row>
@@ -6724,7 +7883,7 @@
       </c>
       <c r="B2" s="89" t="inlineStr">
         <is>
-          <t>Busca e Mall</t>
+          <t>Vitrine loja</t>
         </is>
       </c>
       <c r="C2" s="66" t="inlineStr">
@@ -6734,7 +7893,7 @@
       </c>
       <c r="D2" s="89" t="inlineStr">
         <is>
-          <t>BUSCA / MALL / OUTROS</t>
+          <t>VITRINE DA LOJA</t>
         </is>
       </c>
       <c r="F2" s="66" t="inlineStr">
@@ -6744,7 +7903,7 @@
       </c>
       <c r="G2" s="89" t="inlineStr">
         <is>
-          <t>Misto</t>
+          <t>Loja / vendedor</t>
         </is>
       </c>
       <c r="I2" s="66" t="inlineStr">
@@ -6754,7 +7913,7 @@
       </c>
       <c r="K2" s="121" t="inlineStr">
         <is>
-          <t>R$0 — nesta atribuição (API 202605) total = seller(live+vídeo+card)+afiliada, resíduo zero. Sem balde separado.</t>
+          <t>TRANSVERSAL — shop_tab R$89.369 (jul, API 202605) SOBREPÕE card/loja; não somável no NET (lente de superfície, não de último-conteúdo).</t>
         </is>
       </c>
     </row>
@@ -6766,7 +7925,7 @@
       </c>
       <c r="B3" s="89" t="inlineStr">
         <is>
-          <t>A definir — SEO de título/atributo de produto</t>
+          <t>A definir — organizar vitrine por curva e coleção</t>
         </is>
       </c>
     </row>
@@ -6777,7 +7936,7 @@
         </is>
       </c>
       <c r="B4" s="107">
-        <f>Premissas!$C$32</f>
+        <f>Premissas!$C$31</f>
         <v/>
       </c>
       <c r="C4" s="66" t="inlineStr">
@@ -6786,7 +7945,7 @@
         </is>
       </c>
       <c r="D4" s="107">
-        <f>Premissas!$D$32</f>
+        <f>Premissas!$D$31</f>
         <v/>
       </c>
       <c r="F4" s="66" t="inlineStr">
@@ -7152,6 +8311,475 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="10" customWidth="1" style="62" min="1" max="1"/>
+    <col width="22" customWidth="1" style="62" min="2" max="2"/>
+    <col width="5" customWidth="1" style="62" min="3" max="3"/>
+    <col width="12" customWidth="1" style="62" min="4" max="4"/>
+    <col width="8" customWidth="1" style="62" min="5" max="5"/>
+    <col width="10" customWidth="1" style="62" min="6" max="7"/>
+    <col width="11" customWidth="1" style="62" min="8" max="8"/>
+    <col width="12" customWidth="1" style="62" min="9" max="9"/>
+    <col width="9" customWidth="1" style="62" min="10" max="10"/>
+    <col width="11" customWidth="1" style="62" min="11" max="11"/>
+    <col width="13" customWidth="1" style="62" min="12" max="12"/>
+    <col width="12" customWidth="1" style="62" min="13" max="13"/>
+    <col width="13" customWidth="1" style="62" min="14" max="15"/>
+    <col width="11" customWidth="1" style="62" min="16" max="16"/>
+    <col width="12" customWidth="1" style="62" min="17" max="18"/>
+    <col width="14" customWidth="1" style="62" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.15" customHeight="1" s="63">
+      <c r="A1" s="64" t="inlineStr">
+        <is>
+          <t>Busca e Mall — meta por SKU e pace diário</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="63">
+      <c r="A2" s="66" t="inlineStr">
+        <is>
+          <t>Canal (chave):</t>
+        </is>
+      </c>
+      <c r="B2" s="89" t="inlineStr">
+        <is>
+          <t>Busca e Mall</t>
+        </is>
+      </c>
+      <c r="C2" s="66" t="inlineStr">
+        <is>
+          <t>Superfície:</t>
+        </is>
+      </c>
+      <c r="D2" s="89" t="inlineStr">
+        <is>
+          <t>BUSCA / MALL / OUTROS</t>
+        </is>
+      </c>
+      <c r="F2" s="66" t="inlineStr">
+        <is>
+          <t>Atribuição:</t>
+        </is>
+      </c>
+      <c r="G2" s="89" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="I2" s="66" t="inlineStr">
+        <is>
+          <t>Confiança da base jul:</t>
+        </is>
+      </c>
+      <c r="K2" s="121" t="inlineStr">
+        <is>
+          <t>R$0 — nesta atribuição (API 202605) total = seller(live+vídeo+card)+afiliada, resíduo zero. Sem balde separado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="63">
+      <c r="A3" s="66" t="inlineStr">
+        <is>
+          <t>Alavanca principal:</t>
+        </is>
+      </c>
+      <c r="B3" s="89" t="inlineStr">
+        <is>
+          <t>A definir — SEO de título/atributo de produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="63">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>Crescimento vs base:</t>
+        </is>
+      </c>
+      <c r="B4" s="107">
+        <f>Premissas!$C$32</f>
+        <v/>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Comissão afiliada:</t>
+        </is>
+      </c>
+      <c r="D4" s="107">
+        <f>Premissas!$D$32</f>
+        <v/>
+      </c>
+      <c r="F4" s="66" t="inlineStr">
+        <is>
+          <t>CPV padrão:</t>
+        </is>
+      </c>
+      <c r="G4" s="108">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="63">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>Meta do canal (pç):</t>
+        </is>
+      </c>
+      <c r="B5" s="109">
+        <f>G9</f>
+        <v/>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>Meta GMV:</t>
+        </is>
+      </c>
+      <c r="D5" s="110">
+        <f>I9</f>
+        <v/>
+      </c>
+      <c r="F5" s="66" t="inlineStr">
+        <is>
+          <t>Contribuição meta:</t>
+        </is>
+      </c>
+      <c r="G5" s="110">
+        <f>L9</f>
+        <v/>
+      </c>
+      <c r="I5" s="66" t="inlineStr">
+        <is>
+          <t>Índice de pace:</t>
+        </is>
+      </c>
+      <c r="K5" s="111">
+        <f>P9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="63">
+      <c r="A7" s="72" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B7" s="72" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>Base jul (pç)</t>
+        </is>
+      </c>
+      <c r="E7" s="72" t="inlineStr">
+        <is>
+          <t>Mix jul</t>
+        </is>
+      </c>
+      <c r="F7" s="72" t="inlineStr">
+        <is>
+          <t>Ajuste (pç)</t>
+        </is>
+      </c>
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>Meta (pç)</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="inlineStr">
+        <is>
+          <t>Preço plan.</t>
+        </is>
+      </c>
+      <c r="I7" s="72" t="inlineStr">
+        <is>
+          <t>Meta GMV</t>
+        </is>
+      </c>
+      <c r="J7" s="72" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="K7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib./pç</t>
+        </is>
+      </c>
+      <c r="L7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib. meta</t>
+        </is>
+      </c>
+      <c r="M7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (pç)</t>
+        </is>
+      </c>
+      <c r="N7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (R$)</t>
+        </is>
+      </c>
+      <c r="O7" s="72" t="inlineStr">
+        <is>
+          <t>Esperado MTD</t>
+        </is>
+      </c>
+      <c r="P7" s="72" t="inlineStr">
+        <is>
+          <t>Índice pace</t>
+        </is>
+      </c>
+      <c r="Q7" s="72" t="inlineStr">
+        <is>
+          <t>Projeção fim</t>
+        </is>
+      </c>
+      <c r="R7" s="72" t="inlineStr">
+        <is>
+          <t>Gap vs meta</t>
+        </is>
+      </c>
+      <c r="S7" s="72" t="inlineStr">
+        <is>
+          <t>Pç/dia p/ fechar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="63">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B8" s="74" t="inlineStr">
+        <is>
+          <t>Sem base de julho para este canal</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="113">
+        <f>IFERROR(D8/$D$9,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="112">
+        <f>ROUND(D8*(1+$B$4),0)+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="114">
+        <f>G8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K8" s="116">
+        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="114">
+        <f>G8*K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="112">
+        <f>G8*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P8" s="117">
+        <f>IFERROR(M8/O8,0)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="112">
+        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R8" s="112">
+        <f>Q8-G8</f>
+        <v/>
+      </c>
+      <c r="S8" s="118">
+        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="63">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="n"/>
+      <c r="C9" s="81" t="n"/>
+      <c r="D9" s="82">
+        <f>SUM(D8:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="85">
+        <f>SUM(E8:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="82">
+        <f>SUM(F8:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="82">
+        <f>SUM(G8:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="119" t="n"/>
+      <c r="I9" s="83">
+        <f>SUM(I8:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="119" t="n"/>
+      <c r="K9" s="119" t="n"/>
+      <c r="L9" s="83">
+        <f>SUM(L8:L8)</f>
+        <v/>
+      </c>
+      <c r="M9" s="82">
+        <f>SUM(M8:M8)</f>
+        <v/>
+      </c>
+      <c r="N9" s="83">
+        <f>SUM(N8:N8)</f>
+        <v/>
+      </c>
+      <c r="O9" s="82">
+        <f>SUM(O8:O8)</f>
+        <v/>
+      </c>
+      <c r="P9" s="84">
+        <f>IFERROR(M9/O9,0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="82">
+        <f>SUM(Q8:Q8)</f>
+        <v/>
+      </c>
+      <c r="R9" s="82">
+        <f>SUM(R8:R8)</f>
+        <v/>
+      </c>
+      <c r="S9" s="120">
+        <f>SUM(S8:S8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="63">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>Σ Hero</t>
+        </is>
+      </c>
+      <c r="B10" s="74" t="n"/>
+      <c r="C10" s="74" t="n"/>
+      <c r="D10" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="E10" s="74" t="n"/>
+      <c r="F10" s="74" t="n"/>
+      <c r="G10" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="H10" s="74" t="n"/>
+      <c r="I10" s="74" t="n"/>
+      <c r="J10" s="74" t="n"/>
+      <c r="K10" s="74" t="n"/>
+      <c r="L10" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="63">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>Σ Esteira</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="n"/>
+      <c r="C11" s="74" t="n"/>
+      <c r="D11" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="E11" s="74" t="n"/>
+      <c r="F11" s="74" t="n"/>
+      <c r="G11" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="H11" s="74" t="n"/>
+      <c r="I11" s="74" t="n"/>
+      <c r="J11" s="74" t="n"/>
+      <c r="K11" s="74" t="n"/>
+      <c r="L11" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="63">
+      <c r="A13" s="71" t="inlineStr">
+        <is>
+          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="63">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12779,6 +14407,461 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" style="63" min="1" max="1"/>
+    <col width="14" customWidth="1" style="63" min="2" max="2"/>
+    <col width="40" customWidth="1" style="63" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="63">
+      <c r="A1" s="148" t="inlineStr">
+        <is>
+          <t>Simulador — Corrida de Vídeos + GMV Max</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="125" t="inlineStr">
+        <is>
+          <t>Mexa nos AMARELOS. Resultado de 1ª ordem (a corrida) e 2ª ordem (o prêmio real: ROAS do GMV Max + LTV). CPV e co-financiamento TT = dado real jun–ago.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="63">
+      <c r="A4" s="183" t="inlineStr">
+        <is>
+          <t>① A CORRIDA — parâmetros</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="187" t="inlineStr">
+        <is>
+          <t>Meta de vídeos na corrida</t>
+        </is>
+      </c>
+      <c r="B5" s="170" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="187" t="inlineStr">
+        <is>
+          <t>Creators que batem 5+ vídeos (ganham amostra)</t>
+        </is>
+      </c>
+      <c r="B6" s="170" t="n">
+        <v>250</v>
+      </c>
+      <c r="C6" s="178" t="inlineStr">
+        <is>
+          <t>premissa — distribuição do engajamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="187" t="inlineStr">
+        <is>
+          <t>CPV da amostra grátis (custo real)</t>
+        </is>
+      </c>
+      <c r="B7" s="188" t="n">
+        <v>45</v>
+      </c>
+      <c r="C7" s="178" t="inlineStr">
+        <is>
+          <t>custos_sku (R$39–49)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="187" t="inlineStr">
+        <is>
+          <t>Prêmios de pódio (1º+2º+3º, total)</t>
+        </is>
+      </c>
+      <c r="B8" s="188" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="187" t="inlineStr">
+        <is>
+          <t>Peças vendidas por vídeo (conversão)</t>
+        </is>
+      </c>
+      <c r="B9" s="174" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C9" s="178" t="inlineStr">
+        <is>
+          <t>o maior risco — vídeo != venda</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="187" t="inlineStr">
+        <is>
+          <t>Contribuição por peça s/ mídia (real)</t>
+        </is>
+      </c>
+      <c r="B10" s="200" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="C10" s="178" t="inlineStr">
+        <is>
+          <t>settlement 31,3% menos CPV</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="187" t="inlineStr">
+        <is>
+          <t>Peças vendidas pela corrida</t>
+        </is>
+      </c>
+      <c r="B11" s="201">
+        <f>B5*B9</f>
+        <v/>
+      </c>
+      <c r="C11" s="178" t="inlineStr">
+        <is>
+          <t>vídeos × conversão</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="63">
+      <c r="A12" s="190" t="inlineStr">
+        <is>
+          <t>② O CUPOM — quem paga</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="187" t="inlineStr">
+        <is>
+          <t>Valor do cupom p/ audiência (R$)</t>
+        </is>
+      </c>
+      <c r="B13" s="188" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="187" t="inlineStr">
+        <is>
+          <t>% dos pedidos que usam o cupom</t>
+        </is>
+      </c>
+      <c r="B14" s="189" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="187" t="inlineStr">
+        <is>
+          <t>% do cupom bancado pela TikTok</t>
+        </is>
+      </c>
+      <c r="B15" s="189" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="178" t="inlineStr">
+        <is>
+          <t>HOJE ~3,5%; sobe só entrando em campanha TT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="187" t="inlineStr">
+        <is>
+          <t>Resgates de cupom</t>
+        </is>
+      </c>
+      <c r="B16" s="201">
+        <f>B11*B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="187" t="inlineStr">
+        <is>
+          <t>Custo do cupom que a RHODE paga</t>
+        </is>
+      </c>
+      <c r="B17" s="202">
+        <f>-B16*B13*(1-B15)</f>
+        <v/>
+      </c>
+      <c r="C17" s="178" t="inlineStr">
+        <is>
+          <t>cada R$10 come a contribuição de R$7,5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="63">
+      <c r="A18" s="193" t="inlineStr">
+        <is>
+          <t>③ RESULTADO DA CORRIDA (1ª ordem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="187" t="inlineStr">
+        <is>
+          <t>(+) Contribuição das peças vendidas</t>
+        </is>
+      </c>
+      <c r="B19" s="203">
+        <f>B11*B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="187" t="inlineStr">
+        <is>
+          <t>(−) Amostras grátis</t>
+        </is>
+      </c>
+      <c r="B20" s="202">
+        <f>-B6*B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="187" t="inlineStr">
+        <is>
+          <t>(−) Prêmios de pódio</t>
+        </is>
+      </c>
+      <c r="B21" s="202">
+        <f>-B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="155">
+        <f> RESULTADO 1ª ordem</f>
+        <v/>
+      </c>
+      <c r="B22" s="204">
+        <f>B19+B20+B21+B17</f>
+        <v/>
+      </c>
+      <c r="C22" s="178" t="inlineStr">
+        <is>
+          <t>se negativo, só paga na 2ª ordem</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="63">
+      <c r="A23" s="192" t="inlineStr">
+        <is>
+          <t>④ O PRÊMIO REAL — criativo destrava o GMV Max (2ª ordem)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="187" t="inlineStr">
+        <is>
+          <t>Budget de GMV Max / mês</t>
+        </is>
+      </c>
+      <c r="B24" s="188" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="187" t="inlineStr">
+        <is>
+          <t>Margem de contribuição s/ GMV</t>
+        </is>
+      </c>
+      <c r="B25" s="189" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="C25" s="178" t="inlineStr">
+        <is>
+          <t>~R$7,5 em ~R$82 pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="187" t="inlineStr">
+        <is>
+          <t>Break-even do ROAS (não perder $)</t>
+        </is>
+      </c>
+      <c r="B26" s="205">
+        <f>1/B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="178" t="inlineStr">
+        <is>
+          <t>abaixo disso o GMV Max SANGRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="187" t="inlineStr">
+        <is>
+          <t>ROAS hoje (sem criativo)</t>
+        </is>
+      </c>
+      <c r="B27" s="194" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" s="178" t="inlineStr">
+        <is>
+          <t>&lt; break-even → perde dinheiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="187" t="inlineStr">
+        <is>
+          <t>ROAS com criativo da corrida</t>
+        </is>
+      </c>
+      <c r="B28" s="194" t="n">
+        <v>11</v>
+      </c>
+      <c r="C28" s="178" t="inlineStr">
+        <is>
+          <t>meta realista; 14 é upside</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="187" t="inlineStr">
+        <is>
+          <t>Contribuição GMV Max HOJE</t>
+        </is>
+      </c>
+      <c r="B29" s="202">
+        <f>B24*(B27*B25-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="187" t="inlineStr">
+        <is>
+          <t>Contribuição GMV Max PÓS-corrida</t>
+        </is>
+      </c>
+      <c r="B30" s="203">
+        <f>B24*(B28*B25-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="155">
+        <f> GANHO recorrente/mês no GMV Max</f>
+        <v/>
+      </c>
+      <c r="B31" s="206">
+        <f>B30-B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="63">
+      <c r="A32" s="207" t="inlineStr">
+        <is>
+          <t>⑤ LTV — clientes novos da corrida</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="187" t="inlineStr">
+        <is>
+          <t>Taxa de recompra</t>
+        </is>
+      </c>
+      <c r="B33" s="189" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="C33" s="178" t="inlineStr">
+        <is>
+          <t>piso medido</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="187" t="inlineStr">
+        <is>
+          <t>Contribuição por pedido de recompra</t>
+        </is>
+      </c>
+      <c r="B34" s="188" t="n">
+        <v>25</v>
+      </c>
+      <c r="C34" s="178" t="inlineStr">
+        <is>
+          <t>sem CAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="187" t="inlineStr">
+        <is>
+          <t>Contribuição futura (LTV)</t>
+        </is>
+      </c>
+      <c r="B35" s="208">
+        <f>B16*B33*B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="63">
+      <c r="A36" s="183" t="inlineStr">
+        <is>
+          <t>VEREDITO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="155" t="inlineStr">
+        <is>
+          <t>2ª ordem + recorrente (swing GMV Max + LTV)</t>
+        </is>
+      </c>
+      <c r="B37" s="206">
+        <f>B31+B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="40" customHeight="1" s="63">
+      <c r="A38" s="175" t="inlineStr">
+        <is>
+          <t>A corrida quase sempre dá ~zero/negativo na 1ª ordem. Ela se paga SE (a) os vídeos virarem criativo e o ROAS cruzar o break-even (~11x), e (b) o cupom vier de campanha co-financiada OU preso a combo. O KPI de sucesso é o SWING do GMV Max — não a contagem de vídeos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A38:C40"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -14180,1565 +16263,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:S28"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="10" customWidth="1" style="62" min="1" max="1"/>
-    <col width="22" customWidth="1" style="62" min="2" max="2"/>
-    <col width="5" customWidth="1" style="62" min="3" max="3"/>
-    <col width="12" customWidth="1" style="62" min="4" max="4"/>
-    <col width="8" customWidth="1" style="62" min="5" max="5"/>
-    <col width="10" customWidth="1" style="62" min="6" max="7"/>
-    <col width="11" customWidth="1" style="62" min="8" max="8"/>
-    <col width="12" customWidth="1" style="62" min="9" max="9"/>
-    <col width="9" customWidth="1" style="62" min="10" max="10"/>
-    <col width="11" customWidth="1" style="62" min="11" max="11"/>
-    <col width="13" customWidth="1" style="62" min="12" max="12"/>
-    <col width="12" customWidth="1" style="62" min="13" max="13"/>
-    <col width="13" customWidth="1" style="62" min="14" max="15"/>
-    <col width="11" customWidth="1" style="62" min="16" max="16"/>
-    <col width="12" customWidth="1" style="62" min="17" max="18"/>
-    <col width="14" customWidth="1" style="62" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="63">
-      <c r="A1" s="64" t="inlineStr">
-        <is>
-          <t>Vídeo afiliada — meta por SKU e pace diário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="63">
-      <c r="A2" s="66" t="inlineStr">
-        <is>
-          <t>Canal (chave):</t>
-        </is>
-      </c>
-      <c r="B2" s="89" t="inlineStr">
-        <is>
-          <t>Vídeo afiliada</t>
-        </is>
-      </c>
-      <c r="C2" s="66" t="inlineStr">
-        <is>
-          <t>Superfície:</t>
-        </is>
-      </c>
-      <c r="D2" s="89" t="inlineStr">
-        <is>
-          <t>VÍDEO</t>
-        </is>
-      </c>
-      <c r="F2" s="66" t="inlineStr">
-        <is>
-          <t>Atribuição:</t>
-        </is>
-      </c>
-      <c r="G2" s="89" t="inlineStr">
-        <is>
-          <t>Afiliada</t>
-        </is>
-      </c>
-      <c r="I2" s="66" t="inlineStr">
-        <is>
-          <t>Confiança da base jul:</t>
-        </is>
-      </c>
-      <c r="K2" s="89" t="inlineStr">
-        <is>
-          <t>EXATO — extrato de afiliada</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="63">
-      <c r="A3" s="66" t="inlineStr">
-        <is>
-          <t>Alavanca principal:</t>
-        </is>
-      </c>
-      <c r="B3" s="89" t="inlineStr">
-        <is>
-          <t>Copa Rhode Creators (gamificação) + Academia + desova de seeding</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="63">
-      <c r="A4" s="66" t="inlineStr">
-        <is>
-          <t>Crescimento vs base:</t>
-        </is>
-      </c>
-      <c r="B4" s="107">
-        <f>Premissas!$C$26</f>
-        <v/>
-      </c>
-      <c r="C4" s="66" t="inlineStr">
-        <is>
-          <t>Comissão afiliada:</t>
-        </is>
-      </c>
-      <c r="D4" s="107">
-        <f>Premissas!$D$26</f>
-        <v/>
-      </c>
-      <c r="F4" s="66" t="inlineStr">
-        <is>
-          <t>CPV padrão:</t>
-        </is>
-      </c>
-      <c r="G4" s="108">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="63">
-      <c r="A5" s="66" t="inlineStr">
-        <is>
-          <t>Meta do canal (pç):</t>
-        </is>
-      </c>
-      <c r="B5" s="109">
-        <f>G23</f>
-        <v/>
-      </c>
-      <c r="C5" s="66" t="inlineStr">
-        <is>
-          <t>Meta GMV:</t>
-        </is>
-      </c>
-      <c r="D5" s="110">
-        <f>I23</f>
-        <v/>
-      </c>
-      <c r="F5" s="66" t="inlineStr">
-        <is>
-          <t>Contribuição meta:</t>
-        </is>
-      </c>
-      <c r="G5" s="110">
-        <f>L23</f>
-        <v/>
-      </c>
-      <c r="I5" s="66" t="inlineStr">
-        <is>
-          <t>Índice de pace:</t>
-        </is>
-      </c>
-      <c r="K5" s="111">
-        <f>P23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="63">
-      <c r="A7" s="72" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B7" s="72" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="C7" s="72" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="D7" s="72" t="inlineStr">
-        <is>
-          <t>Base jul (pç)</t>
-        </is>
-      </c>
-      <c r="E7" s="72" t="inlineStr">
-        <is>
-          <t>Mix jul</t>
-        </is>
-      </c>
-      <c r="F7" s="72" t="inlineStr">
-        <is>
-          <t>Ajuste (pç)</t>
-        </is>
-      </c>
-      <c r="G7" s="72" t="inlineStr">
-        <is>
-          <t>Meta (pç)</t>
-        </is>
-      </c>
-      <c r="H7" s="72" t="inlineStr">
-        <is>
-          <t>Preço plan.</t>
-        </is>
-      </c>
-      <c r="I7" s="72" t="inlineStr">
-        <is>
-          <t>Meta GMV</t>
-        </is>
-      </c>
-      <c r="J7" s="72" t="inlineStr">
-        <is>
-          <t>CPV</t>
-        </is>
-      </c>
-      <c r="K7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib./pç</t>
-        </is>
-      </c>
-      <c r="L7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib. meta</t>
-        </is>
-      </c>
-      <c r="M7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (pç)</t>
-        </is>
-      </c>
-      <c r="N7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (R$)</t>
-        </is>
-      </c>
-      <c r="O7" s="72" t="inlineStr">
-        <is>
-          <t>Esperado MTD</t>
-        </is>
-      </c>
-      <c r="P7" s="72" t="inlineStr">
-        <is>
-          <t>Índice pace</t>
-        </is>
-      </c>
-      <c r="Q7" s="72" t="inlineStr">
-        <is>
-          <t>Projeção fim</t>
-        </is>
-      </c>
-      <c r="R7" s="72" t="inlineStr">
-        <is>
-          <t>Gap vs meta</t>
-        </is>
-      </c>
-      <c r="S7" s="72" t="inlineStr">
-        <is>
-          <t>Pç/dia p/ fechar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="63">
-      <c r="A8" s="73" t="inlineStr">
-        <is>
-          <t>REF516</t>
-        </is>
-      </c>
-      <c r="B8" s="74" t="inlineStr">
-        <is>
-          <t>Marmorizada</t>
-        </is>
-      </c>
-      <c r="C8" s="74" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D8" s="112" t="n">
-        <v>715</v>
-      </c>
-      <c r="E8" s="113">
-        <f>IFERROR(D8/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="112">
-        <f>ROUND(D8*(1+$B$4),0)+F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="97" t="n">
-        <v>93</v>
-      </c>
-      <c r="I8" s="114">
-        <f>G8*H8</f>
-        <v/>
-      </c>
-      <c r="J8" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K8" s="116">
-        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="114">
-        <f>G8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="112">
-        <f>G8*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P8" s="117">
-        <f>IFERROR(M8/O8,0)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="112">
-        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R8" s="112">
-        <f>Q8-G8</f>
-        <v/>
-      </c>
-      <c r="S8" s="118">
-        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="63">
-      <c r="A9" s="73" t="inlineStr">
-        <is>
-          <t>REF527</t>
-        </is>
-      </c>
-      <c r="B9" s="74" t="inlineStr">
-        <is>
-          <t>Sky Used</t>
-        </is>
-      </c>
-      <c r="C9" s="74" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D9" s="112" t="n">
-        <v>183</v>
-      </c>
-      <c r="E9" s="113">
-        <f>IFERROR(D9/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="112">
-        <f>ROUND(D9*(1+$B$4),0)+F9</f>
-        <v/>
-      </c>
-      <c r="H9" s="97" t="n">
-        <v>93.73999999999999</v>
-      </c>
-      <c r="I9" s="114">
-        <f>G9*H9</f>
-        <v/>
-      </c>
-      <c r="J9" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K9" s="116">
-        <f>H9*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J9</f>
-        <v/>
-      </c>
-      <c r="L9" s="114">
-        <f>G9*K9</f>
-        <v/>
-      </c>
-      <c r="M9" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A9)</f>
-        <v/>
-      </c>
-      <c r="N9" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A9)</f>
-        <v/>
-      </c>
-      <c r="O9" s="112">
-        <f>G9*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P9" s="117">
-        <f>IFERROR(M9/O9,0)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="112">
-        <f>IFERROR(M9/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R9" s="112">
-        <f>Q9-G9</f>
-        <v/>
-      </c>
-      <c r="S9" s="118">
-        <f>IFERROR(MAX(0,G9-M9)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="63">
-      <c r="A10" s="73" t="inlineStr">
-        <is>
-          <t>REF525</t>
-        </is>
-      </c>
-      <c r="B10" s="74" t="inlineStr">
-        <is>
-          <t>Stone Used</t>
-        </is>
-      </c>
-      <c r="C10" s="74" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D10" s="112" t="n">
-        <v>139</v>
-      </c>
-      <c r="E10" s="113">
-        <f>IFERROR(D10/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F10" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="112">
-        <f>ROUND(D10*(1+$B$4),0)+F10</f>
-        <v/>
-      </c>
-      <c r="H10" s="97" t="n">
-        <v>98.27</v>
-      </c>
-      <c r="I10" s="114">
-        <f>G10*H10</f>
-        <v/>
-      </c>
-      <c r="J10" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K10" s="116">
-        <f>H10*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J10</f>
-        <v/>
-      </c>
-      <c r="L10" s="114">
-        <f>G10*K10</f>
-        <v/>
-      </c>
-      <c r="M10" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A10)</f>
-        <v/>
-      </c>
-      <c r="N10" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A10)</f>
-        <v/>
-      </c>
-      <c r="O10" s="112">
-        <f>G10*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P10" s="117">
-        <f>IFERROR(M10/O10,0)</f>
-        <v/>
-      </c>
-      <c r="Q10" s="112">
-        <f>IFERROR(M10/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R10" s="112">
-        <f>Q10-G10</f>
-        <v/>
-      </c>
-      <c r="S10" s="118">
-        <f>IFERROR(MAX(0,G10-M10)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="63">
-      <c r="A11" s="73" t="inlineStr">
-        <is>
-          <t>REF588</t>
-        </is>
-      </c>
-      <c r="B11" s="74" t="inlineStr">
-        <is>
-          <t>Mom Marmorizada</t>
-        </is>
-      </c>
-      <c r="C11" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D11" s="112" t="n">
-        <v>127</v>
-      </c>
-      <c r="E11" s="113">
-        <f>IFERROR(D11/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="112">
-        <f>ROUND(D11*(1+$B$4),0)+F11</f>
-        <v/>
-      </c>
-      <c r="H11" s="97" t="n">
-        <v>95.76000000000001</v>
-      </c>
-      <c r="I11" s="114">
-        <f>G11*H11</f>
-        <v/>
-      </c>
-      <c r="J11" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K11" s="116">
-        <f>H11*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J11</f>
-        <v/>
-      </c>
-      <c r="L11" s="114">
-        <f>G11*K11</f>
-        <v/>
-      </c>
-      <c r="M11" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A11)</f>
-        <v/>
-      </c>
-      <c r="O11" s="112">
-        <f>G11*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P11" s="117">
-        <f>IFERROR(M11/O11,0)</f>
-        <v/>
-      </c>
-      <c r="Q11" s="112">
-        <f>IFERROR(M11/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R11" s="112">
-        <f>Q11-G11</f>
-        <v/>
-      </c>
-      <c r="S11" s="118">
-        <f>IFERROR(MAX(0,G11-M11)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="63">
-      <c r="A12" s="73" t="inlineStr">
-        <is>
-          <t>REF587</t>
-        </is>
-      </c>
-      <c r="B12" s="74" t="inlineStr">
-        <is>
-          <t>Baggy Marmorizada</t>
-        </is>
-      </c>
-      <c r="C12" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D12" s="112" t="n">
-        <v>83</v>
-      </c>
-      <c r="E12" s="113">
-        <f>IFERROR(D12/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F12" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="112">
-        <f>ROUND(D12*(1+$B$4),0)+F12</f>
-        <v/>
-      </c>
-      <c r="H12" s="97" t="n">
-        <v>98.44</v>
-      </c>
-      <c r="I12" s="114">
-        <f>G12*H12</f>
-        <v/>
-      </c>
-      <c r="J12" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K12" s="116">
-        <f>H12*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J12</f>
-        <v/>
-      </c>
-      <c r="L12" s="114">
-        <f>G12*K12</f>
-        <v/>
-      </c>
-      <c r="M12" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A12)</f>
-        <v/>
-      </c>
-      <c r="N12" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A12)</f>
-        <v/>
-      </c>
-      <c r="O12" s="112">
-        <f>G12*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P12" s="117">
-        <f>IFERROR(M12/O12,0)</f>
-        <v/>
-      </c>
-      <c r="Q12" s="112">
-        <f>IFERROR(M12/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R12" s="112">
-        <f>Q12-G12</f>
-        <v/>
-      </c>
-      <c r="S12" s="118">
-        <f>IFERROR(MAX(0,G12-M12)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="63">
-      <c r="A13" s="73" t="inlineStr">
-        <is>
-          <t>REF549</t>
-        </is>
-      </c>
-      <c r="B13" s="74" t="inlineStr">
-        <is>
-          <t>Rosa Bebê</t>
-        </is>
-      </c>
-      <c r="C13" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D13" s="112" t="n">
-        <v>45</v>
-      </c>
-      <c r="E13" s="113">
-        <f>IFERROR(D13/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F13" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="112">
-        <f>ROUND(D13*(1+$B$4),0)+F13</f>
-        <v/>
-      </c>
-      <c r="H13" s="97" t="n">
-        <v>97.23</v>
-      </c>
-      <c r="I13" s="114">
-        <f>G13*H13</f>
-        <v/>
-      </c>
-      <c r="J13" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K13" s="116">
-        <f>H13*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J13</f>
-        <v/>
-      </c>
-      <c r="L13" s="114">
-        <f>G13*K13</f>
-        <v/>
-      </c>
-      <c r="M13" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A13)</f>
-        <v/>
-      </c>
-      <c r="O13" s="112">
-        <f>G13*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P13" s="117">
-        <f>IFERROR(M13/O13,0)</f>
-        <v/>
-      </c>
-      <c r="Q13" s="112">
-        <f>IFERROR(M13/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R13" s="112">
-        <f>Q13-G13</f>
-        <v/>
-      </c>
-      <c r="S13" s="118">
-        <f>IFERROR(MAX(0,G13-M13)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="63">
-      <c r="A14" s="73" t="inlineStr">
-        <is>
-          <t>REF559</t>
-        </is>
-      </c>
-      <c r="B14" s="74" t="inlineStr">
-        <is>
-          <t>Mom Rosa</t>
-        </is>
-      </c>
-      <c r="C14" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D14" s="112" t="n">
-        <v>26</v>
-      </c>
-      <c r="E14" s="113">
-        <f>IFERROR(D14/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F14" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="112">
-        <f>ROUND(D14*(1+$B$4),0)+F14</f>
-        <v/>
-      </c>
-      <c r="H14" s="97" t="n">
-        <v>76.3</v>
-      </c>
-      <c r="I14" s="114">
-        <f>G14*H14</f>
-        <v/>
-      </c>
-      <c r="J14" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K14" s="116">
-        <f>H14*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J14</f>
-        <v/>
-      </c>
-      <c r="L14" s="114">
-        <f>G14*K14</f>
-        <v/>
-      </c>
-      <c r="M14" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A14)</f>
-        <v/>
-      </c>
-      <c r="O14" s="112">
-        <f>G14*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P14" s="117">
-        <f>IFERROR(M14/O14,0)</f>
-        <v/>
-      </c>
-      <c r="Q14" s="112">
-        <f>IFERROR(M14/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R14" s="112">
-        <f>Q14-G14</f>
-        <v/>
-      </c>
-      <c r="S14" s="118">
-        <f>IFERROR(MAX(0,G14-M14)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="63">
-      <c r="A15" s="73" t="inlineStr">
-        <is>
-          <t>REF566</t>
-        </is>
-      </c>
-      <c r="B15" s="74" t="inlineStr">
-        <is>
-          <t>Mom Choco</t>
-        </is>
-      </c>
-      <c r="C15" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D15" s="112" t="n">
-        <v>21</v>
-      </c>
-      <c r="E15" s="113">
-        <f>IFERROR(D15/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="112">
-        <f>ROUND(D15*(1+$B$4),0)+F15</f>
-        <v/>
-      </c>
-      <c r="H15" s="97" t="n">
-        <v>95.68000000000001</v>
-      </c>
-      <c r="I15" s="114">
-        <f>G15*H15</f>
-        <v/>
-      </c>
-      <c r="J15" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K15" s="116">
-        <f>H15*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J15</f>
-        <v/>
-      </c>
-      <c r="L15" s="114">
-        <f>G15*K15</f>
-        <v/>
-      </c>
-      <c r="M15" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A15)</f>
-        <v/>
-      </c>
-      <c r="O15" s="112">
-        <f>G15*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P15" s="117">
-        <f>IFERROR(M15/O15,0)</f>
-        <v/>
-      </c>
-      <c r="Q15" s="112">
-        <f>IFERROR(M15/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R15" s="112">
-        <f>Q15-G15</f>
-        <v/>
-      </c>
-      <c r="S15" s="118">
-        <f>IFERROR(MAX(0,G15-M15)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="63">
-      <c r="A16" s="73" t="inlineStr">
-        <is>
-          <t>REF558</t>
-        </is>
-      </c>
-      <c r="B16" s="74" t="inlineStr">
-        <is>
-          <t>(sem de-para)</t>
-        </is>
-      </c>
-      <c r="C16" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D16" s="112" t="n">
-        <v>20</v>
-      </c>
-      <c r="E16" s="113">
-        <f>IFERROR(D16/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="112">
-        <f>ROUND(D16*(1+$B$4),0)+F16</f>
-        <v/>
-      </c>
-      <c r="H16" s="97" t="n">
-        <v>75.98999999999999</v>
-      </c>
-      <c r="I16" s="114">
-        <f>G16*H16</f>
-        <v/>
-      </c>
-      <c r="J16" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K16" s="116">
-        <f>H16*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J16</f>
-        <v/>
-      </c>
-      <c r="L16" s="114">
-        <f>G16*K16</f>
-        <v/>
-      </c>
-      <c r="M16" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A16)</f>
-        <v/>
-      </c>
-      <c r="N16" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A16)</f>
-        <v/>
-      </c>
-      <c r="O16" s="112">
-        <f>G16*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P16" s="117">
-        <f>IFERROR(M16/O16,0)</f>
-        <v/>
-      </c>
-      <c r="Q16" s="112">
-        <f>IFERROR(M16/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R16" s="112">
-        <f>Q16-G16</f>
-        <v/>
-      </c>
-      <c r="S16" s="118">
-        <f>IFERROR(MAX(0,G16-M16)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="63">
-      <c r="A17" s="73" t="inlineStr">
-        <is>
-          <t>REF562</t>
-        </is>
-      </c>
-      <c r="B17" s="74" t="inlineStr">
-        <is>
-          <t>Chocolate</t>
-        </is>
-      </c>
-      <c r="C17" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D17" s="112" t="n">
-        <v>20</v>
-      </c>
-      <c r="E17" s="113">
-        <f>IFERROR(D17/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="92" t="n">
-        <v>149</v>
-      </c>
-      <c r="G17" s="112">
-        <f>ROUND(D17*(1+$B$4),0)+F17</f>
-        <v/>
-      </c>
-      <c r="H17" s="97" t="n">
-        <v>101.71</v>
-      </c>
-      <c r="I17" s="114">
-        <f>G17*H17</f>
-        <v/>
-      </c>
-      <c r="J17" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K17" s="116">
-        <f>H17*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J17</f>
-        <v/>
-      </c>
-      <c r="L17" s="114">
-        <f>G17*K17</f>
-        <v/>
-      </c>
-      <c r="M17" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A17)</f>
-        <v/>
-      </c>
-      <c r="N17" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A17)</f>
-        <v/>
-      </c>
-      <c r="O17" s="112">
-        <f>G17*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P17" s="117">
-        <f>IFERROR(M17/O17,0)</f>
-        <v/>
-      </c>
-      <c r="Q17" s="112">
-        <f>IFERROR(M17/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R17" s="112">
-        <f>Q17-G17</f>
-        <v/>
-      </c>
-      <c r="S17" s="118">
-        <f>IFERROR(MAX(0,G17-M17)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="63">
-      <c r="A18" s="73" t="inlineStr">
-        <is>
-          <t>REF550</t>
-        </is>
-      </c>
-      <c r="B18" s="74" t="inlineStr">
-        <is>
-          <t>Amarela</t>
-        </is>
-      </c>
-      <c r="C18" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D18" s="112" t="n">
-        <v>17</v>
-      </c>
-      <c r="E18" s="113">
-        <f>IFERROR(D18/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F18" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="112">
-        <f>ROUND(D18*(1+$B$4),0)+F18</f>
-        <v/>
-      </c>
-      <c r="H18" s="97" t="n">
-        <v>101.41</v>
-      </c>
-      <c r="I18" s="114">
-        <f>G18*H18</f>
-        <v/>
-      </c>
-      <c r="J18" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K18" s="116">
-        <f>H18*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J18</f>
-        <v/>
-      </c>
-      <c r="L18" s="114">
-        <f>G18*K18</f>
-        <v/>
-      </c>
-      <c r="M18" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A18)</f>
-        <v/>
-      </c>
-      <c r="N18" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A18)</f>
-        <v/>
-      </c>
-      <c r="O18" s="112">
-        <f>G18*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P18" s="117">
-        <f>IFERROR(M18/O18,0)</f>
-        <v/>
-      </c>
-      <c r="Q18" s="112">
-        <f>IFERROR(M18/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R18" s="112">
-        <f>Q18-G18</f>
-        <v/>
-      </c>
-      <c r="S18" s="118">
-        <f>IFERROR(MAX(0,G18-M18)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="63">
-      <c r="A19" s="73" t="inlineStr">
-        <is>
-          <t>REF551</t>
-        </is>
-      </c>
-      <c r="B19" s="74" t="inlineStr">
-        <is>
-          <t>Azul Médio</t>
-        </is>
-      </c>
-      <c r="C19" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D19" s="112" t="n">
-        <v>16</v>
-      </c>
-      <c r="E19" s="113">
-        <f>IFERROR(D19/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F19" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="112">
-        <f>ROUND(D19*(1+$B$4),0)+F19</f>
-        <v/>
-      </c>
-      <c r="H19" s="97" t="n">
-        <v>101.08</v>
-      </c>
-      <c r="I19" s="114">
-        <f>G19*H19</f>
-        <v/>
-      </c>
-      <c r="J19" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K19" s="116">
-        <f>H19*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J19</f>
-        <v/>
-      </c>
-      <c r="L19" s="114">
-        <f>G19*K19</f>
-        <v/>
-      </c>
-      <c r="M19" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A19)</f>
-        <v/>
-      </c>
-      <c r="N19" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A19)</f>
-        <v/>
-      </c>
-      <c r="O19" s="112">
-        <f>G19*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P19" s="117">
-        <f>IFERROR(M19/O19,0)</f>
-        <v/>
-      </c>
-      <c r="Q19" s="112">
-        <f>IFERROR(M19/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R19" s="112">
-        <f>Q19-G19</f>
-        <v/>
-      </c>
-      <c r="S19" s="118">
-        <f>IFERROR(MAX(0,G19-M19)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="63">
-      <c r="A20" s="73" t="inlineStr">
-        <is>
-          <t>REF528</t>
-        </is>
-      </c>
-      <c r="B20" s="74" t="inlineStr">
-        <is>
-          <t>Wide 528</t>
-        </is>
-      </c>
-      <c r="C20" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D20" s="112" t="n">
-        <v>15</v>
-      </c>
-      <c r="E20" s="113">
-        <f>IFERROR(D20/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F20" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="112">
-        <f>ROUND(D20*(1+$B$4),0)+F20</f>
-        <v/>
-      </c>
-      <c r="H20" s="97" t="n">
-        <v>83.68000000000001</v>
-      </c>
-      <c r="I20" s="114">
-        <f>G20*H20</f>
-        <v/>
-      </c>
-      <c r="J20" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K20" s="116">
-        <f>H20*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J20</f>
-        <v/>
-      </c>
-      <c r="L20" s="114">
-        <f>G20*K20</f>
-        <v/>
-      </c>
-      <c r="M20" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A20)</f>
-        <v/>
-      </c>
-      <c r="N20" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A20)</f>
-        <v/>
-      </c>
-      <c r="O20" s="112">
-        <f>G20*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P20" s="117">
-        <f>IFERROR(M20/O20,0)</f>
-        <v/>
-      </c>
-      <c r="Q20" s="112">
-        <f>IFERROR(M20/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R20" s="112">
-        <f>Q20-G20</f>
-        <v/>
-      </c>
-      <c r="S20" s="118">
-        <f>IFERROR(MAX(0,G20-M20)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="63">
-      <c r="A21" s="73" t="inlineStr">
-        <is>
-          <t>REF546</t>
-        </is>
-      </c>
-      <c r="B21" s="74" t="inlineStr">
-        <is>
-          <t>(sem de-para)</t>
-        </is>
-      </c>
-      <c r="C21" s="74" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D21" s="112" t="n">
-        <v>9</v>
-      </c>
-      <c r="E21" s="113">
-        <f>IFERROR(D21/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F21" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="112">
-        <f>ROUND(D21*(1+$B$4),0)+F21</f>
-        <v/>
-      </c>
-      <c r="H21" s="97" t="n">
-        <v>116.95</v>
-      </c>
-      <c r="I21" s="114">
-        <f>G21*H21</f>
-        <v/>
-      </c>
-      <c r="J21" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K21" s="116">
-        <f>H21*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J21</f>
-        <v/>
-      </c>
-      <c r="L21" s="114">
-        <f>G21*K21</f>
-        <v/>
-      </c>
-      <c r="M21" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A21)</f>
-        <v/>
-      </c>
-      <c r="N21" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A21)</f>
-        <v/>
-      </c>
-      <c r="O21" s="112">
-        <f>G21*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P21" s="117">
-        <f>IFERROR(M21/O21,0)</f>
-        <v/>
-      </c>
-      <c r="Q21" s="112">
-        <f>IFERROR(M21/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R21" s="112">
-        <f>Q21-G21</f>
-        <v/>
-      </c>
-      <c r="S21" s="118">
-        <f>IFERROR(MAX(0,G21-M21)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="63">
-      <c r="A22" s="73" t="inlineStr">
-        <is>
-          <t>CAUDA</t>
-        </is>
-      </c>
-      <c r="B22" s="74" t="inlineStr">
-        <is>
-          <t>SKUs de cauda não detalhados</t>
-        </is>
-      </c>
-      <c r="C22" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D22" s="112" t="n">
-        <v>39</v>
-      </c>
-      <c r="E22" s="113">
-        <f>IFERROR(D22/$D$23,0)</f>
-        <v/>
-      </c>
-      <c r="F22" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="112">
-        <f>ROUND(D22*(1+$B$4),0)+F22</f>
-        <v/>
-      </c>
-      <c r="H22" s="97" t="n">
-        <v>94.16</v>
-      </c>
-      <c r="I22" s="114">
-        <f>G22*H22</f>
-        <v/>
-      </c>
-      <c r="J22" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K22" s="116">
-        <f>H22*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J22</f>
-        <v/>
-      </c>
-      <c r="L22" s="114">
-        <f>G22*K22</f>
-        <v/>
-      </c>
-      <c r="M22" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A22)</f>
-        <v/>
-      </c>
-      <c r="N22" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A22)</f>
-        <v/>
-      </c>
-      <c r="O22" s="112">
-        <f>G22*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P22" s="117">
-        <f>IFERROR(M22/O22,0)</f>
-        <v/>
-      </c>
-      <c r="Q22" s="112">
-        <f>IFERROR(M22/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R22" s="112">
-        <f>Q22-G22</f>
-        <v/>
-      </c>
-      <c r="S22" s="118">
-        <f>IFERROR(MAX(0,G22-M22)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="63">
-      <c r="A23" s="81" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B23" s="81" t="n"/>
-      <c r="C23" s="81" t="n"/>
-      <c r="D23" s="82">
-        <f>SUM(D8:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="85">
-        <f>SUM(E8:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="82">
-        <f>SUM(F8:F22)</f>
-        <v/>
-      </c>
-      <c r="G23" s="82">
-        <f>SUM(G8:G22)</f>
-        <v/>
-      </c>
-      <c r="H23" s="119" t="n"/>
-      <c r="I23" s="83">
-        <f>SUM(I8:I22)</f>
-        <v/>
-      </c>
-      <c r="J23" s="119" t="n"/>
-      <c r="K23" s="119" t="n"/>
-      <c r="L23" s="83">
-        <f>SUM(L8:L22)</f>
-        <v/>
-      </c>
-      <c r="M23" s="82">
-        <f>SUM(M8:M22)</f>
-        <v/>
-      </c>
-      <c r="N23" s="83">
-        <f>SUM(N8:N22)</f>
-        <v/>
-      </c>
-      <c r="O23" s="82">
-        <f>SUM(O8:O22)</f>
-        <v/>
-      </c>
-      <c r="P23" s="84">
-        <f>IFERROR(M23/O23,0)</f>
-        <v/>
-      </c>
-      <c r="Q23" s="82">
-        <f>SUM(Q8:Q22)</f>
-        <v/>
-      </c>
-      <c r="R23" s="82">
-        <f>SUM(R8:R22)</f>
-        <v/>
-      </c>
-      <c r="S23" s="120">
-        <f>SUM(S8:S22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="63">
-      <c r="A24" s="73" t="inlineStr">
-        <is>
-          <t>Σ Hero</t>
-        </is>
-      </c>
-      <c r="B24" s="74" t="n"/>
-      <c r="C24" s="74" t="n"/>
-      <c r="D24" s="112">
-        <f>SUMIFS(D8:D22,$C$8:$C$22,"H")</f>
-        <v/>
-      </c>
-      <c r="E24" s="74" t="n"/>
-      <c r="F24" s="74" t="n"/>
-      <c r="G24" s="112">
-        <f>SUMIFS(G8:G22,$C$8:$C$22,"H")</f>
-        <v/>
-      </c>
-      <c r="H24" s="74" t="n"/>
-      <c r="I24" s="74" t="n"/>
-      <c r="J24" s="74" t="n"/>
-      <c r="K24" s="74" t="n"/>
-      <c r="L24" s="114">
-        <f>SUMIFS(L8:L22,$C$8:$C$22,"H")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="63">
-      <c r="A25" s="73" t="inlineStr">
-        <is>
-          <t>Σ Esteira</t>
-        </is>
-      </c>
-      <c r="B25" s="74" t="n"/>
-      <c r="C25" s="74" t="n"/>
-      <c r="D25" s="112">
-        <f>SUMIFS(D8:D22,$C$8:$C$22,"E")</f>
-        <v/>
-      </c>
-      <c r="E25" s="74" t="n"/>
-      <c r="F25" s="74" t="n"/>
-      <c r="G25" s="112">
-        <f>SUMIFS(G8:G22,$C$8:$C$22,"E")</f>
-        <v/>
-      </c>
-      <c r="H25" s="74" t="n"/>
-      <c r="I25" s="74" t="n"/>
-      <c r="J25" s="74" t="n"/>
-      <c r="K25" s="74" t="n"/>
-      <c r="L25" s="114">
-        <f>SUMIFS(L8:L22,$C$8:$C$22,"E")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="63">
-      <c r="A27" s="71" t="inlineStr">
-        <is>
-          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="63">
-      <c r="A28" s="71" t="inlineStr">
-        <is>
-          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(live): aba Live Própria — medido 13/08 + distribuição hero×esteira + gap R$230k (volume vs ticket, premium/dia)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
+++ b/dados/marketplace/tiktok/Rhode_SKU_x_Canal_template.xlsx
@@ -19,11 +19,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo afiliada" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card afiliada" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live loja" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo loja" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card loja" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitrine loja" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busca e Mall" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log diário" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Live Própria" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vídeo loja" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card loja" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vitrine loja" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Busca e Mall" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log diário" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -32,7 +33,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="12">
+  <numFmts count="14">
     <numFmt numFmtId="164" formatCode="&quot;R$ &quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="0.00\x"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -45,8 +46,10 @@
     <numFmt numFmtId="173" formatCode="0.0"/>
     <numFmt numFmtId="174" formatCode="&quot;R$&quot; #,##0"/>
     <numFmt numFmtId="175" formatCode="&quot;R$&quot; #,##0.00"/>
+    <numFmt numFmtId="176" formatCode="&quot;R$&quot; #,##0.0"/>
+    <numFmt numFmtId="177" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
-  <fonts count="46">
+  <fonts count="49">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -326,6 +329,21 @@
       <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001E7E34"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00C0392B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A1A1A"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="17">
     <fill>
@@ -461,7 +479,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="209">
+  <cellXfs count="228">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1047,6 +1065,59 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="174" fontId="45" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="46" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="46" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="42" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="47" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="47" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="48" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="33" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="42" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="33" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="47" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="42" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="47" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="47" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6203,6 +6274,509 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" style="63" min="1" max="1"/>
+    <col width="13" customWidth="1" style="63" min="2" max="2"/>
+    <col width="13" customWidth="1" style="63" min="3" max="3"/>
+    <col width="34" customWidth="1" style="63" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="63">
+      <c r="A1" s="148" t="inlineStr">
+        <is>
+          <t>Live Própria (Live loja) — medido + gap p/ R$230k</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="125" t="inlineStr">
+        <is>
+          <t>Medido até 13/08 (fechado). GMV oficial = seller_live da API (bate c/ Seller Center); peças e hero×esteira pelo método do pace (±3%). Amarelo = editável.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="63">
+      <c r="A4" s="183" t="inlineStr">
+        <is>
+          <t>① MEDIDO ATÉ 13/08</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="187" t="inlineStr">
+        <is>
+          <t>Meta de GMV (agosto)</t>
+        </is>
+      </c>
+      <c r="B5" s="188" t="n">
+        <v>230000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="187" t="inlineStr">
+        <is>
+          <t>Meta de peças (agosto)</t>
+        </is>
+      </c>
+      <c r="B6" s="170" t="n">
+        <v>2796</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="187" t="inlineStr">
+        <is>
+          <t>GMV medido (seller_live API, oficial)</t>
+        </is>
+      </c>
+      <c r="B7" s="209" t="n">
+        <v>59257</v>
+      </c>
+      <c r="D7" s="178" t="inlineStr">
+        <is>
+          <t>R$66k incl. 14/08 parcial</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="187" t="inlineStr">
+        <is>
+          <t>Peças medidas (método pace)</t>
+        </is>
+      </c>
+      <c r="B8" s="210" t="n">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="187" t="inlineStr">
+        <is>
+          <t>Dias decorridos (fechados)</t>
+        </is>
+      </c>
+      <c r="B9" s="170" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="187" t="inlineStr">
+        <is>
+          <t>Dias restantes</t>
+        </is>
+      </c>
+      <c r="B10" s="170" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="187" t="inlineStr">
+        <is>
+          <t>Ticket médio medido</t>
+        </is>
+      </c>
+      <c r="B11" s="211">
+        <f>B7/B8</f>
+        <v/>
+      </c>
+      <c r="D11" s="178" t="inlineStr">
+        <is>
+          <t>meta implícita R$82 (230k/2796)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="187" t="inlineStr">
+        <is>
+          <t>% da meta de GMV atingido</t>
+        </is>
+      </c>
+      <c r="B12" s="212">
+        <f>B7/B5</f>
+        <v/>
+      </c>
+      <c r="D12" s="178" t="inlineStr">
+        <is>
+          <t>vs 42% do mês decorrido → atrás</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="187" t="inlineStr">
+        <is>
+          <t>Índice de pace (GMV)</t>
+        </is>
+      </c>
+      <c r="B13" s="213">
+        <f>(B7/B9)/(B5/31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="63">
+      <c r="A14" s="190" t="inlineStr">
+        <is>
+          <t>② DISTRIBUIÇÃO HERO × ESTEIRA (medido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="156" t="inlineStr">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="B15" s="156" t="inlineStr">
+        <is>
+          <t>Peças</t>
+        </is>
+      </c>
+      <c r="C15" s="156" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="D15" s="156" t="inlineStr">
+        <is>
+          <t>% peças</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="214" t="inlineStr">
+        <is>
+          <t>HERO (REF516/525/527)</t>
+        </is>
+      </c>
+      <c r="B16" s="215" t="n">
+        <v>497</v>
+      </c>
+      <c r="C16" s="216" t="n">
+        <v>36093</v>
+      </c>
+      <c r="D16" s="217">
+        <f>B16/B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="218" t="inlineStr">
+        <is>
+          <t>ESTEIRA</t>
+        </is>
+      </c>
+      <c r="B17" s="215" t="n">
+        <v>326</v>
+      </c>
+      <c r="C17" s="216" t="n">
+        <v>25007</v>
+      </c>
+      <c r="D17" s="217">
+        <f>B17/B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="138" t="inlineStr">
+        <is>
+          <t>TOP SKUs (peças em live própria):</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF516 · HERO</t>
+        </is>
+      </c>
+      <c r="B19" s="219" t="n">
+        <v>277</v>
+      </c>
+      <c r="C19" s="220" t="n">
+        <v>19991</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF525 · HERO</t>
+        </is>
+      </c>
+      <c r="B20" s="219" t="n">
+        <v>135</v>
+      </c>
+      <c r="C20" s="220" t="n">
+        <v>9876</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF527 · HERO</t>
+        </is>
+      </c>
+      <c r="B21" s="219" t="n">
+        <v>84</v>
+      </c>
+      <c r="C21" s="220" t="n">
+        <v>6225</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF551 · esteira ·PREMIUM</t>
+        </is>
+      </c>
+      <c r="B22" s="219" t="n">
+        <v>79</v>
+      </c>
+      <c r="C22" s="220" t="n">
+        <v>6225</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF562 · esteira ·Chocolate</t>
+        </is>
+      </c>
+      <c r="B23" s="219" t="n">
+        <v>52</v>
+      </c>
+      <c r="C23" s="220" t="n">
+        <v>4020</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF547 · esteira</t>
+        </is>
+      </c>
+      <c r="B24" s="219" t="n">
+        <v>36</v>
+      </c>
+      <c r="C24" s="220" t="n">
+        <v>2972</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF528 · esteira ·PREMIUM</t>
+        </is>
+      </c>
+      <c r="B25" s="219" t="n">
+        <v>32</v>
+      </c>
+      <c r="C25" s="220" t="n">
+        <v>2646</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="172" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  REF587 · esteira</t>
+        </is>
+      </c>
+      <c r="B26" s="219" t="n">
+        <v>27</v>
+      </c>
+      <c r="C26" s="220" t="n">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="63">
+      <c r="A27" s="192" t="inlineStr">
+        <is>
+          <t>③ FECHAR O GAP ATÉ R$230k — volume vs ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="155" t="inlineStr">
+        <is>
+          <t>Gap de GMV a recuperar</t>
+        </is>
+      </c>
+      <c r="B28" s="221">
+        <f>B5-B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="187" t="inlineStr">
+        <is>
+          <t>GMV/dia atual</t>
+        </is>
+      </c>
+      <c r="B29" s="222">
+        <f>B7/B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="155" t="inlineStr">
+        <is>
+          <t>GMV/dia NECESSÁRIO (restante)</t>
+        </is>
+      </c>
+      <c r="B30" s="223">
+        <f>B28/B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="187" t="inlineStr">
+        <is>
+          <t>Fator (quantas vezes o ritmo atual)</t>
+        </is>
+      </c>
+      <c r="B31" s="224">
+        <f>B30/B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="138" t="inlineStr">
+        <is>
+          <t>Cenários de ticket (quanto sobe o ticket, menos peças/dia):</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="187" t="inlineStr">
+        <is>
+          <t>Peças/dia atual</t>
+        </is>
+      </c>
+      <c r="B34" s="225">
+        <f>B8/B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="187" t="inlineStr">
+        <is>
+          <t>Peças/dia SE segurar ticket atual</t>
+        </is>
+      </c>
+      <c r="B35" s="226">
+        <f>B30/B11</f>
+        <v/>
+      </c>
+      <c r="D35" s="178" t="inlineStr">
+        <is>
+          <t>tudo por volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="187" t="inlineStr">
+        <is>
+          <t>Ticket-alvo com mix premium</t>
+        </is>
+      </c>
+      <c r="B36" s="188" t="n">
+        <v>82</v>
+      </c>
+      <c r="D36" s="178" t="inlineStr">
+        <is>
+          <t>551+528 puxam o ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="187" t="inlineStr">
+        <is>
+          <t>Peças/dia @ ticket-alvo</t>
+        </is>
+      </c>
+      <c r="B37" s="225">
+        <f>B30/B36</f>
+        <v/>
+      </c>
+      <c r="D37" s="178" t="inlineStr">
+        <is>
+          <t>menos peças, mais R$/peça</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="138" t="inlineStr">
+        <is>
+          <t>Peça premium (551+528) carregando o incremento:</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="187" t="inlineStr">
+        <is>
+          <t>Ticket da peça premium (551/528)</t>
+        </is>
+      </c>
+      <c r="B40" s="188" t="n">
+        <v>80</v>
+      </c>
+      <c r="D40" s="178" t="inlineStr">
+        <is>
+          <t>551 R$79 · 528 R$83</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="187" t="inlineStr">
+        <is>
+          <t>Incremento de GMV/dia (acima do atual)</t>
+        </is>
+      </c>
+      <c r="B41" s="227">
+        <f>B30-B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="155" t="inlineStr">
+        <is>
+          <t>→ Peças premium/dia p/ cobrir o incremento</t>
+        </is>
+      </c>
+      <c r="B42" s="171">
+        <f>B41/B40</f>
+        <v/>
+      </c>
+      <c r="D42" s="178" t="inlineStr">
+        <is>
+          <t>hoje premium roda ~8,5/dia</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="42" customHeight="1" s="63">
+      <c r="A43" s="175" t="inlineStr">
+        <is>
+          <t>Leitura: o gap pede ~2x o ritmo. Ticket-alvo via premium (551/528) tira algumas peças/dia da conta, mas premium sozinho não fecha (precisaria ~10x o volume premium de hoje). Fórmula real = MAIS LIVES (volume) + MIX PREMIUM (ticket) juntos. O REF551 já provou que puxa; o 528 é o que falta destravar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A43:D45"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -6826,7 +7400,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7829,475 +8403,6 @@
     </row>
     <row r="21" ht="15" customHeight="1" s="63">
       <c r="A21" s="71" t="inlineStr">
-        <is>
-          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:S14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="10" customWidth="1" style="62" min="1" max="1"/>
-    <col width="22" customWidth="1" style="62" min="2" max="2"/>
-    <col width="5" customWidth="1" style="62" min="3" max="3"/>
-    <col width="12" customWidth="1" style="62" min="4" max="4"/>
-    <col width="8" customWidth="1" style="62" min="5" max="5"/>
-    <col width="10" customWidth="1" style="62" min="6" max="7"/>
-    <col width="11" customWidth="1" style="62" min="8" max="8"/>
-    <col width="12" customWidth="1" style="62" min="9" max="9"/>
-    <col width="9" customWidth="1" style="62" min="10" max="10"/>
-    <col width="11" customWidth="1" style="62" min="11" max="11"/>
-    <col width="13" customWidth="1" style="62" min="12" max="12"/>
-    <col width="12" customWidth="1" style="62" min="13" max="13"/>
-    <col width="13" customWidth="1" style="62" min="14" max="15"/>
-    <col width="11" customWidth="1" style="62" min="16" max="16"/>
-    <col width="12" customWidth="1" style="62" min="17" max="18"/>
-    <col width="14" customWidth="1" style="62" min="19" max="19"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="63">
-      <c r="A1" s="64" t="inlineStr">
-        <is>
-          <t>Vitrine loja — meta por SKU e pace diário</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="63">
-      <c r="A2" s="66" t="inlineStr">
-        <is>
-          <t>Canal (chave):</t>
-        </is>
-      </c>
-      <c r="B2" s="89" t="inlineStr">
-        <is>
-          <t>Vitrine loja</t>
-        </is>
-      </c>
-      <c r="C2" s="66" t="inlineStr">
-        <is>
-          <t>Superfície:</t>
-        </is>
-      </c>
-      <c r="D2" s="89" t="inlineStr">
-        <is>
-          <t>VITRINE DA LOJA</t>
-        </is>
-      </c>
-      <c r="F2" s="66" t="inlineStr">
-        <is>
-          <t>Atribuição:</t>
-        </is>
-      </c>
-      <c r="G2" s="89" t="inlineStr">
-        <is>
-          <t>Loja / vendedor</t>
-        </is>
-      </c>
-      <c r="I2" s="66" t="inlineStr">
-        <is>
-          <t>Confiança da base jul:</t>
-        </is>
-      </c>
-      <c r="K2" s="121" t="inlineStr">
-        <is>
-          <t>TRANSVERSAL — shop_tab R$89.369 (jul, API 202605) SOBREPÕE card/loja; não somável no NET (lente de superfície, não de último-conteúdo).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="63">
-      <c r="A3" s="66" t="inlineStr">
-        <is>
-          <t>Alavanca principal:</t>
-        </is>
-      </c>
-      <c r="B3" s="89" t="inlineStr">
-        <is>
-          <t>A definir — organizar vitrine por curva e coleção</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="63">
-      <c r="A4" s="66" t="inlineStr">
-        <is>
-          <t>Crescimento vs base:</t>
-        </is>
-      </c>
-      <c r="B4" s="107">
-        <f>Premissas!$C$31</f>
-        <v/>
-      </c>
-      <c r="C4" s="66" t="inlineStr">
-        <is>
-          <t>Comissão afiliada:</t>
-        </is>
-      </c>
-      <c r="D4" s="107">
-        <f>Premissas!$D$31</f>
-        <v/>
-      </c>
-      <c r="F4" s="66" t="inlineStr">
-        <is>
-          <t>CPV padrão:</t>
-        </is>
-      </c>
-      <c r="G4" s="108">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="63">
-      <c r="A5" s="66" t="inlineStr">
-        <is>
-          <t>Meta do canal (pç):</t>
-        </is>
-      </c>
-      <c r="B5" s="109">
-        <f>G9</f>
-        <v/>
-      </c>
-      <c r="C5" s="66" t="inlineStr">
-        <is>
-          <t>Meta GMV:</t>
-        </is>
-      </c>
-      <c r="D5" s="110">
-        <f>I9</f>
-        <v/>
-      </c>
-      <c r="F5" s="66" t="inlineStr">
-        <is>
-          <t>Contribuição meta:</t>
-        </is>
-      </c>
-      <c r="G5" s="110">
-        <f>L9</f>
-        <v/>
-      </c>
-      <c r="I5" s="66" t="inlineStr">
-        <is>
-          <t>Índice de pace:</t>
-        </is>
-      </c>
-      <c r="K5" s="111">
-        <f>P9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="63">
-      <c r="A7" s="72" t="inlineStr">
-        <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B7" s="72" t="inlineStr">
-        <is>
-          <t>Produto</t>
-        </is>
-      </c>
-      <c r="C7" s="72" t="inlineStr">
-        <is>
-          <t>Cl</t>
-        </is>
-      </c>
-      <c r="D7" s="72" t="inlineStr">
-        <is>
-          <t>Base jul (pç)</t>
-        </is>
-      </c>
-      <c r="E7" s="72" t="inlineStr">
-        <is>
-          <t>Mix jul</t>
-        </is>
-      </c>
-      <c r="F7" s="72" t="inlineStr">
-        <is>
-          <t>Ajuste (pç)</t>
-        </is>
-      </c>
-      <c r="G7" s="72" t="inlineStr">
-        <is>
-          <t>Meta (pç)</t>
-        </is>
-      </c>
-      <c r="H7" s="72" t="inlineStr">
-        <is>
-          <t>Preço plan.</t>
-        </is>
-      </c>
-      <c r="I7" s="72" t="inlineStr">
-        <is>
-          <t>Meta GMV</t>
-        </is>
-      </c>
-      <c r="J7" s="72" t="inlineStr">
-        <is>
-          <t>CPV</t>
-        </is>
-      </c>
-      <c r="K7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib./pç</t>
-        </is>
-      </c>
-      <c r="L7" s="72" t="inlineStr">
-        <is>
-          <t>Contrib. meta</t>
-        </is>
-      </c>
-      <c r="M7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (pç)</t>
-        </is>
-      </c>
-      <c r="N7" s="72" t="inlineStr">
-        <is>
-          <t>Real MTD (R$)</t>
-        </is>
-      </c>
-      <c r="O7" s="72" t="inlineStr">
-        <is>
-          <t>Esperado MTD</t>
-        </is>
-      </c>
-      <c r="P7" s="72" t="inlineStr">
-        <is>
-          <t>Índice pace</t>
-        </is>
-      </c>
-      <c r="Q7" s="72" t="inlineStr">
-        <is>
-          <t>Projeção fim</t>
-        </is>
-      </c>
-      <c r="R7" s="72" t="inlineStr">
-        <is>
-          <t>Gap vs meta</t>
-        </is>
-      </c>
-      <c r="S7" s="72" t="inlineStr">
-        <is>
-          <t>Pç/dia p/ fechar</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="63">
-      <c r="A8" s="73" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B8" s="74" t="inlineStr">
-        <is>
-          <t>Sem base de julho para este canal</t>
-        </is>
-      </c>
-      <c r="C8" s="74" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="113">
-        <f>IFERROR(D8/$D$9,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="112">
-        <f>ROUND(D8*(1+$B$4),0)+F8</f>
-        <v/>
-      </c>
-      <c r="H8" s="97" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="114">
-        <f>G8*H8</f>
-        <v/>
-      </c>
-      <c r="J8" s="115">
-        <f>Premissas!$C$18</f>
-        <v/>
-      </c>
-      <c r="K8" s="116">
-        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
-        <v/>
-      </c>
-      <c r="L8" s="114">
-        <f>G8*K8</f>
-        <v/>
-      </c>
-      <c r="M8" s="112">
-        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="N8" s="114">
-        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="112">
-        <f>G8*Premissas!$C$10</f>
-        <v/>
-      </c>
-      <c r="P8" s="117">
-        <f>IFERROR(M8/O8,0)</f>
-        <v/>
-      </c>
-      <c r="Q8" s="112">
-        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
-        <v/>
-      </c>
-      <c r="R8" s="112">
-        <f>Q8-G8</f>
-        <v/>
-      </c>
-      <c r="S8" s="118">
-        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="63">
-      <c r="A9" s="81" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B9" s="81" t="n"/>
-      <c r="C9" s="81" t="n"/>
-      <c r="D9" s="82">
-        <f>SUM(D8:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="85">
-        <f>SUM(E8:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="82">
-        <f>SUM(F8:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="82">
-        <f>SUM(G8:G8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="119" t="n"/>
-      <c r="I9" s="83">
-        <f>SUM(I8:I8)</f>
-        <v/>
-      </c>
-      <c r="J9" s="119" t="n"/>
-      <c r="K9" s="119" t="n"/>
-      <c r="L9" s="83">
-        <f>SUM(L8:L8)</f>
-        <v/>
-      </c>
-      <c r="M9" s="82">
-        <f>SUM(M8:M8)</f>
-        <v/>
-      </c>
-      <c r="N9" s="83">
-        <f>SUM(N8:N8)</f>
-        <v/>
-      </c>
-      <c r="O9" s="82">
-        <f>SUM(O8:O8)</f>
-        <v/>
-      </c>
-      <c r="P9" s="84">
-        <f>IFERROR(M9/O9,0)</f>
-        <v/>
-      </c>
-      <c r="Q9" s="82">
-        <f>SUM(Q8:Q8)</f>
-        <v/>
-      </c>
-      <c r="R9" s="82">
-        <f>SUM(R8:R8)</f>
-        <v/>
-      </c>
-      <c r="S9" s="120">
-        <f>SUM(S8:S8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="63">
-      <c r="A10" s="73" t="inlineStr">
-        <is>
-          <t>Σ Hero</t>
-        </is>
-      </c>
-      <c r="B10" s="74" t="n"/>
-      <c r="C10" s="74" t="n"/>
-      <c r="D10" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="E10" s="74" t="n"/>
-      <c r="F10" s="74" t="n"/>
-      <c r="G10" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-      <c r="H10" s="74" t="n"/>
-      <c r="I10" s="74" t="n"/>
-      <c r="J10" s="74" t="n"/>
-      <c r="K10" s="74" t="n"/>
-      <c r="L10" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="63">
-      <c r="A11" s="73" t="inlineStr">
-        <is>
-          <t>Σ Esteira</t>
-        </is>
-      </c>
-      <c r="B11" s="74" t="n"/>
-      <c r="C11" s="74" t="n"/>
-      <c r="D11" s="112">
-        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="E11" s="74" t="n"/>
-      <c r="F11" s="74" t="n"/>
-      <c r="G11" s="112">
-        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-      <c r="H11" s="74" t="n"/>
-      <c r="I11" s="74" t="n"/>
-      <c r="J11" s="74" t="n"/>
-      <c r="K11" s="74" t="n"/>
-      <c r="L11" s="114">
-        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="63">
-      <c r="A13" s="71" t="inlineStr">
-        <is>
-          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="63">
-      <c r="A14" s="71" t="inlineStr">
         <is>
           <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
         </is>
@@ -8340,7 +8445,7 @@
     <row r="1" ht="16.15" customHeight="1" s="63">
       <c r="A1" s="64" t="inlineStr">
         <is>
-          <t>Busca e Mall — meta por SKU e pace diário</t>
+          <t>Vitrine loja — meta por SKU e pace diário</t>
         </is>
       </c>
     </row>
@@ -8352,7 +8457,7 @@
       </c>
       <c r="B2" s="89" t="inlineStr">
         <is>
-          <t>Busca e Mall</t>
+          <t>Vitrine loja</t>
         </is>
       </c>
       <c r="C2" s="66" t="inlineStr">
@@ -8362,7 +8467,7 @@
       </c>
       <c r="D2" s="89" t="inlineStr">
         <is>
-          <t>BUSCA / MALL / OUTROS</t>
+          <t>VITRINE DA LOJA</t>
         </is>
       </c>
       <c r="F2" s="66" t="inlineStr">
@@ -8372,7 +8477,7 @@
       </c>
       <c r="G2" s="89" t="inlineStr">
         <is>
-          <t>Misto</t>
+          <t>Loja / vendedor</t>
         </is>
       </c>
       <c r="I2" s="66" t="inlineStr">
@@ -8382,7 +8487,7 @@
       </c>
       <c r="K2" s="121" t="inlineStr">
         <is>
-          <t>R$0 — nesta atribuição (API 202605) total = seller(live+vídeo+card)+afiliada, resíduo zero. Sem balde separado.</t>
+          <t>TRANSVERSAL — shop_tab R$89.369 (jul, API 202605) SOBREPÕE card/loja; não somável no NET (lente de superfície, não de último-conteúdo).</t>
         </is>
       </c>
     </row>
@@ -8394,7 +8499,7 @@
       </c>
       <c r="B3" s="89" t="inlineStr">
         <is>
-          <t>A definir — SEO de título/atributo de produto</t>
+          <t>A definir — organizar vitrine por curva e coleção</t>
         </is>
       </c>
     </row>
@@ -8405,7 +8510,7 @@
         </is>
       </c>
       <c r="B4" s="107">
-        <f>Premissas!$C$32</f>
+        <f>Premissas!$C$31</f>
         <v/>
       </c>
       <c r="C4" s="66" t="inlineStr">
@@ -8414,7 +8519,7 @@
         </is>
       </c>
       <c r="D4" s="107">
-        <f>Premissas!$D$32</f>
+        <f>Premissas!$D$31</f>
         <v/>
       </c>
       <c r="F4" s="66" t="inlineStr">
@@ -8780,6 +8885,475 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="10" customWidth="1" style="62" min="1" max="1"/>
+    <col width="22" customWidth="1" style="62" min="2" max="2"/>
+    <col width="5" customWidth="1" style="62" min="3" max="3"/>
+    <col width="12" customWidth="1" style="62" min="4" max="4"/>
+    <col width="8" customWidth="1" style="62" min="5" max="5"/>
+    <col width="10" customWidth="1" style="62" min="6" max="7"/>
+    <col width="11" customWidth="1" style="62" min="8" max="8"/>
+    <col width="12" customWidth="1" style="62" min="9" max="9"/>
+    <col width="9" customWidth="1" style="62" min="10" max="10"/>
+    <col width="11" customWidth="1" style="62" min="11" max="11"/>
+    <col width="13" customWidth="1" style="62" min="12" max="12"/>
+    <col width="12" customWidth="1" style="62" min="13" max="13"/>
+    <col width="13" customWidth="1" style="62" min="14" max="15"/>
+    <col width="11" customWidth="1" style="62" min="16" max="16"/>
+    <col width="12" customWidth="1" style="62" min="17" max="18"/>
+    <col width="14" customWidth="1" style="62" min="19" max="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16.15" customHeight="1" s="63">
+      <c r="A1" s="64" t="inlineStr">
+        <is>
+          <t>Busca e Mall — meta por SKU e pace diário</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="63">
+      <c r="A2" s="66" t="inlineStr">
+        <is>
+          <t>Canal (chave):</t>
+        </is>
+      </c>
+      <c r="B2" s="89" t="inlineStr">
+        <is>
+          <t>Busca e Mall</t>
+        </is>
+      </c>
+      <c r="C2" s="66" t="inlineStr">
+        <is>
+          <t>Superfície:</t>
+        </is>
+      </c>
+      <c r="D2" s="89" t="inlineStr">
+        <is>
+          <t>BUSCA / MALL / OUTROS</t>
+        </is>
+      </c>
+      <c r="F2" s="66" t="inlineStr">
+        <is>
+          <t>Atribuição:</t>
+        </is>
+      </c>
+      <c r="G2" s="89" t="inlineStr">
+        <is>
+          <t>Misto</t>
+        </is>
+      </c>
+      <c r="I2" s="66" t="inlineStr">
+        <is>
+          <t>Confiança da base jul:</t>
+        </is>
+      </c>
+      <c r="K2" s="121" t="inlineStr">
+        <is>
+          <t>R$0 — nesta atribuição (API 202605) total = seller(live+vídeo+card)+afiliada, resíduo zero. Sem balde separado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="63">
+      <c r="A3" s="66" t="inlineStr">
+        <is>
+          <t>Alavanca principal:</t>
+        </is>
+      </c>
+      <c r="B3" s="89" t="inlineStr">
+        <is>
+          <t>A definir — SEO de título/atributo de produto</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="63">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>Crescimento vs base:</t>
+        </is>
+      </c>
+      <c r="B4" s="107">
+        <f>Premissas!$C$32</f>
+        <v/>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Comissão afiliada:</t>
+        </is>
+      </c>
+      <c r="D4" s="107">
+        <f>Premissas!$D$32</f>
+        <v/>
+      </c>
+      <c r="F4" s="66" t="inlineStr">
+        <is>
+          <t>CPV padrão:</t>
+        </is>
+      </c>
+      <c r="G4" s="108">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="63">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>Meta do canal (pç):</t>
+        </is>
+      </c>
+      <c r="B5" s="109">
+        <f>G9</f>
+        <v/>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>Meta GMV:</t>
+        </is>
+      </c>
+      <c r="D5" s="110">
+        <f>I9</f>
+        <v/>
+      </c>
+      <c r="F5" s="66" t="inlineStr">
+        <is>
+          <t>Contribuição meta:</t>
+        </is>
+      </c>
+      <c r="G5" s="110">
+        <f>L9</f>
+        <v/>
+      </c>
+      <c r="I5" s="66" t="inlineStr">
+        <is>
+          <t>Índice de pace:</t>
+        </is>
+      </c>
+      <c r="K5" s="111">
+        <f>P9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="63">
+      <c r="A7" s="72" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B7" s="72" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>Cl</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>Base jul (pç)</t>
+        </is>
+      </c>
+      <c r="E7" s="72" t="inlineStr">
+        <is>
+          <t>Mix jul</t>
+        </is>
+      </c>
+      <c r="F7" s="72" t="inlineStr">
+        <is>
+          <t>Ajuste (pç)</t>
+        </is>
+      </c>
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>Meta (pç)</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="inlineStr">
+        <is>
+          <t>Preço plan.</t>
+        </is>
+      </c>
+      <c r="I7" s="72" t="inlineStr">
+        <is>
+          <t>Meta GMV</t>
+        </is>
+      </c>
+      <c r="J7" s="72" t="inlineStr">
+        <is>
+          <t>CPV</t>
+        </is>
+      </c>
+      <c r="K7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib./pç</t>
+        </is>
+      </c>
+      <c r="L7" s="72" t="inlineStr">
+        <is>
+          <t>Contrib. meta</t>
+        </is>
+      </c>
+      <c r="M7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (pç)</t>
+        </is>
+      </c>
+      <c r="N7" s="72" t="inlineStr">
+        <is>
+          <t>Real MTD (R$)</t>
+        </is>
+      </c>
+      <c r="O7" s="72" t="inlineStr">
+        <is>
+          <t>Esperado MTD</t>
+        </is>
+      </c>
+      <c r="P7" s="72" t="inlineStr">
+        <is>
+          <t>Índice pace</t>
+        </is>
+      </c>
+      <c r="Q7" s="72" t="inlineStr">
+        <is>
+          <t>Projeção fim</t>
+        </is>
+      </c>
+      <c r="R7" s="72" t="inlineStr">
+        <is>
+          <t>Gap vs meta</t>
+        </is>
+      </c>
+      <c r="S7" s="72" t="inlineStr">
+        <is>
+          <t>Pç/dia p/ fechar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="63">
+      <c r="A8" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B8" s="74" t="inlineStr">
+        <is>
+          <t>Sem base de julho para este canal</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" s="112" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="113">
+        <f>IFERROR(D8/$D$9,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="112">
+        <f>ROUND(D8*(1+$B$4),0)+F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="97" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="114">
+        <f>G8*H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="115">
+        <f>Premissas!$C$18</f>
+        <v/>
+      </c>
+      <c r="K8" s="116">
+        <f>H8*(1-Premissas!$C$19)*(1-$D$4)*(1-Premissas!$C$20)-J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="114">
+        <f>G8*K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="112">
+        <f>SUMIFS('Log diário'!$D:$D,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="N8" s="114">
+        <f>SUMIFS('Log diário'!$E:$E,'Log diário'!$B:$B,$B$2,'Log diário'!$C:$C,$A8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="112">
+        <f>G8*Premissas!$C$10</f>
+        <v/>
+      </c>
+      <c r="P8" s="117">
+        <f>IFERROR(M8/O8,0)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="112">
+        <f>IFERROR(M8/Premissas!$C$8*Premissas!$C$7,0)</f>
+        <v/>
+      </c>
+      <c r="R8" s="112">
+        <f>Q8-G8</f>
+        <v/>
+      </c>
+      <c r="S8" s="118">
+        <f>IFERROR(MAX(0,G8-M8)/Premissas!$C$9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="63">
+      <c r="A9" s="81" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="n"/>
+      <c r="C9" s="81" t="n"/>
+      <c r="D9" s="82">
+        <f>SUM(D8:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="85">
+        <f>SUM(E8:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="82">
+        <f>SUM(F8:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="82">
+        <f>SUM(G8:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="119" t="n"/>
+      <c r="I9" s="83">
+        <f>SUM(I8:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="119" t="n"/>
+      <c r="K9" s="119" t="n"/>
+      <c r="L9" s="83">
+        <f>SUM(L8:L8)</f>
+        <v/>
+      </c>
+      <c r="M9" s="82">
+        <f>SUM(M8:M8)</f>
+        <v/>
+      </c>
+      <c r="N9" s="83">
+        <f>SUM(N8:N8)</f>
+        <v/>
+      </c>
+      <c r="O9" s="82">
+        <f>SUM(O8:O8)</f>
+        <v/>
+      </c>
+      <c r="P9" s="84">
+        <f>IFERROR(M9/O9,0)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="82">
+        <f>SUM(Q8:Q8)</f>
+        <v/>
+      </c>
+      <c r="R9" s="82">
+        <f>SUM(R8:R8)</f>
+        <v/>
+      </c>
+      <c r="S9" s="120">
+        <f>SUM(S8:S8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="63">
+      <c r="A10" s="73" t="inlineStr">
+        <is>
+          <t>Σ Hero</t>
+        </is>
+      </c>
+      <c r="B10" s="74" t="n"/>
+      <c r="C10" s="74" t="n"/>
+      <c r="D10" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="E10" s="74" t="n"/>
+      <c r="F10" s="74" t="n"/>
+      <c r="G10" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+      <c r="H10" s="74" t="n"/>
+      <c r="I10" s="74" t="n"/>
+      <c r="J10" s="74" t="n"/>
+      <c r="K10" s="74" t="n"/>
+      <c r="L10" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"H")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="63">
+      <c r="A11" s="73" t="inlineStr">
+        <is>
+          <t>Σ Esteira</t>
+        </is>
+      </c>
+      <c r="B11" s="74" t="n"/>
+      <c r="C11" s="74" t="n"/>
+      <c r="D11" s="112">
+        <f>SUMIFS(D8:D8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="E11" s="74" t="n"/>
+      <c r="F11" s="74" t="n"/>
+      <c r="G11" s="112">
+        <f>SUMIFS(G8:G8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+      <c r="H11" s="74" t="n"/>
+      <c r="I11" s="74" t="n"/>
+      <c r="J11" s="74" t="n"/>
+      <c r="K11" s="74" t="n"/>
+      <c r="L11" s="114">
+        <f>SUMIFS(L8:L8,$C$8:$C$8,"E")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="63">
+      <c r="A13" s="71" t="inlineStr">
+        <is>
+          <t>Ajuste (pç) é a coluna azul onde você força um SKU específico — lançamento do 34, pré-escala do Chocolate, abertura do Baggy. Sem ela, o modelo só escala julho de forma plana, o que contradiz a sua própria estratégia de portfólio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1" s="63">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>Índice de pace: 1,00x = exatamente no ritmo da meta. Abaixo de 1,00x = atrasado. Projeção fim = ritmo atual extrapolado até o dia 31.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>